<commit_message>
📊 업데이트 - 2026-06-01 10:13
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R30"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,37 +511,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,55 +571,55 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="P2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="R2" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -629,17 +629,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -667,57 +667,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -727,55 +727,63 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O4" t="n">
-        <v>50</v>
-      </c>
-      <c r="P4" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>50</v>
-      </c>
-      <c r="R4" t="n">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -785,17 +793,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>60.8</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>35.5</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -805,40 +813,40 @@
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O5" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="Q5" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="R5" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -853,7 +861,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -863,17 +871,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -901,37 +909,37 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -941,17 +949,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -987,57 +995,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1047,75 +1055,83 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>2</v>
-      </c>
-      <c r="O8" t="n">
-        <v>50</v>
-      </c>
-      <c r="P8" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>50</v>
-      </c>
-      <c r="R8" t="n">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2-5</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1125,68 +1141,60 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O9" t="n">
+        <v>50</v>
+      </c>
+      <c r="P9" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>50</v>
+      </c>
+      <c r="R9" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>6-5</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1196,12 +1204,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>63.2</t>
+          <t>67.8</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>37.9</t>
+          <t>42.9</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1211,55 +1219,63 @@
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
-        <v>2</v>
-      </c>
-      <c r="O10" t="n">
-        <v>50</v>
-      </c>
-      <c r="P10" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>50</v>
-      </c>
-      <c r="R10" t="n">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>7-4</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1269,17 +1285,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>51.6</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1307,57 +1323,57 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1367,43 +1383,35 @@
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O12" t="n">
+        <v>50</v>
+      </c>
+      <c r="P12" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>50</v>
+      </c>
+      <c r="R12" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1413,37 +1421,37 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>24.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>76.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-8</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>80.2</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>58.7</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1453,43 +1461,35 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
         <v>0</v>
       </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P13" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1499,17 +1499,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1519,17 +1519,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>78.5</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>56.4</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1539,35 +1539,43 @@
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
-        <v>1</v>
-      </c>
-      <c r="O14" t="n">
-        <v>100</v>
-      </c>
-      <c r="P14" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" t="n">
-        <v>100</v>
-      </c>
-      <c r="R14" t="n">
-        <v>100</v>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1577,17 +1585,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7-6</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1597,17 +1605,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>97.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>77.7</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>55.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1617,35 +1625,35 @@
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O15" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="Q15" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="R15" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>8:20</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1655,17 +1663,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1675,17 +1683,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>68.9</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>44.2</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1721,57 +1729,57 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1781,55 +1789,63 @@
       </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
-        <v>2</v>
-      </c>
-      <c r="O17" t="n">
-        <v>50</v>
-      </c>
-      <c r="P17" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>50</v>
-      </c>
-      <c r="R17" t="n">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1839,17 +1855,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1877,37 +1893,37 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:38</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1917,17 +1933,17 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1940,72 +1956,72 @@
         <v>1</v>
       </c>
       <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
         <v>100</v>
       </c>
-      <c r="P19" t="n">
+      <c r="Q19" t="n">
         <v>0</v>
       </c>
-      <c r="Q19" t="n">
-        <v>100</v>
-      </c>
       <c r="R19" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>72.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>28.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2015,83 +2031,75 @@
       </c>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="n">
+        <v>1</v>
+      </c>
+      <c r="O20" t="n">
         <v>0</v>
       </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P20" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2101,63 +2109,55 @@
       </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O21" t="n">
+        <v>50</v>
+      </c>
+      <c r="P21" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>50</v>
+      </c>
+      <c r="R21" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2167,17 +2167,17 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2187,63 +2187,55 @@
       </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>100</v>
+      </c>
+      <c r="P22" t="n">
         <v>0</v>
       </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="Q22" t="n">
+        <v>100</v>
+      </c>
+      <c r="R22" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>2-6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2253,17 +2245,17 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2273,581 +2265,27 @@
       </c>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="n">
-        <v>1</v>
-      </c>
-      <c r="O23" t="n">
-        <v>100</v>
-      </c>
-      <c r="P23" t="n">
         <v>0</v>
       </c>
-      <c r="Q23" t="n">
-        <v>100</v>
-      </c>
-      <c r="R23" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Hanwha Eagles</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>SSG Landers</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>KBO</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>51.0</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>49.0</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>23.3</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>7.9</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="n">
-        <v>1</v>
-      </c>
-      <c r="O24" t="n">
-        <v>100</v>
-      </c>
-      <c r="P24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>100</v>
-      </c>
-      <c r="R24" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Kiwoom Heroes</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>KT Wiz Suwon</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>KBO</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>40.0</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>60.0</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>4-5</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>53.1</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>28.2</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>LG Twins</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>KIA Tigers</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>KBO</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>58.0</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>42.0</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>5-3</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>43.5</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>20.4</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="n">
-        <v>2</v>
-      </c>
-      <c r="O26" t="n">
-        <v>50</v>
-      </c>
-      <c r="P26" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>50</v>
-      </c>
-      <c r="R26" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>NC Dinos</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Lotte Giants</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>KBO</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>54.4</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>29.4</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="n">
-        <v>2</v>
-      </c>
-      <c r="O27" t="n">
-        <v>50</v>
-      </c>
-      <c r="P27" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>50</v>
-      </c>
-      <c r="R27" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>18:05</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Wei Chuan Dragons</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Uni Lions</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>48.0</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>52.0</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>4-5</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>35.2</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>14.6</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="n">
-        <v>1</v>
-      </c>
-      <c r="O28" t="n">
-        <v>100</v>
-      </c>
-      <c r="P28" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>100</v>
-      </c>
-      <c r="R28" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>18:05</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Rakuten Monkeys</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>TSG Hawks</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>42.0</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>58.0</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>3-5</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>35.2</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>14.6</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>18:05</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Fubon Guardians</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Chinatrust Brothers</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>57.0</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>43.0</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>5-3</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>36.6</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>15.5</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="n">
-        <v>2</v>
-      </c>
-      <c r="O30" t="n">
-        <v>50</v>
-      </c>
-      <c r="P30" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>50</v>
-      </c>
-      <c r="R30" t="n">
-        <v>50</v>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-02 15:31
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1421,17 +1421,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>6-5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1441,17 +1441,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>72.1</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>47.9</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1464,32 +1464,32 @@
         <v>1</v>
       </c>
       <c r="O13" t="n">
+        <v>100</v>
+      </c>
+      <c r="P13" t="n">
         <v>0</v>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>100</v>
       </c>
-      <c r="Q13" t="n">
-        <v>0</v>
-      </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1499,22 +1499,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1524,12 +1524,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>33.8</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1539,43 +1539,35 @@
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O14" t="n">
+        <v>50</v>
+      </c>
+      <c r="P14" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>50</v>
+      </c>
+      <c r="R14" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1585,17 +1577,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1605,17 +1597,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1643,17 +1635,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8:20</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1663,37 +1655,37 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1703,43 +1695,35 @@
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" t="n">
+        <v>100</v>
+      </c>
+      <c r="P16" t="n">
         <v>0</v>
       </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="Q16" t="n">
+        <v>100</v>
+      </c>
+      <c r="R16" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1749,37 +1733,37 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1789,43 +1773,35 @@
       </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" t="n">
+        <v>100</v>
+      </c>
+      <c r="P17" t="n">
         <v>0</v>
       </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="Q17" t="n">
+        <v>100</v>
+      </c>
+      <c r="R17" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1835,17 +1811,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1855,17 +1831,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>13.3</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1893,17 +1869,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10:38</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1913,22 +1889,22 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1938,12 +1914,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1953,35 +1929,43 @@
       </c>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="n">
-        <v>1</v>
-      </c>
-      <c r="O19" t="n">
         <v>0</v>
       </c>
-      <c r="P19" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" t="n">
-        <v>0</v>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1991,37 +1975,37 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2034,32 +2018,32 @@
         <v>1</v>
       </c>
       <c r="O20" t="n">
+        <v>100</v>
+      </c>
+      <c r="P20" t="n">
         <v>0</v>
       </c>
-      <c r="P20" t="n">
+      <c r="Q20" t="n">
         <v>100</v>
       </c>
-      <c r="Q20" t="n">
-        <v>0</v>
-      </c>
       <c r="R20" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2069,12 +2053,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2094,12 +2078,12 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2127,37 +2111,37 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:45</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2167,17 +2151,17 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2187,55 +2171,63 @@
       </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
-        <v>1</v>
-      </c>
-      <c r="O22" t="n">
-        <v>100</v>
-      </c>
-      <c r="P22" t="n">
         <v>0</v>
       </c>
-      <c r="Q22" t="n">
-        <v>100</v>
-      </c>
-      <c r="R22" t="n">
-        <v>100</v>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2-6</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2245,17 +2237,17 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2283,6 +2275,420 @@
         </is>
       </c>
       <c r="R23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>64.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>2</v>
+      </c>
+      <c r="O24" t="n">
+        <v>50</v>
+      </c>
+      <c r="P24" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>50</v>
+      </c>
+      <c r="R24" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>82.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>18.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>16.5</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>51.8</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" t="n">
+        <v>100</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>100</v>
+      </c>
+      <c r="R27" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Chinatrust Brothers</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2-6</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>36.6</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-04 12:36
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:R18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,12 +516,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -617,17 +617,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -637,17 +637,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -695,12 +695,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -720,12 +720,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -781,17 +781,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>1-5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -801,17 +801,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>14.3</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -852,12 +852,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -887,17 +887,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -930,12 +930,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -945,37 +945,37 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,35 +985,43 @@
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>2</v>
-      </c>
-      <c r="O7" t="n">
-        <v>50</v>
-      </c>
-      <c r="P7" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R7" t="n">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1023,37 +1031,37 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>46.3</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>22.6</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1063,35 +1071,43 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" t="n">
-        <v>100</v>
-      </c>
-      <c r="P8" t="n">
         <v>0</v>
       </c>
-      <c r="Q8" t="n">
-        <v>100</v>
-      </c>
-      <c r="R8" t="n">
-        <v>100</v>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1101,17 +1117,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>7-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1121,17 +1137,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>51.6</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1141,25 +1157,25 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="P9" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1179,12 +1195,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1204,12 +1220,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>67.8</t>
+          <t>68.9</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>42.9</t>
+          <t>44.2</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1245,17 +1261,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1265,17 +1281,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>7-4</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1285,17 +1301,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>51.6</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1323,17 +1339,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1343,37 +1359,37 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>31.8</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1383,75 +1399,75 @@
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O12" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="P12" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="Q12" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="R12" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>2:05</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2-6</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1461,63 +1477,55 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O13" t="n">
+        <v>50</v>
+      </c>
+      <c r="P13" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>50</v>
+      </c>
+      <c r="R13" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1527,17 +1535,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>35.2</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>14.6</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1573,37 +1581,37 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1613,17 +1621,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1645,6 +1653,248 @@
         <v>50</v>
       </c>
       <c r="R15" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>39.3</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>39.3</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>2</v>
+      </c>
+      <c r="O17" t="n">
+        <v>50</v>
+      </c>
+      <c r="P17" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>50</v>
+      </c>
+      <c r="R17" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>16.5</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>2</v>
+      </c>
+      <c r="O18" t="n">
+        <v>50</v>
+      </c>
+      <c r="P18" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>50</v>
+      </c>
+      <c r="R18" t="n">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-05 12:59
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R18"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,12 +516,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,22 +531,22 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -571,27 +571,19 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O2" t="n">
+        <v>50</v>
+      </c>
+      <c r="P2" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>50</v>
+      </c>
+      <c r="R2" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="3">
@@ -602,12 +594,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -617,17 +609,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -637,17 +629,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>14.3</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -685,7 +677,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,37 +687,37 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>6-5</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,27 +727,19 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O4" t="n">
+        <v>50</v>
+      </c>
+      <c r="P4" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>50</v>
+      </c>
+      <c r="R4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -771,7 +755,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -781,27 +765,27 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -821,27 +805,19 @@
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O5" t="n">
+        <v>50</v>
+      </c>
+      <c r="P5" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>50</v>
+      </c>
+      <c r="R5" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="6">
@@ -852,12 +828,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -867,37 +843,37 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -907,19 +883,27 @@
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" t="n">
-        <v>100</v>
-      </c>
-      <c r="P6" t="n">
         <v>0</v>
       </c>
-      <c r="Q6" t="n">
-        <v>100</v>
-      </c>
-      <c r="R6" t="n">
-        <v>100</v>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -930,12 +914,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -945,37 +929,37 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,27 +969,19 @@
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O7" t="n">
+        <v>50</v>
+      </c>
+      <c r="P7" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R7" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="8">
@@ -1016,12 +992,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1031,12 +1007,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1056,12 +1032,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>46.3</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>22.6</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1102,12 +1078,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1117,17 +1093,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1137,17 +1113,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1157,19 +1133,19 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="P9" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="R9" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10">
@@ -1180,12 +1156,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1195,37 +1171,37 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>68.9</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>44.2</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1235,27 +1211,19 @@
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
         <v>0</v>
       </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P10" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1266,12 +1234,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1281,37 +1249,37 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>64.0</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>36.0</t>
-        </is>
-      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>7-4</t>
+          <t>2-6</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>51.6</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1321,19 +1289,27 @@
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>2</v>
-      </c>
-      <c r="O11" t="n">
-        <v>50</v>
-      </c>
-      <c r="P11" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>50</v>
-      </c>
-      <c r="R11" t="n">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1344,12 +1320,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1359,12 +1335,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1384,12 +1360,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1417,7 +1393,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2:05</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1427,7 +1403,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1437,17 +1413,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1457,17 +1433,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,35 +1453,35 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O13" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="Q13" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2:35</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1525,7 +1501,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>4-8</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1535,17 +1511,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1581,17 +1557,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1601,17 +1577,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1621,17 +1597,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>36.7</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1659,17 +1635,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>8:07</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1679,37 +1655,37 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>76.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>24.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>7-2</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1745,17 +1721,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1765,12 +1741,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1790,12 +1766,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1823,37 +1799,37 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>9:15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1863,17 +1839,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>16.5</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1896,6 +1872,498 @@
       </c>
       <c r="R18" t="n">
         <v>50</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>9:15</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>61.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>39.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>2</v>
+      </c>
+      <c r="O19" t="n">
+        <v>50</v>
+      </c>
+      <c r="P19" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>50</v>
+      </c>
+      <c r="R19" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>9:40</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>4-7</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>92.1</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>73.1</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>49.2</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>71.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>29.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>6-3</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>49.1</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>24.8</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>25.8</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="n">
+        <v>2</v>
+      </c>
+      <c r="O23" t="n">
+        <v>50</v>
+      </c>
+      <c r="P23" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>50</v>
+      </c>
+      <c r="R23" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Chinatrust Brothers</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>24.5</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-06 10:52
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,17 +511,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -556,12 +556,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -589,17 +589,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -609,17 +609,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -629,17 +629,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -649,25 +649,25 @@
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O3" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="P3" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="R3" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6-5</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -707,17 +707,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>31.8</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -745,17 +745,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -765,17 +765,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -785,17 +785,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -823,17 +823,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -843,37 +843,37 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -883,27 +883,19 @@
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O6" t="n">
+        <v>50</v>
+      </c>
+      <c r="P6" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>50</v>
+      </c>
+      <c r="R6" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -929,37 +921,37 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -969,35 +961,43 @@
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>2</v>
-      </c>
-      <c r="O7" t="n">
-        <v>50</v>
-      </c>
-      <c r="P7" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R7" t="n">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1007,37 +1007,37 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>31.8</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1047,43 +1047,35 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O8" t="n">
+        <v>50</v>
+      </c>
+      <c r="P8" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>50</v>
+      </c>
+      <c r="R8" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1093,17 +1085,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1113,17 +1105,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1133,35 +1125,35 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="Q9" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="R9" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1171,12 +1163,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1196,12 +1188,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1211,25 +1203,25 @@
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O10" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="P10" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="R10" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1249,12 +1241,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1315,17 +1307,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1335,37 +1327,37 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>33.8</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1375,35 +1367,43 @@
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
-        <v>2</v>
-      </c>
-      <c r="O12" t="n">
-        <v>50</v>
-      </c>
-      <c r="P12" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>50</v>
-      </c>
-      <c r="R12" t="n">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>3:20</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1413,17 +1413,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1433,17 +1433,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1456,72 +1456,72 @@
         <v>1</v>
       </c>
       <c r="O13" t="n">
+        <v>100</v>
+      </c>
+      <c r="P13" t="n">
         <v>0</v>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>100</v>
       </c>
-      <c r="Q13" t="n">
-        <v>0</v>
-      </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4-8</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>76.8</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1531,63 +1531,55 @@
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O14" t="n">
+        <v>50</v>
+      </c>
+      <c r="P14" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>50</v>
+      </c>
+      <c r="R14" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1597,17 +1589,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>36.7</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1635,42 +1627,42 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8:07</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>76.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>24.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>7-2</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1680,12 +1672,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1713,654 +1705,6 @@
         </is>
       </c>
       <c r="R16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>8:10</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Miami Marlins</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>58.0</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>42.0</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>5-3</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>42.1</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>19.4</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="n">
-        <v>2</v>
-      </c>
-      <c r="O17" t="n">
-        <v>50</v>
-      </c>
-      <c r="P17" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>50</v>
-      </c>
-      <c r="R17" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>9:15</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Texas Rangers</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Cleveland Guardians</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>61.0</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>39.0</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>5-2</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>28.4</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>10.6</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="n">
-        <v>2</v>
-      </c>
-      <c r="O18" t="n">
-        <v>50</v>
-      </c>
-      <c r="P18" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>50</v>
-      </c>
-      <c r="R18" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>9:15</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>St.Louis Cardinals</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Cincinnati Reds</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>61.0</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>39.0</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>42.1</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>19.4</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="n">
-        <v>2</v>
-      </c>
-      <c r="O19" t="n">
-        <v>50</v>
-      </c>
-      <c r="P19" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>50</v>
-      </c>
-      <c r="R19" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>9:40</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Colorado Rockies</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Milwaukee Brewers</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>40.0</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>60.0</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>4-7</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>92.1</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>73.1</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>49.2</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>San Diego Padres</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>New York Mets</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>3-4</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>27.1</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>9.9</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>19:35</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Uni Lions</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Fubon Guardians</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>71.0</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>29.0</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>6-3</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>49.1</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>24.8</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="n">
-        <v>1</v>
-      </c>
-      <c r="O22" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>0</v>
-      </c>
-      <c r="R22" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>19:35</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>TSG Hawks</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Wei Chuan Dragons</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>60.0</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>40.0</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>25.8</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>9.2</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="n">
-        <v>2</v>
-      </c>
-      <c r="O23" t="n">
-        <v>50</v>
-      </c>
-      <c r="P23" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>50</v>
-      </c>
-      <c r="R23" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>19:35</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Chinatrust Brothers</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Rakuten Monkeys</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>45.0</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>3-4</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>24.5</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-07 08:06
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,17 +511,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,37 +531,37 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,35 +571,43 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O2" t="n">
-        <v>50</v>
-      </c>
-      <c r="P2" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>50</v>
-      </c>
-      <c r="R2" t="n">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -609,17 +617,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -629,17 +637,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -649,19 +657,19 @@
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O3" t="n">
-        <v>100</v>
+        <v>33.3</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>66.7</v>
       </c>
       <c r="Q3" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="R3" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="4">
@@ -672,12 +680,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -687,17 +695,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -707,17 +715,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -727,19 +735,19 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O4" t="n">
-        <v>50</v>
+        <v>33.3</v>
       </c>
       <c r="P4" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="Q4" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="R4" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="5">
@@ -750,12 +758,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -765,37 +773,37 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>60.0</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>40.0</t>
-        </is>
-      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -805,19 +813,27 @@
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>2</v>
-      </c>
-      <c r="O5" t="n">
-        <v>50</v>
-      </c>
-      <c r="P5" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>50</v>
-      </c>
-      <c r="R5" t="n">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -828,12 +844,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -843,17 +859,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -863,17 +879,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -883,25 +899,25 @@
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O6" t="n">
-        <v>50</v>
+        <v>33.3</v>
       </c>
       <c r="P6" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="Q6" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="R6" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -921,17 +937,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -941,17 +957,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -987,7 +1003,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1007,37 +1023,37 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1056,10 +1072,10 @@
         <v>50</v>
       </c>
       <c r="Q8" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="R8" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -1070,12 +1086,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1085,37 +1101,37 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1125,19 +1141,27 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>2</v>
-      </c>
-      <c r="O9" t="n">
-        <v>50</v>
-      </c>
-      <c r="P9" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>50</v>
-      </c>
-      <c r="R9" t="n">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1148,12 +1172,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1163,22 +1187,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>2-6</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1188,12 +1212,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1203,19 +1227,27 @@
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
-        <v>2</v>
-      </c>
-      <c r="O10" t="n">
-        <v>50</v>
-      </c>
-      <c r="P10" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>50</v>
-      </c>
-      <c r="R10" t="n">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -1226,12 +1258,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1241,37 +1273,37 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2-6</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1281,27 +1313,19 @@
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="O11" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P11" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="R11" t="n">
+        <v>66.7</v>
       </c>
     </row>
     <row r="12">
@@ -1312,12 +1336,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1327,37 +1351,37 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>25.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>31.8</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1393,17 +1417,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3:20</t>
+          <t>2:37</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1413,17 +1437,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1433,17 +1457,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1453,75 +1477,75 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O13" t="n">
-        <v>100</v>
+        <v>33.3</v>
       </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>66.7</v>
       </c>
       <c r="Q13" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="R13" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>2:40</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>59.6</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>34.2</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1531,50 +1555,58 @@
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
-        <v>2</v>
-      </c>
-      <c r="O14" t="n">
-        <v>50</v>
-      </c>
-      <c r="P14" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>50</v>
-      </c>
-      <c r="R14" t="n">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1594,12 +1626,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1609,60 +1641,60 @@
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O15" t="n">
-        <v>50</v>
+        <v>33.3</v>
       </c>
       <c r="P15" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="Q15" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="R15" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>3:15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1672,12 +1704,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1687,27 +1719,331 @@
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="O16" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P16" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="R16" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>9:30</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>2</v>
+      </c>
+      <c r="O17" t="n">
+        <v>50</v>
+      </c>
+      <c r="P17" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>100</v>
+      </c>
+      <c r="R17" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>25.8</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>3</v>
+      </c>
+      <c r="O18" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P18" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="R18" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>67.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>33.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>6-3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>49.1</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>24.8</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>2</v>
+      </c>
+      <c r="O19" t="n">
+        <v>50</v>
+      </c>
+      <c r="P19" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>50</v>
+      </c>
+      <c r="R19" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Chinatrust Brothers</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>36.6</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>3</v>
+      </c>
+      <c r="O20" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P20" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="R20" t="n">
+        <v>66.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-09 13:47
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,32 +511,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7:35</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -556,12 +556,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,83 +571,75 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O2" t="n">
+        <v>50</v>
+      </c>
+      <c r="P2" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R2" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,55 +649,55 @@
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="P3" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="Q3" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="R3" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,17 +707,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>16.5</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,55 +727,55 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O4" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="P4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="Q4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="R4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>8:07</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -793,17 +785,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -813,40 +805,40 @@
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O5" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="P5" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="Q5" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="R5" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>11:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -861,7 +853,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -871,17 +863,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -904,6 +896,1544 @@
       </c>
       <c r="R6" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Chiba Lotte Marines</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Chunichi Dragons</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" t="n">
+        <v>50</v>
+      </c>
+      <c r="P7" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>100</v>
+      </c>
+      <c r="R7" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Hanwha Eagles</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>KIA Tigers</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>7-5</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>81.7</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>60.9</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="n">
+        <v>5</v>
+      </c>
+      <c r="O8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P8" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>80</v>
+      </c>
+      <c r="R8" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Kiwoom Heroes</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>NC Dinos</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>37.0</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>3-6</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>55.7</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>30.6</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>KT Wiz Suwon</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>46.3</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>22.6</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="n">
+        <v>5</v>
+      </c>
+      <c r="O10" t="n">
+        <v>20</v>
+      </c>
+      <c r="P10" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>80</v>
+      </c>
+      <c r="R10" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SSG Landers</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>43.5</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" t="n">
+        <v>20</v>
+      </c>
+      <c r="P11" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>80</v>
+      </c>
+      <c r="R11" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>5-6</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>92.1</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>51.6</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>7:35</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="n">
+        <v>2</v>
+      </c>
+      <c r="O14" t="n">
+        <v>50</v>
+      </c>
+      <c r="P14" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>100</v>
+      </c>
+      <c r="R14" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>33.8</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>13.8</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="n">
+        <v>4</v>
+      </c>
+      <c r="O15" t="n">
+        <v>25</v>
+      </c>
+      <c r="P15" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>75</v>
+      </c>
+      <c r="R15" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>65.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>36.7</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>5</v>
+      </c>
+      <c r="O17" t="n">
+        <v>20</v>
+      </c>
+      <c r="P17" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>80</v>
+      </c>
+      <c r="R17" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>64.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>50.4</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>25.9</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>8:07</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>18.5</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>4</v>
+      </c>
+      <c r="O20" t="n">
+        <v>25</v>
+      </c>
+      <c r="P20" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>75</v>
+      </c>
+      <c r="R20" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>53.1</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>28.2</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>5</v>
+      </c>
+      <c r="O21" t="n">
+        <v>20</v>
+      </c>
+      <c r="P21" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>80</v>
+      </c>
+      <c r="R21" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>37.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>46.3</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>22.6</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>5</v>
+      </c>
+      <c r="O22" t="n">
+        <v>20</v>
+      </c>
+      <c r="P22" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>80</v>
+      </c>
+      <c r="R22" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>9:40</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>98.6</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>81.7</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>60.9</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="n">
+        <v>1</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>100</v>
+      </c>
+      <c r="R23" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Chinatrust Brothers</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>36.6</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>9.7</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="n">
+        <v>5</v>
+      </c>
+      <c r="O25" t="n">
+        <v>20</v>
+      </c>
+      <c r="P25" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>80</v>
+      </c>
+      <c r="R25" t="n">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-11 08:31
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:R15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,12 +516,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -594,12 +594,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -609,37 +609,37 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -649,19 +649,27 @@
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>5</v>
-      </c>
-      <c r="O3" t="n">
-        <v>20</v>
-      </c>
-      <c r="P3" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>80</v>
-      </c>
-      <c r="R3" t="n">
-        <v>80</v>
+        <v>0</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -672,12 +680,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -687,17 +695,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -707,17 +715,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -727,19 +735,19 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O4" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="P4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="Q4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="R4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5">
@@ -750,12 +758,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -765,37 +773,37 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -805,19 +813,19 @@
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="P5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="Q5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="R5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6">
@@ -828,12 +836,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -843,17 +851,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>73.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -863,7 +871,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -914,12 +922,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -929,12 +937,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -969,19 +977,19 @@
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O7" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="P7" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="Q7" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="R7" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">
@@ -992,12 +1000,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1007,37 +1015,37 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>66.7</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>41.7</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1047,27 +1055,19 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P8" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>80</v>
+      </c>
+      <c r="R8" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="9">
@@ -1078,12 +1078,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1093,37 +1093,37 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>2-5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1133,19 +1133,27 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>5</v>
-      </c>
-      <c r="O9" t="n">
-        <v>20</v>
-      </c>
-      <c r="P9" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>80</v>
-      </c>
-      <c r="R9" t="n">
-        <v>80</v>
+        <v>0</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1196,12 +1204,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1234,12 +1242,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1249,17 +1257,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>25.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1269,17 +1277,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>65.6</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>40.4</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1289,13 +1297,13 @@
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O11" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>66.7</v>
+        <v>100</v>
       </c>
       <c r="Q11" t="n">
         <v>100</v>
@@ -1312,12 +1320,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1327,37 +1335,37 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>81.7</t>
+          <t>73.1</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>60.9</t>
+          <t>49.2</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1367,19 +1375,27 @@
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
-        <v>5</v>
-      </c>
-      <c r="O12" t="n">
-        <v>20</v>
-      </c>
-      <c r="P12" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>80</v>
-      </c>
-      <c r="R12" t="n">
-        <v>80</v>
+        <v>0</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -1390,12 +1406,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1405,17 +1421,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1425,17 +1441,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1445,19 +1461,175 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O13" t="n">
-        <v>33.3</v>
+        <v>25</v>
       </c>
       <c r="P13" t="n">
-        <v>66.7</v>
+        <v>75</v>
       </c>
       <c r="Q13" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="R13" t="n">
-        <v>100</v>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>36.6</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="n">
+        <v>5</v>
+      </c>
+      <c r="O14" t="n">
+        <v>20</v>
+      </c>
+      <c r="P14" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>80</v>
+      </c>
+      <c r="R14" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="n">
+        <v>5</v>
+      </c>
+      <c r="O15" t="n">
+        <v>20</v>
+      </c>
+      <c r="P15" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>80</v>
+      </c>
+      <c r="R15" t="n">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-12 14:35
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,12 +516,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,37 +531,37 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,19 +571,19 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O2" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="P2" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="Q2" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="R2" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
@@ -594,12 +594,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -609,37 +609,37 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -649,27 +649,19 @@
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="O3" t="n">
+        <v>25</v>
+      </c>
+      <c r="P3" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>75</v>
+      </c>
+      <c r="R3" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="4">
@@ -680,12 +672,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,17 +687,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,17 +707,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,19 +727,19 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O4" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q4" t="n">
-        <v>80</v>
+        <v>66.7</v>
       </c>
       <c r="R4" t="n">
-        <v>80</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="5">
@@ -758,12 +750,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -773,37 +765,37 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -813,19 +805,27 @@
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>5</v>
-      </c>
-      <c r="O5" t="n">
-        <v>20</v>
-      </c>
-      <c r="P5" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>80</v>
-      </c>
-      <c r="R5" t="n">
-        <v>80</v>
+        <v>0</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -836,12 +836,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -851,17 +851,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -871,17 +871,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -922,12 +922,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -937,17 +937,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1000,12 +1000,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1015,17 +1015,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1035,17 +1035,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>66.7</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>41.7</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1055,19 +1055,19 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O8" t="n">
-        <v>20</v>
+        <v>33.3</v>
       </c>
       <c r="P8" t="n">
-        <v>80</v>
+        <v>66.7</v>
       </c>
       <c r="Q8" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="R8" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -1078,12 +1078,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1093,37 +1093,37 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2-5</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>33.8</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1133,27 +1133,19 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="O9" t="n">
+        <v>25</v>
+      </c>
+      <c r="P9" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>75</v>
+      </c>
+      <c r="R9" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="10">
@@ -1169,7 +1161,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1179,37 +1171,37 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1219,19 +1211,19 @@
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O10" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="Q10" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="R10" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -1242,12 +1234,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1257,37 +1249,37 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>85.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>1-7</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>46.3</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>31.8</t>
+          <t>22.6</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1297,19 +1289,27 @@
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>1</v>
-      </c>
-      <c r="O11" t="n">
         <v>0</v>
       </c>
-      <c r="P11" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>100</v>
-      </c>
-      <c r="R11" t="n">
-        <v>100</v>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1335,37 +1335,37 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>73.1</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>49.2</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1375,63 +1375,55 @@
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O12" t="n">
+        <v>20</v>
+      </c>
+      <c r="P12" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>80</v>
+      </c>
+      <c r="R12" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1441,17 +1433,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1461,75 +1453,75 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O13" t="n">
-        <v>25</v>
+        <v>33.3</v>
       </c>
       <c r="P13" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="Q13" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="R13" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
           <t>55.0</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>45.0</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>6-4</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>87.0</t>
-        </is>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1539,55 +1531,55 @@
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O14" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q14" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="R14" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1597,17 +1589,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>64.4</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>39.2</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1617,18 +1609,1196 @@
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
+        <v>4</v>
+      </c>
+      <c r="O15" t="n">
+        <v>25</v>
+      </c>
+      <c r="P15" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>75</v>
+      </c>
+      <c r="R15" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>9.7</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>3</v>
+      </c>
+      <c r="O16" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P16" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>100</v>
+      </c>
+      <c r="R16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>100</v>
+      </c>
+      <c r="R17" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>3</v>
+      </c>
+      <c r="O18" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P18" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>100</v>
+      </c>
+      <c r="R18" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>63.2</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>37.9</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>2</v>
+      </c>
+      <c r="O19" t="n">
+        <v>50</v>
+      </c>
+      <c r="P19" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>100</v>
+      </c>
+      <c r="R19" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>8:37</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>7-5</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>79.4</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>57.5</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
         <v>5</v>
       </c>
-      <c r="O15" t="n">
+      <c r="O20" t="n">
         <v>20</v>
       </c>
-      <c r="P15" t="n">
+      <c r="P20" t="n">
         <v>80</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="Q20" t="n">
         <v>80</v>
       </c>
-      <c r="R15" t="n">
+      <c r="R20" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>2</v>
+      </c>
+      <c r="O21" t="n">
+        <v>50</v>
+      </c>
+      <c r="P21" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>100</v>
+      </c>
+      <c r="R21" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>29.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>71.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>43.5</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>43.5</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="n">
+        <v>4</v>
+      </c>
+      <c r="O23" t="n">
+        <v>25</v>
+      </c>
+      <c r="P23" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>75</v>
+      </c>
+      <c r="R23" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>3</v>
+      </c>
+      <c r="O24" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P24" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>100</v>
+      </c>
+      <c r="R24" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>10:38</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>31.1</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="n">
+        <v>3</v>
+      </c>
+      <c r="O25" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P25" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>100</v>
+      </c>
+      <c r="R25" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>66.7</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>41.7</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>100</v>
+      </c>
+      <c r="R26" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>61.0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>39.0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>53.1</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>28.2</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="n">
+        <v>5</v>
+      </c>
+      <c r="O27" t="n">
+        <v>20</v>
+      </c>
+      <c r="P27" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>80</v>
+      </c>
+      <c r="R27" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>36.6</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="n">
+        <v>5</v>
+      </c>
+      <c r="O28" t="n">
+        <v>20</v>
+      </c>
+      <c r="P28" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>80</v>
+      </c>
+      <c r="R28" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>16.5</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="n">
+        <v>5</v>
+      </c>
+      <c r="O29" t="n">
+        <v>20</v>
+      </c>
+      <c r="P29" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>80</v>
+      </c>
+      <c r="R29" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Chinatrust Brothers</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="n">
+        <v>5</v>
+      </c>
+      <c r="O30" t="n">
+        <v>20</v>
+      </c>
+      <c r="P30" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>80</v>
+      </c>
+      <c r="R30" t="n">
         <v>80</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-13 18:26
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1380,6 +1380,1122 @@
       </c>
       <c r="R12" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3:10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="n">
+        <v>5</v>
+      </c>
+      <c r="O13" t="n">
+        <v>20</v>
+      </c>
+      <c r="P13" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>80</v>
+      </c>
+      <c r="R13" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>4:07</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>8-4</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>80.2</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>58.7</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="n">
+        <v>3</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="R14" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>5:05</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>64.4</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>39.2</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>100</v>
+      </c>
+      <c r="R15" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>5:05</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>5:10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>6-3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>5</v>
+      </c>
+      <c r="O17" t="n">
+        <v>20</v>
+      </c>
+      <c r="P17" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>80</v>
+      </c>
+      <c r="R17" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>5:10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>64.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>5</v>
+      </c>
+      <c r="O18" t="n">
+        <v>20</v>
+      </c>
+      <c r="P18" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>80</v>
+      </c>
+      <c r="R18" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>5:10</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>5:10</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>2</v>
+      </c>
+      <c r="O20" t="n">
+        <v>50</v>
+      </c>
+      <c r="P20" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>100</v>
+      </c>
+      <c r="R20" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>5:10</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>9.7</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>1</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>100</v>
+      </c>
+      <c r="R21" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>5</v>
+      </c>
+      <c r="O22" t="n">
+        <v>20</v>
+      </c>
+      <c r="P22" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>80</v>
+      </c>
+      <c r="R22" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="n">
+        <v>1</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>100</v>
+      </c>
+      <c r="R23" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>32.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>31.1</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>4</v>
+      </c>
+      <c r="O24" t="n">
+        <v>25</v>
+      </c>
+      <c r="P24" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>75</v>
+      </c>
+      <c r="R24" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>58.3</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>33.0</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>11:07</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>6-5</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>92.1</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>71.0</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>46.7</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="n">
+        <v>5</v>
+      </c>
+      <c r="O26" t="n">
+        <v>20</v>
+      </c>
+      <c r="P26" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>80</v>
+      </c>
+      <c r="R26" t="n">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-14 13:31
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:R22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,17 +511,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,37 +531,37 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,43 +571,35 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O2" t="n">
+        <v>20</v>
+      </c>
+      <c r="P2" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>80</v>
+      </c>
+      <c r="R2" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -617,37 +609,37 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,35 +649,43 @@
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>4</v>
-      </c>
-      <c r="O3" t="n">
-        <v>25</v>
-      </c>
-      <c r="P3" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>75</v>
-      </c>
-      <c r="R3" t="n">
-        <v>75</v>
+        <v>0</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,12 +695,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>73.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -735,35 +735,35 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="P4" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="Q4" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="R4" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -793,17 +793,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -831,17 +831,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -851,17 +851,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>73.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -871,17 +871,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -900,26 +900,26 @@
         <v>100</v>
       </c>
       <c r="Q6" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="R6" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -929,12 +929,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -954,12 +954,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -987,17 +987,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1007,37 +1007,37 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-6</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1047,19 +1047,27 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>3</v>
-      </c>
-      <c r="O8" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="P8" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>100</v>
-      </c>
-      <c r="R8" t="n">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -1070,12 +1078,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1085,22 +1093,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1-6</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1125,27 +1133,19 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O9" t="n">
+        <v>20</v>
+      </c>
+      <c r="P9" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>80</v>
+      </c>
+      <c r="R9" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="10">
@@ -1196,12 +1196,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>58.3</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>31.8</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1249,12 +1249,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1312,12 +1312,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1327,22 +1327,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1352,12 +1352,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>33.8</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1367,35 +1367,35 @@
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O12" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="P12" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="Q12" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="R12" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>1:15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1405,22 +1405,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>60.0</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>40.0</t>
-        </is>
-      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1430,12 +1430,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1445,35 +1445,43 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
-        <v>5</v>
-      </c>
-      <c r="O13" t="n">
-        <v>20</v>
-      </c>
-      <c r="P13" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>80</v>
-      </c>
-      <c r="R13" t="n">
-        <v>80</v>
+        <v>0</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4:07</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1483,17 +1491,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>8-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1503,17 +1511,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>80.2</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>58.7</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1523,35 +1531,35 @@
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O14" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="P14" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="Q14" t="n">
-        <v>66.7</v>
+        <v>80</v>
       </c>
       <c r="R14" t="n">
-        <v>66.7</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>5:05</t>
+          <t>2:37</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1561,22 +1569,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>8-4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1586,12 +1594,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>64.4</t>
+          <t>80.2</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>39.2</t>
+          <t>58.7</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1601,35 +1609,35 @@
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="P15" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="Q15" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="R15" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>5:05</t>
+          <t>2:40</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1639,37 +1647,37 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1679,43 +1687,35 @@
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="O16" t="n">
+        <v>25</v>
+      </c>
+      <c r="P16" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>75</v>
+      </c>
+      <c r="R16" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>2:40</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1725,17 +1725,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1745,17 +1745,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1765,25 +1765,25 @@
       </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O17" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="P17" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="Q17" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="R17" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>2:40</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1803,17 +1803,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1823,17 +1823,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1861,17 +1861,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1881,37 +1881,37 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>43.0</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>57.0</t>
-        </is>
-      </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1921,43 +1921,35 @@
       </c>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O19" t="n">
+        <v>20</v>
+      </c>
+      <c r="P19" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>80</v>
+      </c>
+      <c r="R19" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1967,37 +1959,37 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2007,35 +1999,35 @@
       </c>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O20" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="P20" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="Q20" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="R20" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2045,17 +2037,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2065,17 +2057,17 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2085,35 +2077,43 @@
       </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="n">
-        <v>1</v>
-      </c>
-      <c r="O21" t="n">
         <v>0</v>
       </c>
-      <c r="P21" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>100</v>
-      </c>
-      <c r="R21" t="n">
-        <v>100</v>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>8:20</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2123,17 +2123,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2175,326 +2175,6 @@
         <v>80</v>
       </c>
       <c r="R22" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>8:10</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Kansas City Royals</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Houston Astros</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>46.0</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>54.0</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>3-5</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>42.1</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>19.4</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="n">
-        <v>1</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>100</v>
-      </c>
-      <c r="R23" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>11:05</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>San Francisco Giants</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>68.0</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>32.0</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>31.1</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>12.1</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="n">
-        <v>4</v>
-      </c>
-      <c r="O24" t="n">
-        <v>25</v>
-      </c>
-      <c r="P24" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>75</v>
-      </c>
-      <c r="R24" t="n">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>11:05</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Athletics</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Colorado Rockies</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>42.0</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>58.0</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>4-5</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>58.3</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>33.0</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>11:07</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Los Angeles Angels</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>62.0</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>38.0</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>6-5</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>92.1</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>71.0</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>46.7</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="n">
-        <v>5</v>
-      </c>
-      <c r="O26" t="n">
-        <v>20</v>
-      </c>
-      <c r="P26" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>80</v>
-      </c>
-      <c r="R26" t="n">
         <v>80</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-16 12:10
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:R18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,37 +511,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>60.8</t>
+          <t>14.3</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>35.5</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,40 +571,48 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O2" t="n">
-        <v>50</v>
-      </c>
-      <c r="P2" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>100</v>
-      </c>
-      <c r="R2" t="n">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -619,7 +627,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -629,17 +637,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>66.7</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>41.7</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -667,57 +675,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -727,75 +735,83 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>4</v>
-      </c>
-      <c r="O4" t="n">
-        <v>25</v>
-      </c>
-      <c r="P4" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>75</v>
-      </c>
-      <c r="R4" t="n">
-        <v>75</v>
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>8:45</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -805,13 +821,13 @@
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>66.7</v>
+        <v>100</v>
       </c>
       <c r="Q5" t="n">
         <v>100</v>
@@ -823,37 +839,37 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>76.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>24.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>8-3</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -863,17 +879,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>51.6</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -883,75 +899,83 @@
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O6" t="n">
-        <v>20</v>
-      </c>
-      <c r="P6" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>80</v>
-      </c>
-      <c r="R6" t="n">
-        <v>80</v>
+        <v>0</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>79.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6-2</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -961,68 +985,60 @@
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O7" t="n">
+        <v>50</v>
+      </c>
+      <c r="P7" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>100</v>
+      </c>
+      <c r="R7" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1032,12 +1048,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>64.4</t>
+          <t>63.2</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>39.2</t>
+          <t>37.9</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1047,35 +1063,43 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>3</v>
-      </c>
-      <c r="O8" t="n">
         <v>0</v>
       </c>
-      <c r="P8" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="R8" t="n">
-        <v>66.7</v>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1095,7 +1119,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1105,17 +1129,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1151,17 +1175,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1171,17 +1195,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>72.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>28.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1211,35 +1235,35 @@
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O10" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="Q10" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="R10" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1249,17 +1273,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1269,17 +1293,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1289,18 +1313,564 @@
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
+        <v>4</v>
+      </c>
+      <c r="O11" t="n">
+        <v>25</v>
+      </c>
+      <c r="P11" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>75</v>
+      </c>
+      <c r="R11" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>51.8</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="n">
+        <v>4</v>
+      </c>
+      <c r="O12" t="n">
+        <v>25</v>
+      </c>
+      <c r="P12" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>75</v>
+      </c>
+      <c r="R12" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>31.1</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>100</v>
+      </c>
+      <c r="R13" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>8:45</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>37.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>28.4</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>10.6</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="n">
         <v>5</v>
       </c>
-      <c r="O11" t="n">
+      <c r="O14" t="n">
         <v>20</v>
       </c>
-      <c r="P11" t="n">
+      <c r="P14" t="n">
         <v>80</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="Q14" t="n">
         <v>80</v>
       </c>
-      <c r="R11" t="n">
+      <c r="R14" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>9:05</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="n">
+        <v>5</v>
+      </c>
+      <c r="O15" t="n">
+        <v>20</v>
+      </c>
+      <c r="P15" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>80</v>
+      </c>
+      <c r="R15" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>2</v>
+      </c>
+      <c r="O16" t="n">
+        <v>50</v>
+      </c>
+      <c r="P16" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>100</v>
+      </c>
+      <c r="R16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Chinatrust Brothers</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>16.3</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>5</v>
+      </c>
+      <c r="O17" t="n">
+        <v>20</v>
+      </c>
+      <c r="P17" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>80</v>
+      </c>
+      <c r="R17" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>64.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>25.8</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>5</v>
+      </c>
+      <c r="O18" t="n">
+        <v>20</v>
+      </c>
+      <c r="P18" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>80</v>
+      </c>
+      <c r="R18" t="n">
         <v>80</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-17 15:06
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R18"/>
+  <dimension ref="A1:R22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,12 +516,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,37 +531,37 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,63 +571,55 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O2" t="n">
+        <v>20</v>
+      </c>
+      <c r="P2" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>80</v>
+      </c>
+      <c r="R2" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-6</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -637,17 +629,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,19 +649,27 @@
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>2</v>
-      </c>
-      <c r="O3" t="n">
-        <v>50</v>
-      </c>
-      <c r="P3" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>100</v>
-      </c>
-      <c r="R3" t="n">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -680,12 +680,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,17 +695,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>3-6</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,17 +715,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -781,37 +781,37 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>66.7</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>31.8</t>
+          <t>41.7</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,19 +821,19 @@
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="P5" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="Q5" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="R5" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6">
@@ -859,12 +859,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>76.0</t>
+          <t>82.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>24.0</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -884,12 +884,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>73.1</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>51.6</t>
+          <t>49.2</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -945,37 +945,37 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>48.0</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>52.0</t>
-        </is>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>47.7</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>31.8</t>
+          <t>23.7</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,13 +985,13 @@
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O7" t="n">
-        <v>50</v>
+        <v>33.3</v>
       </c>
       <c r="P7" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="Q7" t="n">
         <v>100</v>
@@ -1003,57 +1003,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>1:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>63.2</t>
+          <t>39.3</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>37.9</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1063,43 +1063,35 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P8" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>80</v>
+      </c>
+      <c r="R8" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>2:05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1109,37 +1101,37 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1149,43 +1141,35 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="O9" t="n">
+        <v>25</v>
+      </c>
+      <c r="P9" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>75</v>
+      </c>
+      <c r="R9" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>2:05</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1195,17 +1179,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>7-2</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1215,17 +1199,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1235,35 +1219,35 @@
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O10" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="P10" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="Q10" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="R10" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1273,17 +1257,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1293,17 +1277,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1313,35 +1297,35 @@
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O11" t="n">
-        <v>25</v>
+        <v>33.3</v>
       </c>
       <c r="P11" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="Q11" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="R11" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>3:15</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1351,17 +1335,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1371,17 +1355,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1409,17 +1393,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>4:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1429,22 +1413,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1454,12 +1438,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1469,35 +1453,35 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="P13" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="Q13" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="R13" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8:45</t>
+          <t>4:40</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1507,17 +1491,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1527,17 +1511,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1547,35 +1531,35 @@
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O14" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q14" t="n">
-        <v>80</v>
+        <v>66.7</v>
       </c>
       <c r="R14" t="n">
-        <v>80</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1585,17 +1569,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1605,17 +1589,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1625,35 +1609,35 @@
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O15" t="n">
-        <v>20</v>
+        <v>33.3</v>
       </c>
       <c r="P15" t="n">
-        <v>80</v>
+        <v>66.7</v>
       </c>
       <c r="Q15" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="R15" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1663,37 +1647,37 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>23.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>7-2</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1703,75 +1687,83 @@
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
-        <v>2</v>
-      </c>
-      <c r="O16" t="n">
-        <v>50</v>
-      </c>
-      <c r="P16" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>100</v>
-      </c>
-      <c r="R16" t="n">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>60.0</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>40.0</t>
-        </is>
-      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1781,55 +1773,63 @@
       </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
-        <v>5</v>
-      </c>
-      <c r="O17" t="n">
-        <v>20</v>
-      </c>
-      <c r="P17" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>80</v>
-      </c>
-      <c r="R17" t="n">
-        <v>80</v>
+        <v>0</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1839,17 +1839,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1859,19 +1859,331 @@
       </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="n">
+        <v>3</v>
+      </c>
+      <c r="O18" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P18" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>100</v>
+      </c>
+      <c r="R18" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>9:05</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>25.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>32.4</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>12.9</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>100</v>
+      </c>
+      <c r="R19" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>31.1</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>4</v>
+      </c>
+      <c r="O20" t="n">
+        <v>25</v>
+      </c>
+      <c r="P20" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>75</v>
+      </c>
+      <c r="R20" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
         <v>5</v>
       </c>
-      <c r="O18" t="n">
+      <c r="O21" t="n">
         <v>20</v>
       </c>
-      <c r="P18" t="n">
+      <c r="P21" t="n">
         <v>80</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="Q21" t="n">
         <v>80</v>
       </c>
-      <c r="R18" t="n">
+      <c r="R21" t="n">
         <v>80</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>4</v>
+      </c>
+      <c r="O22" t="n">
+        <v>25</v>
+      </c>
+      <c r="P22" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>75</v>
+      </c>
+      <c r="R22" t="n">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-18 11:34
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R22"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,37 +511,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>82.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>8-3</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>46.7</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,19 +571,27 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>5</v>
-      </c>
-      <c r="O2" t="n">
-        <v>20</v>
-      </c>
-      <c r="P2" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>80</v>
-      </c>
-      <c r="R2" t="n">
-        <v>80</v>
+        <v>0</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -594,12 +602,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -609,17 +617,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-6</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -629,17 +637,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -695,12 +703,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -844,12 +852,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,37 +867,37 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>82.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>8-3</t>
+          <t>3-6</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>73.1</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>49.2</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -925,57 +933,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>3:35</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>47.7</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>23.7</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,30 +993,38 @@
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>3</v>
-      </c>
-      <c r="O7" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="P7" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>100</v>
-      </c>
-      <c r="R7" t="n">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1:40</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1023,17 +1039,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,17 +1059,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1063,35 +1079,35 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O8" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q8" t="n">
-        <v>80</v>
+        <v>66.7</v>
       </c>
       <c r="R8" t="n">
-        <v>80</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2:05</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1101,37 +1117,37 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>65.6</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>40.4</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1141,55 +1157,63 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>4</v>
-      </c>
-      <c r="O9" t="n">
-        <v>25</v>
-      </c>
-      <c r="P9" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>75</v>
-      </c>
-      <c r="R9" t="n">
-        <v>75</v>
+        <v>0</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2:05</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7-2</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1199,17 +1223,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1237,57 +1261,57 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1297,55 +1321,63 @@
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>3</v>
-      </c>
-      <c r="O11" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="P11" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>100</v>
-      </c>
-      <c r="R11" t="n">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3:15</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1355,17 +1387,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>50.4</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>25.9</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1387,802 +1419,6 @@
         <v>75</v>
       </c>
       <c r="R12" t="n">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>4:10</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Los Angeles Dodgers</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>65.0</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>35.0</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>28.4</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>10.6</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="n">
-        <v>4</v>
-      </c>
-      <c r="O13" t="n">
-        <v>25</v>
-      </c>
-      <c r="P13" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>75</v>
-      </c>
-      <c r="R13" t="n">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>4:40</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Arizona Diamondbacks</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Los Angeles Angels</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>69.0</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>31.0</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>42.1</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>19.4</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="n">
-        <v>3</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="R14" t="n">
-        <v>66.7</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>7:45</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Toronto Blue Jays</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>52.0</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>48.0</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>51.8</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>27.1</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="n">
-        <v>3</v>
-      </c>
-      <c r="O15" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="P15" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>100</v>
-      </c>
-      <c r="R15" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>8:05</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>New York Yankees</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Chicago White Sox</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>77.0</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>23.0</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>7-2</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>54.4</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>29.4</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>8:15</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Atlanta Braves</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>San Francisco Giants</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>40.0</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>60.0</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>3-5</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>40.7</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>18.4</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>8:40</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Milwaukee Brewers</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Cleveland Guardians</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>52.0</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>48.0</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>3-2</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>23.8</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>11.4</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>2.8</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="n">
-        <v>3</v>
-      </c>
-      <c r="O18" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="P18" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>100</v>
-      </c>
-      <c r="R18" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>9:05</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Colorado Rockies</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>75.0</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>25.0</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>32.4</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>12.9</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="n">
-        <v>1</v>
-      </c>
-      <c r="O19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>100</v>
-      </c>
-      <c r="R19" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Seattle Mariners</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Baltimore Orioles</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>54.0</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>46.0</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>31.1</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>12.1</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="n">
-        <v>4</v>
-      </c>
-      <c r="O20" t="n">
-        <v>25</v>
-      </c>
-      <c r="P20" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>75</v>
-      </c>
-      <c r="R20" t="n">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>19:35</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>TSG Hawks</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Rakuten Monkeys</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>56.0</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>44.0</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>27.1</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>9.9</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="n">
-        <v>5</v>
-      </c>
-      <c r="O21" t="n">
-        <v>20</v>
-      </c>
-      <c r="P21" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>80</v>
-      </c>
-      <c r="R21" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>19:35</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Wei Chuan Dragons</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Fubon Guardians</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>27.1</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>9.9</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="n">
-        <v>4</v>
-      </c>
-      <c r="O22" t="n">
-        <v>25</v>
-      </c>
-      <c r="P22" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>75</v>
-      </c>
-      <c r="R22" t="n">
         <v>75</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-19 13:49
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,37 +511,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>82.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>8-3</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>46.7</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,58 +571,50 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O2" t="n">
+        <v>20</v>
+      </c>
+      <c r="P2" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>80</v>
+      </c>
+      <c r="R2" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -642,12 +634,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,83 +649,75 @@
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O3" t="n">
+        <v>50</v>
+      </c>
+      <c r="P3" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>100</v>
+      </c>
+      <c r="R3" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-6</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -743,63 +727,55 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P4" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>80</v>
+      </c>
+      <c r="R4" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>72.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>28.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -809,17 +785,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>66.7</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>41.7</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -829,75 +805,75 @@
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O5" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="Q5" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="R5" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-6</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>55.7</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>30.6</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -907,63 +883,55 @@
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
+        <v>3</v>
+      </c>
+      <c r="O6" t="n">
         <v>0</v>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P6" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="R6" t="n">
+        <v>66.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3:35</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -973,17 +941,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1019,37 +987,37 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1059,17 +1027,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>46.3</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>22.6</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1082,52 +1050,52 @@
         <v>3</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="P8" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="Q8" t="n">
-        <v>66.7</v>
+        <v>100</v>
       </c>
       <c r="R8" t="n">
-        <v>66.7</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1137,17 +1105,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>65.6</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>40.4</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1183,37 +1151,37 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1223,17 +1191,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1261,57 +1229,57 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1321,63 +1289,55 @@
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O11" t="n">
+        <v>20</v>
+      </c>
+      <c r="P11" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>80</v>
+      </c>
+      <c r="R11" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1387,17 +1347,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>47.7</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>23.7</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1407,19 +1367,1291 @@
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
+        <v>3</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="R12" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3:20</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>40.7</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="n">
         <v>4</v>
       </c>
-      <c r="O12" t="n">
+      <c r="O13" t="n">
         <v>25</v>
       </c>
-      <c r="P12" t="n">
+      <c r="P13" t="n">
         <v>75</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="Q13" t="n">
         <v>75</v>
       </c>
-      <c r="R12" t="n">
+      <c r="R13" t="n">
         <v>75</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>31.1</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="n">
+        <v>5</v>
+      </c>
+      <c r="O14" t="n">
+        <v>20</v>
+      </c>
+      <c r="P14" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>80</v>
+      </c>
+      <c r="R14" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>8:05</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>100</v>
+      </c>
+      <c r="R15" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>43.5</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>100</v>
+      </c>
+      <c r="R16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>100</v>
+      </c>
+      <c r="R17" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>9:05</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>5</v>
+      </c>
+      <c r="O20" t="n">
+        <v>20</v>
+      </c>
+      <c r="P20" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>80</v>
+      </c>
+      <c r="R20" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>9:15</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>65.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>4</v>
+      </c>
+      <c r="O21" t="n">
+        <v>25</v>
+      </c>
+      <c r="P21" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>75</v>
+      </c>
+      <c r="R21" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>9:40</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>5-6</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>92.1</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>74.0</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>50.4</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>100</v>
+      </c>
+      <c r="R22" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="n">
+        <v>3</v>
+      </c>
+      <c r="O23" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P23" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>100</v>
+      </c>
+      <c r="R23" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>74.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>53.1</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>28.2</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>1</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>100</v>
+      </c>
+      <c r="R24" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>18.5</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="n">
+        <v>1</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>100</v>
+      </c>
+      <c r="R25" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>28.0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>51.8</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="n">
+        <v>2</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>50</v>
+      </c>
+      <c r="R26" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Chinatrust Brothers</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>28.4</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>10.6</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="n">
+        <v>4</v>
+      </c>
+      <c r="O27" t="n">
+        <v>25</v>
+      </c>
+      <c r="P27" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>75</v>
+      </c>
+      <c r="R27" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>39.0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>61.0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>36.6</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-20 16:14
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R28"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,17 +511,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>35.2</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>14.6</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -589,17 +589,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -609,37 +609,37 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>72.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>28.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -652,22 +652,22 @@
         <v>2</v>
       </c>
       <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q3" t="n">
         <v>50</v>
       </c>
-      <c r="P3" t="n">
+      <c r="R3" t="n">
         <v>50</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>100</v>
-      </c>
-      <c r="R3" t="n">
-        <v>100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -707,17 +707,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -727,35 +727,35 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O4" t="n">
-        <v>20</v>
+        <v>33.3</v>
       </c>
       <c r="P4" t="n">
-        <v>80</v>
+        <v>66.7</v>
       </c>
       <c r="Q4" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="R4" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -765,17 +765,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -785,17 +785,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -805,19 +805,19 @@
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="P5" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="Q5" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="R5" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6">
@@ -828,12 +828,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -843,17 +843,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -863,17 +863,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -883,19 +883,19 @@
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="P6" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="Q6" t="n">
-        <v>66.7</v>
+        <v>80</v>
       </c>
       <c r="R6" t="n">
-        <v>66.7</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7">
@@ -931,7 +931,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -941,17 +941,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -987,17 +987,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1007,17 +1007,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1027,17 +1027,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>46.3</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>22.6</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1047,35 +1047,35 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O8" t="n">
-        <v>33.3</v>
+        <v>20</v>
       </c>
       <c r="P8" t="n">
-        <v>66.7</v>
+        <v>80</v>
       </c>
       <c r="Q8" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="R8" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1085,37 +1085,37 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>47.7</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>23.7</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1125,43 +1125,35 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="O9" t="n">
+        <v>25</v>
+      </c>
+      <c r="P9" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>75</v>
+      </c>
+      <c r="R9" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1171,37 +1163,37 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1211,35 +1203,43 @@
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
-        <v>5</v>
-      </c>
-      <c r="O10" t="n">
-        <v>20</v>
-      </c>
-      <c r="P10" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>80</v>
-      </c>
-      <c r="R10" t="n">
-        <v>80</v>
+        <v>0</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1249,17 +1249,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>6-5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>66.7</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>41.7</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1307,17 +1307,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1327,22 +1327,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1352,12 +1352,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>47.7</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>23.7</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1367,35 +1367,43 @@
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
-        <v>3</v>
-      </c>
-      <c r="O12" t="n">
         <v>0</v>
       </c>
-      <c r="P12" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="R12" t="n">
-        <v>66.7</v>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3:20</t>
+          <t>2:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1405,17 +1413,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1425,17 +1433,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1445,35 +1453,35 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="P13" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="Q13" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="R13" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1483,17 +1491,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1503,17 +1511,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1541,17 +1549,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>3:20</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1561,17 +1569,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1581,17 +1589,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1619,17 +1627,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>5:05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1639,37 +1647,37 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1679,25 +1687,25 @@
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O16" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="P16" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="Q16" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="R16" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1717,37 +1725,37 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>39.3</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1757,13 +1765,13 @@
       </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O17" t="n">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="P17" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="Q17" t="n">
         <v>100</v>
@@ -1775,17 +1783,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1795,37 +1803,37 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>42.0</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>58.0</t>
-        </is>
-      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1835,43 +1843,35 @@
       </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O18" t="n">
+        <v>20</v>
+      </c>
+      <c r="P18" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>80</v>
+      </c>
+      <c r="R18" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1881,17 +1881,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1901,17 +1901,17 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1947,17 +1947,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1967,17 +1967,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1987,17 +1987,17 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2025,17 +2025,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>9:15</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2045,37 +2045,37 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>3-1</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2085,25 +2085,33 @@
       </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="n">
-        <v>4</v>
-      </c>
-      <c r="O21" t="n">
-        <v>25</v>
-      </c>
-      <c r="P21" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>75</v>
-      </c>
-      <c r="R21" t="n">
-        <v>75</v>
+        <v>0</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2123,37 +2131,37 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2163,35 +2171,35 @@
       </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O22" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="P22" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="Q22" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="R22" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>11:05</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2201,37 +2209,37 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>51.6</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2241,13 +2249,13 @@
       </c>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O23" t="n">
-        <v>33.3</v>
+        <v>50</v>
       </c>
       <c r="P23" t="n">
-        <v>66.7</v>
+        <v>50</v>
       </c>
       <c r="Q23" t="n">
         <v>100</v>
@@ -2279,12 +2287,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2304,12 +2312,12 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2319,7 +2327,7 @@
       </c>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
@@ -2328,10 +2336,10 @@
         <v>100</v>
       </c>
       <c r="Q24" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="R24" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="25">
@@ -2342,12 +2350,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2357,37 +2365,37 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>7-4</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>50.4</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2397,7 +2405,7 @@
       </c>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
@@ -2406,66 +2414,66 @@
         <v>100</v>
       </c>
       <c r="Q25" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="R25" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2475,37 +2483,45 @@
       </c>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="n">
-        <v>2</v>
-      </c>
-      <c r="O26" t="n">
         <v>0</v>
       </c>
-      <c r="P26" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>50</v>
-      </c>
-      <c r="R26" t="n">
-        <v>50</v>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
           <t>Chinatrust Brothers</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Fubon Guardians</t>
-        </is>
-      </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>CPB</t>
@@ -2513,37 +2529,37 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>3-6</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>49.1</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>24.8</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2553,30 +2569,38 @@
       </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="n">
-        <v>4</v>
-      </c>
-      <c r="O27" t="n">
-        <v>25</v>
-      </c>
-      <c r="P27" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>75</v>
-      </c>
-      <c r="R27" t="n">
-        <v>75</v>
+        <v>0</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2591,37 +2615,37 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2631,27 +2655,97 @@
       </c>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="n">
+        <v>5</v>
+      </c>
+      <c r="O28" t="n">
+        <v>20</v>
+      </c>
+      <c r="P28" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>80</v>
+      </c>
+      <c r="R28" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>69.0</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>31.0</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="n">
+        <v>3</v>
+      </c>
+      <c r="O29" t="n">
         <v>0</v>
       </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P29" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="R29" t="n">
+        <v>66.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-23 10:59
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:R17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,17 +511,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,37 +531,37 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,83 +571,75 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O2" t="n">
         <v>0</v>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P2" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="R2" t="n">
+        <v>66.7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>7:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,55 +649,55 @@
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O3" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="Q3" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="R3" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,17 +707,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,63 +727,55 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
         <v>0</v>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -801,17 +785,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -839,57 +823,57 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>64.4</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>39.2</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,50 +883,50 @@
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="P6" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="Q6" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="R6" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>8:07</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -962,12 +946,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -977,65 +961,65 @@
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="Q7" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="R7" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1055,75 +1039,75 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O8" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="P8" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="Q8" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="R8" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3-6</t>
+          <t>6-5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>65.6</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>40.4</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1133,63 +1117,55 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="O9" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P9" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>100</v>
+      </c>
+      <c r="R9" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1199,17 +1175,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>64.4</t>
+          <t>68.9</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>39.2</t>
+          <t>44.2</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1219,63 +1195,55 @@
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
+        <v>2</v>
+      </c>
+      <c r="O10" t="n">
         <v>0</v>
       </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P10" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>50</v>
+      </c>
+      <c r="R10" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1285,17 +1253,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1305,75 +1273,75 @@
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O11" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>8:45</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1383,35 +1351,35 @@
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O12" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1421,37 +1389,37 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6-8</t>
+          <t>6-5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>98.6</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>90.9</t>
+          <t>65.6</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>76.5</t>
+          <t>40.4</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1461,43 +1429,35 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="O13" t="n">
+        <v>25</v>
+      </c>
+      <c r="P13" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>75</v>
+      </c>
+      <c r="R13" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>10:38</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1507,37 +1467,37 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1547,63 +1507,55 @@
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O14" t="n">
+        <v>20</v>
+      </c>
+      <c r="P14" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>80</v>
+      </c>
+      <c r="R14" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1613,17 +1565,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1633,19 +1585,175 @@
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
+        <v>5</v>
+      </c>
+      <c r="O15" t="n">
+        <v>20</v>
+      </c>
+      <c r="P15" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>80</v>
+      </c>
+      <c r="R15" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>4</v>
+      </c>
+      <c r="O16" t="n">
+        <v>25</v>
+      </c>
+      <c r="P16" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>75</v>
+      </c>
+      <c r="R16" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>9.7</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
         <v>3</v>
       </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="n">
+      <c r="O17" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P17" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q17" t="n">
         <v>100</v>
       </c>
-      <c r="Q15" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="R15" t="n">
-        <v>66.7</v>
+      <c r="R17" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-24 11:50
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R17"/>
+  <dimension ref="A1:R21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,17 +531,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>26.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,19 +571,27 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O2" t="n">
         <v>0</v>
       </c>
-      <c r="P2" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="R2" t="n">
-        <v>66.7</v>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -594,12 +602,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -609,17 +617,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>5-1</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -629,17 +637,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -649,19 +657,27 @@
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>3</v>
-      </c>
-      <c r="O3" t="n">
         <v>0</v>
       </c>
-      <c r="P3" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="R3" t="n">
-        <v>66.7</v>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -672,12 +688,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -687,37 +703,37 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -727,19 +743,27 @@
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O4" t="n">
         <v>0</v>
       </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0</v>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -750,12 +774,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -765,17 +789,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -785,17 +809,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>23.3</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>7.9</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -805,19 +829,27 @@
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>5</v>
-      </c>
-      <c r="O5" t="n">
-        <v>20</v>
-      </c>
-      <c r="P5" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>80</v>
-      </c>
-      <c r="R5" t="n">
-        <v>80</v>
+        <v>0</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -828,12 +860,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -843,17 +875,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -863,17 +895,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -883,55 +915,63 @@
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O6" t="n">
-        <v>20</v>
-      </c>
-      <c r="P6" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>80</v>
-      </c>
-      <c r="R6" t="n">
-        <v>80</v>
+        <v>0</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -941,17 +981,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -961,19 +1001,27 @@
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>2</v>
-      </c>
-      <c r="O7" t="n">
         <v>0</v>
       </c>
-      <c r="P7" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R7" t="n">
-        <v>50</v>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -984,12 +1032,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -999,17 +1047,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1019,17 +1067,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1039,19 +1087,27 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>2</v>
-      </c>
-      <c r="O8" t="n">
-        <v>50</v>
-      </c>
-      <c r="P8" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>100</v>
-      </c>
-      <c r="R8" t="n">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -1062,12 +1118,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1087,7 +1143,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>6-5</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1097,17 +1153,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>65.6</t>
+          <t>58.3</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>40.4</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1117,19 +1173,27 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>3</v>
-      </c>
-      <c r="O9" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="P9" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>100</v>
-      </c>
-      <c r="R9" t="n">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1140,12 +1204,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1155,37 +1219,37 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>68.9</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>44.2</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1195,19 +1259,27 @@
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
-        <v>2</v>
-      </c>
-      <c r="O10" t="n">
         <v>0</v>
       </c>
-      <c r="P10" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>50</v>
-      </c>
-      <c r="R10" t="n">
-        <v>50</v>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -1218,12 +1290,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1233,17 +1305,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1253,17 +1325,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1273,65 +1345,73 @@
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>1</v>
-      </c>
-      <c r="O11" t="n">
         <v>0</v>
       </c>
-      <c r="P11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0</v>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>2:10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1351,35 +1431,43 @@
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
-        <v>1</v>
-      </c>
-      <c r="O12" t="n">
         <v>0</v>
       </c>
-      <c r="P12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" t="n">
-        <v>0</v>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1389,22 +1477,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6-5</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1414,12 +1502,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>65.6</t>
+          <t>59.6</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>40.4</t>
+          <t>34.2</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1429,35 +1517,43 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
-        <v>4</v>
-      </c>
-      <c r="O13" t="n">
-        <v>25</v>
-      </c>
-      <c r="P13" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>75</v>
-      </c>
-      <c r="R13" t="n">
-        <v>75</v>
+        <v>0</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>8:07</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1467,37 +1563,37 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1507,75 +1603,83 @@
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
-        <v>5</v>
-      </c>
-      <c r="O14" t="n">
-        <v>20</v>
-      </c>
-      <c r="P14" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>80</v>
-      </c>
-      <c r="R14" t="n">
-        <v>80</v>
+        <v>0</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>56.0</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>44.0</t>
-        </is>
-      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1585,19 +1689,27 @@
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
-        <v>5</v>
-      </c>
-      <c r="O15" t="n">
-        <v>20</v>
-      </c>
-      <c r="P15" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>80</v>
-      </c>
-      <c r="R15" t="n">
-        <v>80</v>
+        <v>0</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -1608,7 +1720,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1623,37 +1735,37 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1663,19 +1775,27 @@
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
-        <v>4</v>
-      </c>
-      <c r="O16" t="n">
-        <v>25</v>
-      </c>
-      <c r="P16" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>75</v>
-      </c>
-      <c r="R16" t="n">
-        <v>75</v>
+        <v>0</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -1686,12 +1806,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1701,17 +1821,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1721,17 +1841,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>47.7</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>23.7</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1741,19 +1861,371 @@
       </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
-        <v>3</v>
-      </c>
-      <c r="O17" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="P17" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>100</v>
-      </c>
-      <c r="R17" t="n">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1:05</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sugar Land</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>El Paso Chihuahuas</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>PCL</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>31.8</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>3:00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Holguin</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Las Tunas</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>LIE</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>28.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>6-10</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>99.6</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>97.5</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>91.6</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>7:05</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Norfolk Tides</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Durham Bulls</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>3-7</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>66.7</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>41.7</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>8:04</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Charlotte Knights</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Rochester Red Wings</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>28.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>84.5</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>65.3</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-26 13:14
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:R34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,17 +511,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -617,37 +617,37 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5-1</t>
+          <t>1-4</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -688,12 +688,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -703,22 +703,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -728,12 +728,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -774,12 +774,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -789,22 +789,22 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -814,12 +814,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>23.3</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>7.9</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -855,17 +855,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -875,22 +875,22 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -946,12 +946,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -961,17 +961,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -981,17 +981,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1032,12 +1032,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1047,37 +1047,37 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1118,12 +1118,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1133,12 +1133,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1158,12 +1158,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>58.3</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1204,12 +1204,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1244,12 +1244,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1305,17 +1305,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>2-5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1325,17 +1325,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1371,17 +1371,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2:10</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1391,12 +1391,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1416,12 +1416,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1457,17 +1457,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>8:07</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1477,37 +1477,37 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
           <t>55.0</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>5-6</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>92.1</t>
-        </is>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>59.6</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>34.2</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1543,17 +1543,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8:07</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1563,37 +1563,37 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1649,37 +1649,37 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1715,37 +1715,37 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1755,17 +1755,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1801,32 +1801,32 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1846,12 +1846,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>47.7</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>23.7</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1887,57 +1887,57 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1:05</t>
+          <t>8:45</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Sugar Land</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>El Paso Chihuahuas</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PCL</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>47.0</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>31.8</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1973,57 +1973,57 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3:00</t>
+          <t>9:10</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Holguin</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Las Tunas</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>LIE</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>26.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>6-10</t>
+          <t>5-1</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>99.6</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>97.5</t>
+          <t>23.3</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>91.6</t>
+          <t>7.9</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2059,57 +2059,57 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>7:05</t>
+          <t>9:15</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Norfolk Tides</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Durham Bulls</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>3-7</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>66.7</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>41.7</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2145,57 +2145,57 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>8:04</t>
+          <t>10:38</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Charlotte Knights</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Rochester Red Wings</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>84.5</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>65.3</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2223,6 +2223,1124 @@
         </is>
       </c>
       <c r="R21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>18.5</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>16.3</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Chinatrust Brothers</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>36.6</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2:00</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Vienna Wanderers</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Traiskirchen</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>BUN</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>8-6</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>98.6</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>92.5</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>79.6</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>3:00</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Mayabeque</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Industriales</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>LIE</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>5-6</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>92.1</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>78.5</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>56.4</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>3:00</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Holguin</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Las Tunas</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>LIE</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>8-11</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>99.9</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>99.4</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>97.5</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>7:35</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Norfolk Tides</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Durham Bulls</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>65.0</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>31.8</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Worcester</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Toledo Mud Hens</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>31.1</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>8:04</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Charlotte Knights</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Rochester Red Wings</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>9-7</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>99.6</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>96.8</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>89.5</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>8:05</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Indianapolis Indians</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Scranton/WB</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>6-5</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>92.1</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>75.9</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>52.8</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>8:35</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Nashville Sounds</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Gwinnett Stripers</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>80.0</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>6-2</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>43.5</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>9:35</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Albuquerque Isotopes</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Salt Lake Bees</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>PCL</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>73.1</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>49.2</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-27 11:21
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R34"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,12 +516,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,47 +551,43 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>47.7</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>23.7</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>11</v>
+      </c>
+      <c r="O2" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="P2" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -602,12 +598,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -617,17 +613,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1-4</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -642,42 +638,38 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>13</v>
+      </c>
+      <c r="O3" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="P3" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -688,12 +680,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -703,22 +695,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -728,58 +720,54 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>13</v>
+      </c>
+      <c r="O4" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="P4" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -789,12 +777,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -814,63 +802,59 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>13</v>
+      </c>
+      <c r="O5" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="P5" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -885,7 +869,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -895,63 +879,59 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>13</v>
+      </c>
+      <c r="O6" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="P6" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -961,73 +941,69 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>13</v>
+      </c>
+      <c r="O7" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="P7" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1082,48 +1058,44 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>13</v>
+      </c>
+      <c r="O8" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="P8" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1133,12 +1105,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1158,164 +1130,156 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>12</v>
+      </c>
+      <c r="O9" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P9" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>2-6</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="N10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>13</v>
+      </c>
+      <c r="O10" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="P10" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2-5</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1325,255 +1289,243 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>35.2</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>14.6</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="N11" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>13</v>
+      </c>
+      <c r="O11" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="P11" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>1:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Bonn</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Regensburg</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>BUD</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>58.3</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="N12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>13</v>
+      </c>
+      <c r="O12" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="P12" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8:07</t>
+          <t>1:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Paderborn</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Mainz</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>BUD</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>64.4</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>39.2</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="N13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>9</v>
+      </c>
+      <c r="O13" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="P13" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Sundbyberg</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Leksand</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>ELT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>10-6</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1583,169 +1535,161 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>99.6</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>97.7</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>91.9</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>9</v>
+      </c>
+      <c r="O14" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P14" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Traiskirchen</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Vienna Wanderers</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>BUN</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>85.8</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>67.3</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="N15" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>13</v>
+      </c>
+      <c r="O15" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="P15" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>BSC Grosseto</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Collecchio</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>SA1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1755,68 +1699,64 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>9</v>
+      </c>
+      <c r="O16" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="P16" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Savigny</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>La Rochelle</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>DV1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1831,7 +1771,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1841,103 +1781,99 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>83.8</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>64.2</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N17" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>9</v>
+      </c>
+      <c r="O17" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P17" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>8:45</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>14.3</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1947,83 +1883,75 @@
       </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O18" t="n">
+        <v>40</v>
+      </c>
+      <c r="P18" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>5-1</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>23.3</t>
+          <t>39.3</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>7.9</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2033,83 +1961,75 @@
       </c>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O19" t="n">
+        <v>40</v>
+      </c>
+      <c r="P19" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>9:15</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>2-5</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2119,63 +2039,55 @@
       </c>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O20" t="n">
+        <v>40</v>
+      </c>
+      <c r="P20" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10:38</t>
+          <t>1:00</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Wr. Neustadt</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Vienna Metrostars</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>BUN</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>7-6</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2185,17 +2097,17 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>97.4</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>91.3</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>77.3</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2205,63 +2117,55 @@
       </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>2:00</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Heidenheim</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>BUD</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2271,17 +2175,17 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2291,63 +2195,55 @@
       </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>7</v>
+      </c>
+      <c r="O22" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="P22" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Expos</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>XL5</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>SMS</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>10-7</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2357,17 +2253,17 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>99.8</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>99.1</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>96.1</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2377,63 +2273,55 @@
       </c>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Stockholm</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Rattvik</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>ELT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>88.0</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-9</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2443,17 +2331,17 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>85.8</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>67.3</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2489,57 +2377,57 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Hunstetten</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>BDN</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>6-2</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2549,68 +2437,60 @@
       </c>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Vienna Wanderers</t>
+          <t>Beziers Pirates</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Traiskirchen</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>BUN</t>
+          <t>DV1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>8-6</t>
+          <t>6-8</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2620,12 +2500,12 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>92.5</t>
+          <t>93.5</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>79.6</t>
+          <t>81.8</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2635,63 +2515,55 @@
       </c>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>7</v>
+      </c>
+      <c r="O26" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="P26" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Mayabeque</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Industriales</t>
+          <t>Rouen</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>LIE</t>
+          <t>DV1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2701,17 +2573,17 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>78.5</t>
+          <t>84.5</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>56.4</t>
+          <t>65.3</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2721,83 +2593,75 @@
       </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="O27" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="P27" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Holguin</t>
+          <t>Senart</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Las Tunas</t>
+          <t>Stade Toulousain</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>LIE</t>
+          <t>DV1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
           <t>34.0</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>66.0</t>
-        </is>
-      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>8-11</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>99.9</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>99.4</t>
+          <t>58.3</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>97.5</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2807,543 +2671,19 @@
       </c>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>7:35</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Norfolk Tides</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Durham Bulls</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>35.0</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>65.0</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>4-5</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>57.0</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>31.8</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>7:45</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Worcester</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Toledo Mud Hens</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>41.0</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>59.0</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>3-4</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>31.1</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>12.1</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>8:04</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Charlotte Knights</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Rochester Red Wings</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>9-7</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>99.6</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>96.8</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>89.5</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>8:05</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Indianapolis Indians</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Scranton/WB</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>56.0</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>44.0</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>6-5</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>92.1</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>75.9</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>52.8</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>8:35</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Nashville Sounds</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Gwinnett Stripers</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>IL</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>80.0</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>6-2</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>43.5</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>20.4</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>9:35</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Albuquerque Isotopes</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Salt Lake Bees</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>PCL</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>49.0</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>51.0</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>5-7</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>95.4</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>73.1</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>49.2</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-06-30 12:22
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,37 +511,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,79 +551,75 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="O2" t="n">
-        <v>46.2</v>
+        <v>25</v>
       </c>
       <c r="P2" t="n">
-        <v>46.2</v>
+        <v>75</v>
       </c>
       <c r="Q2" t="n">
-        <v>7.7</v>
+        <v>75</v>
       </c>
       <c r="R2" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,79 +629,75 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>36.7</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="O3" t="n">
-        <v>46.7</v>
+        <v>20</v>
       </c>
       <c r="P3" t="n">
-        <v>46.7</v>
+        <v>80</v>
       </c>
       <c r="Q3" t="n">
-        <v>6.7</v>
+        <v>80</v>
       </c>
       <c r="R3" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,79 +707,75 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>49.1</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>24.8</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="O4" t="n">
-        <v>46.2</v>
+        <v>25</v>
       </c>
       <c r="P4" t="n">
-        <v>46.2</v>
+        <v>75</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.7</v>
+        <v>75</v>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Monclova</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Toros de Tijuana</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>LMB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,79 +785,75 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="O5" t="n">
-        <v>46.2</v>
+        <v>33.3</v>
       </c>
       <c r="P5" t="n">
-        <v>46.2</v>
+        <v>66.7</v>
       </c>
       <c r="Q5" t="n">
-        <v>7.7</v>
+        <v>100</v>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Oaxaca</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Diablos Rojos</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LMB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -879,79 +863,75 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="O6" t="n">
-        <v>46.7</v>
+        <v>33.3</v>
       </c>
       <c r="P6" t="n">
-        <v>40</v>
+        <v>66.7</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R6" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -966,74 +946,70 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>23.3</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>7.9</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="O7" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>55.6</v>
+        <v>100</v>
       </c>
       <c r="Q7" t="n">
-        <v>11.1</v>
+        <v>66.7</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,119 +1019,111 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="O8" t="n">
-        <v>55.6</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>38.9</v>
+        <v>50</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>65.6</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>40.4</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>38.5</v>
+        <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>53.8</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
         <v>0</v>
@@ -1167,37 +1135,37 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,79 +1175,75 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="O10" t="n">
-        <v>33.3</v>
+        <v>20</v>
       </c>
       <c r="P10" t="n">
-        <v>55.6</v>
+        <v>80</v>
       </c>
       <c r="Q10" t="n">
-        <v>11.1</v>
+        <v>80</v>
       </c>
       <c r="R10" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1289,37 +1253,33 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="O11" t="n">
-        <v>55.6</v>
+        <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>38.9</v>
+        <v>0</v>
       </c>
       <c r="Q11" t="n">
         <v>0</v>
@@ -1331,99 +1291,95 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>6-7</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>97.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>85.8</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>67.3</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="O12" t="n">
-        <v>60</v>
+        <v>33.3</v>
       </c>
       <c r="P12" t="n">
-        <v>40</v>
+        <v>66.7</v>
       </c>
       <c r="Q12" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="R12" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>7:35</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1433,22 +1389,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1473,19 +1429,19 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O13" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="Q13" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14">
@@ -1511,17 +1467,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>6-2</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1531,17 +1487,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1551,19 +1507,19 @@
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O14" t="n">
-        <v>50</v>
+        <v>33.3</v>
       </c>
       <c r="P14" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="Q14" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="R14" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
@@ -1589,17 +1545,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>72.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>28.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1609,17 +1565,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>59.6</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>34.2</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1629,35 +1585,35 @@
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O15" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="Q15" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="R15" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1667,17 +1623,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1687,17 +1643,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>81.7</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>60.9</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1707,19 +1663,253 @@
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="O16" t="n">
-        <v>57.1</v>
+        <v>0</v>
       </c>
       <c r="P16" t="n">
-        <v>42.9</v>
+        <v>50</v>
       </c>
       <c r="Q16" t="n">
-        <v>14.3</v>
+        <v>50</v>
       </c>
       <c r="R16" t="n">
-        <v>14.3</v>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>65.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>32.4</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>12.9</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>4</v>
+      </c>
+      <c r="O17" t="n">
+        <v>25</v>
+      </c>
+      <c r="P17" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>75</v>
+      </c>
+      <c r="R17" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>15.3</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>5</v>
+      </c>
+      <c r="O19" t="n">
+        <v>20</v>
+      </c>
+      <c r="P19" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>80</v>
+      </c>
+      <c r="R19" t="n">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-01 12:29
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,12 +516,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,75 +551,79 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr"/>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N2" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="O2" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="P2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="Q2" t="n">
         <v>25</v>
       </c>
-      <c r="P2" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>75</v>
-      </c>
       <c r="R2" t="n">
-        <v>75</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -634,34 +638,38 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="O3" t="n">
-        <v>20</v>
+        <v>58.3</v>
       </c>
       <c r="P3" t="n">
-        <v>80</v>
+        <v>33.3</v>
       </c>
       <c r="Q3" t="n">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="R3" t="n">
-        <v>80</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -672,12 +680,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -687,17 +695,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -707,39 +715,43 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>49.1</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>24.8</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr"/>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N4" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="O4" t="n">
-        <v>25</v>
+        <v>53.8</v>
       </c>
       <c r="P4" t="n">
-        <v>75</v>
+        <v>38.5</v>
       </c>
       <c r="Q4" t="n">
-        <v>75</v>
+        <v>23.1</v>
       </c>
       <c r="R4" t="n">
-        <v>75</v>
+        <v>23.1</v>
       </c>
     </row>
     <row r="5">
@@ -750,12 +762,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -765,7 +777,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -775,7 +787,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -785,39 +797,43 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr"/>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N5" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="O5" t="n">
-        <v>33.3</v>
+        <v>53.8</v>
       </c>
       <c r="P5" t="n">
-        <v>66.7</v>
+        <v>38.5</v>
       </c>
       <c r="Q5" t="n">
-        <v>100</v>
+        <v>23.1</v>
       </c>
       <c r="R5" t="n">
-        <v>100</v>
+        <v>23.1</v>
       </c>
     </row>
     <row r="6">
@@ -828,12 +844,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -843,12 +859,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -868,70 +884,74 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr"/>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N6" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="O6" t="n">
-        <v>33.3</v>
+        <v>53.3</v>
       </c>
       <c r="P6" t="n">
-        <v>66.7</v>
+        <v>40</v>
       </c>
       <c r="Q6" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="R6" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -941,39 +961,43 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>23.3</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>7.9</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr"/>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N7" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>53.3</v>
       </c>
       <c r="P7" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="Q7" t="n">
-        <v>66.7</v>
+        <v>20</v>
       </c>
       <c r="R7" t="n">
-        <v>66.7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
@@ -984,12 +1008,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -999,173 +1023,181 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>46.0</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>54.0</t>
-        </is>
-      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr"/>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N8" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>53.3</v>
       </c>
       <c r="P8" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="Q8" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="R8" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>65.6</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>40.4</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr"/>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N9" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>53.8</v>
       </c>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>38.5</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>23.1</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>23.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1175,153 +1207,161 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>36.7</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N10" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="O10" t="n">
-        <v>20</v>
+        <v>53.8</v>
       </c>
       <c r="P10" t="n">
-        <v>80</v>
+        <v>38.5</v>
       </c>
       <c r="Q10" t="n">
-        <v>80</v>
+        <v>23.1</v>
       </c>
       <c r="R10" t="n">
-        <v>80</v>
+        <v>23.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>9:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr"/>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N11" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="O11" t="n">
-        <v>0</v>
+        <v>52.9</v>
       </c>
       <c r="P11" t="n">
-        <v>0</v>
+        <v>41.2</v>
       </c>
       <c r="Q11" t="n">
-        <v>0</v>
+        <v>23.5</v>
       </c>
       <c r="R11" t="n">
-        <v>0</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1331,133 +1371,141 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr"/>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N12" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="O12" t="n">
-        <v>33.3</v>
+        <v>53.8</v>
       </c>
       <c r="P12" t="n">
-        <v>66.7</v>
+        <v>38.5</v>
       </c>
       <c r="Q12" t="n">
-        <v>100</v>
+        <v>30.8</v>
       </c>
       <c r="R12" t="n">
-        <v>100</v>
+        <v>30.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>49.1</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>24.8</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N13" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>44.4</v>
       </c>
       <c r="P13" t="n">
-        <v>50</v>
+        <v>44.4</v>
       </c>
       <c r="Q13" t="n">
-        <v>50</v>
+        <v>22.2</v>
       </c>
       <c r="R13" t="n">
-        <v>50</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>4:07</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1467,75 +1515,79 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>52.0</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>48.0</t>
-        </is>
-      </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="N14" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="O14" t="n">
-        <v>33.3</v>
+        <v>54.5</v>
       </c>
       <c r="P14" t="n">
-        <v>66.7</v>
+        <v>36.4</v>
       </c>
       <c r="Q14" t="n">
-        <v>100</v>
+        <v>18.2</v>
       </c>
       <c r="R14" t="n">
-        <v>100</v>
+        <v>18.2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8:07</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1545,22 +1597,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1570,70 +1622,74 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>59.6</t>
+          <t>63.2</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>34.2</t>
+          <t>37.9</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr"/>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="N15" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="P15" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="Q15" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="R15" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1643,17 +1699,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1663,253 +1719,19 @@
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O16" t="n">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="P16" t="n">
         <v>50</v>
       </c>
       <c r="Q16" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>8:15</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Atlanta Braves</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>St.Louis Cardinals</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>65.0</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>35.0</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>32.4</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>12.9</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="n">
-        <v>4</v>
-      </c>
-      <c r="O17" t="n">
-        <v>25</v>
-      </c>
-      <c r="P17" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>75</v>
-      </c>
-      <c r="R17" t="n">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>8:40</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Kansas City Royals</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>34.0</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>66.0</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>1-4</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>23.8</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>11.4</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>2.8</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="n">
-        <v>1</v>
-      </c>
-      <c r="O18" t="n">
         <v>0</v>
-      </c>
-      <c r="P18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>19:35</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Fubon Guardians</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Uni Lions</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>57.0</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>43.0</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>4-2</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>39.4</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>15.3</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>4.3</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="n">
-        <v>5</v>
-      </c>
-      <c r="O19" t="n">
-        <v>20</v>
-      </c>
-      <c r="P19" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>80</v>
-      </c>
-      <c r="R19" t="n">
-        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-02 11:39
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -511,83 +511,83 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="O2" t="n">
-        <v>56.2</v>
+        <v>20</v>
       </c>
       <c r="P2" t="n">
-        <v>37.5</v>
+        <v>70</v>
       </c>
       <c r="Q2" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -623,7 +623,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>35.2</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>14.6</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,19 +657,19 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="O3" t="n">
-        <v>58.3</v>
+        <v>55</v>
       </c>
       <c r="P3" t="n">
-        <v>33.3</v>
+        <v>35</v>
       </c>
       <c r="Q3" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="R3" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -680,12 +680,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,17 +695,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,17 +715,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -739,19 +739,19 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="O4" t="n">
-        <v>53.8</v>
+        <v>53.6</v>
       </c>
       <c r="P4" t="n">
-        <v>38.5</v>
+        <v>35.7</v>
       </c>
       <c r="Q4" t="n">
-        <v>23.1</v>
+        <v>14.3</v>
       </c>
       <c r="R4" t="n">
-        <v>23.1</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="5">
@@ -762,12 +762,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -777,17 +777,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>50.4</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>25.9</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,75 +821,75 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="O5" t="n">
-        <v>53.8</v>
+        <v>53.3</v>
       </c>
       <c r="P5" t="n">
-        <v>38.5</v>
+        <v>40</v>
       </c>
       <c r="Q5" t="n">
-        <v>23.1</v>
+        <v>13.3</v>
       </c>
       <c r="R5" t="n">
-        <v>23.1</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,59 +899,59 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="O6" t="n">
-        <v>53.3</v>
+        <v>37.5</v>
       </c>
       <c r="P6" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="Q6" t="n">
-        <v>20</v>
+        <v>6.2</v>
       </c>
       <c r="R6" t="n">
-        <v>20</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,17 +961,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -994,36 +994,36 @@
         <v>40</v>
       </c>
       <c r="Q7" t="n">
-        <v>20</v>
+        <v>13.3</v>
       </c>
       <c r="R7" t="n">
-        <v>20</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,17 +1043,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1067,30 +1067,30 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="O8" t="n">
-        <v>53.3</v>
+        <v>48</v>
       </c>
       <c r="P8" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="Q8" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="R8" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2:35</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1105,17 +1105,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1125,17 +1125,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1149,55 +1149,55 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="O9" t="n">
-        <v>53.8</v>
+        <v>45.8</v>
       </c>
       <c r="P9" t="n">
-        <v>38.5</v>
+        <v>45.8</v>
       </c>
       <c r="Q9" t="n">
-        <v>23.1</v>
+        <v>12.5</v>
       </c>
       <c r="R9" t="n">
-        <v>23.1</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2:35</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>6-5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,17 +1207,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>68.9</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>36.7</t>
+          <t>44.2</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1231,55 +1231,55 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="O10" t="n">
-        <v>53.8</v>
+        <v>45.8</v>
       </c>
       <c r="P10" t="n">
-        <v>38.5</v>
+        <v>45.8</v>
       </c>
       <c r="Q10" t="n">
-        <v>23.1</v>
+        <v>12.5</v>
       </c>
       <c r="R10" t="n">
-        <v>23.1</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1289,22 +1289,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1313,55 +1313,55 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="O11" t="n">
-        <v>52.9</v>
+        <v>44.4</v>
       </c>
       <c r="P11" t="n">
-        <v>41.2</v>
+        <v>44.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>23.5</v>
+        <v>14.8</v>
       </c>
       <c r="R11" t="n">
-        <v>23.5</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1371,22 +1371,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>16.5</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1395,75 +1395,75 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="O12" t="n">
-        <v>53.8</v>
+        <v>44.4</v>
       </c>
       <c r="P12" t="n">
-        <v>38.5</v>
+        <v>48.1</v>
       </c>
       <c r="Q12" t="n">
-        <v>30.8</v>
+        <v>14.8</v>
       </c>
       <c r="R12" t="n">
-        <v>30.8</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>49.1</t>
+          <t>65.6</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>24.8</t>
+          <t>40.4</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1473,11 +1473,11 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="O13" t="n">
         <v>44.4</v>
@@ -1486,31 +1486,31 @@
         <v>44.4</v>
       </c>
       <c r="Q13" t="n">
-        <v>22.2</v>
+        <v>5.6</v>
       </c>
       <c r="R13" t="n">
-        <v>22.2</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4:07</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1540,12 +1540,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1559,40 +1559,40 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="O14" t="n">
-        <v>54.5</v>
+        <v>47.4</v>
       </c>
       <c r="P14" t="n">
-        <v>36.4</v>
+        <v>42.1</v>
       </c>
       <c r="Q14" t="n">
-        <v>18.2</v>
+        <v>10.5</v>
       </c>
       <c r="R14" t="n">
-        <v>18.2</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1617,17 +1617,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>63.2</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>37.9</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1641,60 +1641,60 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="O15" t="n">
-        <v>50</v>
+        <v>44.4</v>
       </c>
       <c r="P15" t="n">
-        <v>40</v>
+        <v>44.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>10</v>
+        <v>5.6</v>
       </c>
       <c r="R15" t="n">
-        <v>10</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>76.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>24.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1704,12 +1704,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1719,13 +1719,13 @@
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O16" t="n">
-        <v>33.3</v>
+        <v>57.1</v>
       </c>
       <c r="P16" t="n">
-        <v>50</v>
+        <v>28.6</v>
       </c>
       <c r="Q16" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-03 11:46
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,119 +511,119 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>4-1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>13.3</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N2" t="n">
+        <v>20</v>
+      </c>
+      <c r="O2" t="n">
+        <v>60</v>
+      </c>
+      <c r="P2" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q2" t="n">
         <v>10</v>
       </c>
-      <c r="O2" t="n">
-        <v>20</v>
-      </c>
-      <c r="P2" t="n">
-        <v>70</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
       <c r="R2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>5:05</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>73.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>7-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,50 +657,50 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="O3" t="n">
-        <v>55</v>
+        <v>56.2</v>
       </c>
       <c r="P3" t="n">
-        <v>35</v>
+        <v>37.5</v>
       </c>
       <c r="Q3" t="n">
-        <v>15</v>
+        <v>6.2</v>
       </c>
       <c r="R3" t="n">
-        <v>15</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -720,17 +720,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -739,19 +739,19 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="O4" t="n">
-        <v>53.6</v>
+        <v>55.2</v>
       </c>
       <c r="P4" t="n">
-        <v>35.7</v>
+        <v>34.5</v>
       </c>
       <c r="Q4" t="n">
-        <v>14.3</v>
+        <v>10.3</v>
       </c>
       <c r="R4" t="n">
-        <v>14.3</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="5">
@@ -762,12 +762,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -777,37 +777,37 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>2-5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -817,79 +817,79 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="O5" t="n">
-        <v>53.3</v>
+        <v>40.7</v>
       </c>
       <c r="P5" t="n">
-        <v>40</v>
+        <v>48.1</v>
       </c>
       <c r="Q5" t="n">
-        <v>13.3</v>
+        <v>3.7</v>
       </c>
       <c r="R5" t="n">
-        <v>13.3</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,54 +899,54 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="O6" t="n">
-        <v>37.5</v>
+        <v>47.5</v>
       </c>
       <c r="P6" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="Q6" t="n">
-        <v>6.2</v>
+        <v>7.5</v>
       </c>
       <c r="R6" t="n">
-        <v>6.2</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -966,12 +966,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,60 +985,60 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="O7" t="n">
-        <v>53.3</v>
+        <v>45.2</v>
       </c>
       <c r="P7" t="n">
-        <v>40</v>
+        <v>45.2</v>
       </c>
       <c r="Q7" t="n">
-        <v>13.3</v>
+        <v>9.5</v>
       </c>
       <c r="R7" t="n">
-        <v>13.3</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1063,79 +1063,79 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O8" t="n">
-        <v>48</v>
+        <v>40.7</v>
       </c>
       <c r="P8" t="n">
-        <v>44</v>
+        <v>48.1</v>
       </c>
       <c r="Q8" t="n">
-        <v>12</v>
+        <v>3.7</v>
       </c>
       <c r="R8" t="n">
-        <v>12</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>3-6</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1145,64 +1145,64 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="O9" t="n">
-        <v>45.8</v>
+        <v>44.4</v>
       </c>
       <c r="P9" t="n">
-        <v>45.8</v>
+        <v>50</v>
       </c>
       <c r="Q9" t="n">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>12.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>6-5</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1212,12 +1212,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>68.9</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>44.2</t>
+          <t>51.6</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1227,141 +1227,141 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O10" t="n">
-        <v>45.8</v>
+        <v>43.5</v>
       </c>
       <c r="P10" t="n">
-        <v>45.8</v>
+        <v>52.2</v>
       </c>
       <c r="Q10" t="n">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>12.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="O11" t="n">
         <v>44.4</v>
       </c>
       <c r="P11" t="n">
-        <v>44.4</v>
+        <v>50</v>
       </c>
       <c r="Q11" t="n">
-        <v>14.8</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>14.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1371,22 +1371,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>16.5</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1395,137 +1395,137 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="O12" t="n">
-        <v>44.4</v>
+        <v>45.9</v>
       </c>
       <c r="P12" t="n">
-        <v>48.1</v>
+        <v>45.9</v>
       </c>
       <c r="Q12" t="n">
-        <v>14.8</v>
+        <v>8.1</v>
       </c>
       <c r="R12" t="n">
-        <v>14.8</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>65.6</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>40.4</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="O13" t="n">
-        <v>44.4</v>
+        <v>47.5</v>
       </c>
       <c r="P13" t="n">
-        <v>44.4</v>
+        <v>42.5</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.6</v>
+        <v>10</v>
       </c>
       <c r="R13" t="n">
-        <v>5.6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>9:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>6-7</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1535,22 +1535,22 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>97.4</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>33.8</t>
+          <t>87.5</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>70.3</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1559,101 +1559,101 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="O14" t="n">
-        <v>47.4</v>
+        <v>43.5</v>
       </c>
       <c r="P14" t="n">
-        <v>42.1</v>
+        <v>52.2</v>
       </c>
       <c r="Q14" t="n">
-        <v>10.5</v>
+        <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>10.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>9:15</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N15" t="n">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="O15" t="n">
-        <v>44.4</v>
+        <v>45.9</v>
       </c>
       <c r="P15" t="n">
-        <v>44.4</v>
+        <v>45.9</v>
       </c>
       <c r="Q15" t="n">
-        <v>5.6</v>
+        <v>8.1</v>
       </c>
       <c r="R15" t="n">
-        <v>5.6</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="16">
@@ -1664,12 +1664,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1679,17 +1679,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>76.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>24.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1704,34 +1704,694 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr"/>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="N16" t="n">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="O16" t="n">
-        <v>57.1</v>
+        <v>45.9</v>
       </c>
       <c r="P16" t="n">
-        <v>28.6</v>
+        <v>45.9</v>
       </c>
       <c r="Q16" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="R16" t="n">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Chinatrust Brothers</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>7-5</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>77.7</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>55.2</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>40</v>
+      </c>
+      <c r="O17" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="P17" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="R17" t="n">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>36.6</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>28</v>
+      </c>
+      <c r="O18" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="P18" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="R18" t="n">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>25.8</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>40</v>
+      </c>
+      <c r="O19" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="P19" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>10</v>
+      </c>
+      <c r="R19" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Orix Buffaloes</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Seibu Lions</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>25.8</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>38</v>
+      </c>
+      <c r="O20" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="P20" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="R20" t="n">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Rakuten Gold. Eagles</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Nippon Ham Fighters</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>9</v>
+      </c>
+      <c r="O21" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="P21" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="Q21" t="n">
         <v>0</v>
       </c>
-      <c r="R16" t="n">
+      <c r="R21" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Chunichi Dragons</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Yomiuri Giants</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>36</v>
+      </c>
+      <c r="O22" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="P22" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="R22" t="n">
+        <v>8.300000000000001</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>55.7</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>30.6</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>31</v>
+      </c>
+      <c r="O23" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="P23" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="R23" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>31</v>
+      </c>
+      <c r="O24" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="P24" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="R24" t="n">
+        <v>3.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-03 16:48
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1659,17 +1659,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>10:38</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1704,12 +1704,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1723,55 +1723,55 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="O16" t="n">
-        <v>45.9</v>
+        <v>53.3</v>
       </c>
       <c r="P16" t="n">
-        <v>45.9</v>
+        <v>36.7</v>
       </c>
       <c r="Q16" t="n">
-        <v>8.1</v>
+        <v>13.3</v>
       </c>
       <c r="R16" t="n">
-        <v>8.1</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1781,17 +1781,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>77.7</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>55.2</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1805,55 +1805,55 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="O17" t="n">
-        <v>47.5</v>
+        <v>45.9</v>
       </c>
       <c r="P17" t="n">
-        <v>45</v>
+        <v>45.9</v>
       </c>
       <c r="Q17" t="n">
-        <v>7.5</v>
+        <v>8.1</v>
       </c>
       <c r="R17" t="n">
-        <v>7.5</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>3-6</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1863,17 +1863,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>50.4</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>25.9</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1887,19 +1887,19 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="O18" t="n">
-        <v>42.9</v>
+        <v>44.4</v>
       </c>
       <c r="P18" t="n">
-        <v>46.4</v>
+        <v>50</v>
       </c>
       <c r="Q18" t="n">
-        <v>3.6</v>
+        <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>3.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1910,12 +1910,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1925,17 +1925,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1945,17 +1945,17 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>77.7</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>55.2</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1975,177 +1975,177 @@
         <v>47.5</v>
       </c>
       <c r="P19" t="n">
-        <v>42.5</v>
+        <v>45</v>
       </c>
       <c r="Q19" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="R19" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N20" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="O20" t="n">
-        <v>44.7</v>
+        <v>42.9</v>
       </c>
       <c r="P20" t="n">
-        <v>47.4</v>
+        <v>46.4</v>
       </c>
       <c r="Q20" t="n">
-        <v>7.9</v>
+        <v>3.6</v>
       </c>
       <c r="R20" t="n">
-        <v>7.9</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N21" t="n">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="O21" t="n">
-        <v>44.4</v>
+        <v>47.5</v>
       </c>
       <c r="P21" t="n">
-        <v>44.4</v>
+        <v>42.5</v>
       </c>
       <c r="Q21" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R21" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22">
@@ -2156,12 +2156,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2171,17 +2171,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2191,17 +2191,17 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2215,55 +2215,55 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="O22" t="n">
-        <v>44.4</v>
+        <v>44.7</v>
       </c>
       <c r="P22" t="n">
-        <v>47.2</v>
+        <v>47.4</v>
       </c>
       <c r="Q22" t="n">
-        <v>8.300000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="R22" t="n">
-        <v>8.300000000000001</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2273,17 +2273,17 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>55.7</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>30.6</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2297,101 +2297,421 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="O23" t="n">
-        <v>45.2</v>
+        <v>44.4</v>
       </c>
       <c r="P23" t="n">
-        <v>45.2</v>
+        <v>44.4</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="R23" t="n">
-        <v>3.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Chunichi Dragons</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Yomiuri Giants</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>36</v>
+      </c>
+      <c r="O24" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="P24" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="R24" t="n">
+        <v>8.300000000000001</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>55.7</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>30.6</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>31</v>
+      </c>
+      <c r="O25" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="P25" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="R25" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>10:45</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Arizona Diamondbacks</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>MLB</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>47.0</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>53.0</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>4-5</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>79.3</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>54.4</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>29.4</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>원정승</t>
         </is>
       </c>
-      <c r="N24" t="n">
+      <c r="N26" t="n">
         <v>31</v>
       </c>
-      <c r="O24" t="n">
+      <c r="O26" t="n">
         <v>45.2</v>
       </c>
-      <c r="P24" t="n">
+      <c r="P26" t="n">
         <v>45.2</v>
       </c>
-      <c r="Q24" t="n">
+      <c r="Q26" t="n">
         <v>3.2</v>
       </c>
-      <c r="R24" t="n">
+      <c r="R26" t="n">
         <v>3.2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>80.0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>20.8</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>6.7</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="n">
+        <v>4</v>
+      </c>
+      <c r="O27" t="n">
+        <v>50</v>
+      </c>
+      <c r="P27" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>78.0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>39.3</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="n">
+        <v>7</v>
+      </c>
+      <c r="O28" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="P28" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-04 13:23
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R28"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -531,12 +531,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -575,35 +575,35 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="O2" t="n">
-        <v>60</v>
+        <v>58.8</v>
       </c>
       <c r="P2" t="n">
-        <v>35</v>
+        <v>35.3</v>
       </c>
       <c r="Q2" t="n">
-        <v>10</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="R2" t="n">
-        <v>10</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>5:05</t>
+          <t>9:08</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -613,17 +613,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>73.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>7-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>55.7</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>30.6</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,50 +657,50 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="O3" t="n">
-        <v>56.2</v>
+        <v>55.2</v>
       </c>
       <c r="P3" t="n">
-        <v>37.5</v>
+        <v>37.9</v>
       </c>
       <c r="Q3" t="n">
-        <v>6.2</v>
+        <v>10.3</v>
       </c>
       <c r="R3" t="n">
-        <v>6.2</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -720,17 +720,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -739,19 +739,19 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="O4" t="n">
-        <v>55.2</v>
+        <v>46.2</v>
       </c>
       <c r="P4" t="n">
-        <v>34.5</v>
+        <v>44.2</v>
       </c>
       <c r="Q4" t="n">
-        <v>10.3</v>
+        <v>7.7</v>
       </c>
       <c r="R4" t="n">
-        <v>10.3</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="5">
@@ -762,12 +762,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -777,37 +777,37 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2-5</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -817,23 +817,23 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="O5" t="n">
-        <v>40.7</v>
+        <v>46.2</v>
       </c>
       <c r="P5" t="n">
-        <v>48.1</v>
+        <v>44.2</v>
       </c>
       <c r="Q5" t="n">
-        <v>3.7</v>
+        <v>7.7</v>
       </c>
       <c r="R5" t="n">
-        <v>3.7</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="6">
@@ -844,12 +844,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,37 +859,37 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,23 +899,23 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="O6" t="n">
-        <v>47.5</v>
+        <v>43.5</v>
       </c>
       <c r="P6" t="n">
-        <v>45</v>
+        <v>45.7</v>
       </c>
       <c r="Q6" t="n">
-        <v>7.5</v>
+        <v>4.3</v>
       </c>
       <c r="R6" t="n">
-        <v>7.5</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="7">
@@ -926,12 +926,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -941,37 +941,37 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -981,59 +981,59 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="O7" t="n">
-        <v>45.2</v>
+        <v>44.4</v>
       </c>
       <c r="P7" t="n">
-        <v>45.2</v>
+        <v>48.1</v>
       </c>
       <c r="Q7" t="n">
-        <v>9.5</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>9.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>2-6</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>16.5</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1067,35 +1067,35 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="O8" t="n">
-        <v>40.7</v>
+        <v>38.1</v>
       </c>
       <c r="P8" t="n">
-        <v>48.1</v>
+        <v>52.4</v>
       </c>
       <c r="Q8" t="n">
-        <v>3.7</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>3.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1105,17 +1105,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3-6</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1130,12 +1130,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1149,10 +1149,10 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="O9" t="n">
-        <v>44.4</v>
+        <v>42.3</v>
       </c>
       <c r="P9" t="n">
         <v>50</v>
@@ -1167,7 +1167,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1187,17 +1187,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,17 +1207,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>65.6</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>51.6</t>
+          <t>40.4</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1231,13 +1231,13 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="O10" t="n">
-        <v>43.5</v>
+        <v>40</v>
       </c>
       <c r="P10" t="n">
-        <v>52.2</v>
+        <v>53.3</v>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
@@ -1249,17 +1249,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1289,17 +1289,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1313,65 +1313,65 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="O11" t="n">
-        <v>44.4</v>
+        <v>40.5</v>
       </c>
       <c r="P11" t="n">
-        <v>50</v>
+        <v>47.6</v>
       </c>
       <c r="Q11" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="R11" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1391,39 +1391,39 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="O12" t="n">
-        <v>45.9</v>
+        <v>39</v>
       </c>
       <c r="P12" t="n">
-        <v>45.9</v>
+        <v>51.2</v>
       </c>
       <c r="Q12" t="n">
-        <v>8.1</v>
+        <v>2.4</v>
       </c>
       <c r="R12" t="n">
-        <v>8.1</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>5:05</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1433,12 +1433,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1458,12 +1458,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,35 +1477,35 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="O13" t="n">
-        <v>47.5</v>
+        <v>46.2</v>
       </c>
       <c r="P13" t="n">
-        <v>42.5</v>
+        <v>44.2</v>
       </c>
       <c r="Q13" t="n">
-        <v>10</v>
+        <v>5.8</v>
       </c>
       <c r="R13" t="n">
-        <v>10</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>9:08</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1515,17 +1515,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>6-7</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1535,17 +1535,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>97.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>87.5</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>70.3</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1559,35 +1559,35 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="O14" t="n">
-        <v>43.5</v>
+        <v>42.6</v>
       </c>
       <c r="P14" t="n">
-        <v>52.2</v>
+        <v>46.8</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="R14" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>9:15</t>
+          <t>9:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1597,37 +1597,37 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>51.0</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>49.0</t>
-        </is>
-      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>46.3</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>22.6</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1637,64 +1637,64 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N15" t="n">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="O15" t="n">
-        <v>45.9</v>
+        <v>42.6</v>
       </c>
       <c r="P15" t="n">
-        <v>45.9</v>
+        <v>46.8</v>
       </c>
       <c r="Q15" t="n">
-        <v>8.1</v>
+        <v>4.3</v>
       </c>
       <c r="R15" t="n">
-        <v>8.1</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10:38</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1704,12 +1704,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1719,64 +1719,64 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N16" t="n">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>53.3</v>
+        <v>39</v>
       </c>
       <c r="P16" t="n">
-        <v>36.7</v>
+        <v>51.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>13.3</v>
+        <v>2.4</v>
       </c>
       <c r="R16" t="n">
-        <v>13.3</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1786,12 +1786,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>16.5</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1801,59 +1801,59 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="O17" t="n">
-        <v>45.9</v>
+        <v>43.2</v>
       </c>
       <c r="P17" t="n">
-        <v>45.9</v>
+        <v>45.5</v>
       </c>
       <c r="Q17" t="n">
-        <v>8.1</v>
+        <v>2.3</v>
       </c>
       <c r="R17" t="n">
-        <v>8.1</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>3-6</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1863,17 +1863,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1887,55 +1887,55 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="O18" t="n">
-        <v>44.4</v>
+        <v>37.5</v>
       </c>
       <c r="P18" t="n">
         <v>50</v>
       </c>
       <c r="Q18" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="R18" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1945,22 +1945,22 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>77.7</t>
+          <t>23.3</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>55.2</t>
+          <t>7.9</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1969,749 +1969,101 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="O19" t="n">
-        <v>47.5</v>
+        <v>44</v>
       </c>
       <c r="P19" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Q19" t="n">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="R19" t="n">
-        <v>7.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>50.4</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>25.9</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N20" t="n">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="O20" t="n">
-        <v>42.9</v>
+        <v>44.4</v>
       </c>
       <c r="P20" t="n">
-        <v>46.4</v>
+        <v>46.3</v>
       </c>
       <c r="Q20" t="n">
-        <v>3.6</v>
+        <v>7.4</v>
       </c>
       <c r="R20" t="n">
-        <v>3.6</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>19:35</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Wei Chuan Dragons</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Fubon Guardians</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>58.0</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>42.0</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>25.8</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>9.2</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N21" t="n">
-        <v>40</v>
-      </c>
-      <c r="O21" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="P21" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>10</v>
-      </c>
-      <c r="R21" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Orix Buffaloes</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Seibu Lions</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>NPB</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>25.8</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>9.2</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N22" t="n">
-        <v>38</v>
-      </c>
-      <c r="O22" t="n">
-        <v>44.7</v>
-      </c>
-      <c r="P22" t="n">
-        <v>47.4</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="R22" t="n">
-        <v>7.9</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Rakuten Gold. Eagles</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Nippon Ham Fighters</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>NPB</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>34.0</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>66.0</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>2-3</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>23.8</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>3.6</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>0.6</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N23" t="n">
-        <v>9</v>
-      </c>
-      <c r="O23" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="P23" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Chunichi Dragons</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Yomiuri Giants</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>NPB</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>52.0</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>48.0</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>3-2</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>23.8</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>7.5</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>1.6</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N24" t="n">
-        <v>36</v>
-      </c>
-      <c r="O24" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="P24" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="R24" t="n">
-        <v>8.300000000000001</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>7:45</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Washington Nationals</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Pittsburgh Pirates</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>4-5</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>55.7</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>30.6</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N25" t="n">
-        <v>31</v>
-      </c>
-      <c r="O25" t="n">
-        <v>45.2</v>
-      </c>
-      <c r="P25" t="n">
-        <v>45.2</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="R25" t="n">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>10:45</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Arizona Diamondbacks</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Milwaukee Brewers</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>4-5</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>54.4</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>29.4</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N26" t="n">
-        <v>31</v>
-      </c>
-      <c r="O26" t="n">
-        <v>45.2</v>
-      </c>
-      <c r="P26" t="n">
-        <v>45.2</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="R26" t="n">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>8:10</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Cleveland Guardians</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Chicago White Sox</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>80.0</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>4-2</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>39.4</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>20.8</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>6.7</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="n">
-        <v>4</v>
-      </c>
-      <c r="O27" t="n">
-        <v>50</v>
-      </c>
-      <c r="P27" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>11:10</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Los Angeles Dodgers</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>San Diego Padres</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>78.0</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>22.0</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>5-3</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>39.3</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>17.4</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>❓</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="n">
-        <v>7</v>
-      </c>
-      <c r="O28" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="P28" t="n">
-        <v>42.9</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" t="n">
-        <v>0</v>
+        <v>7.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-05 11:55
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -511,139 +511,139 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>2:05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4-1</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>13.3</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="O2" t="n">
-        <v>58.8</v>
+        <v>25</v>
       </c>
       <c r="P2" t="n">
-        <v>35.3</v>
+        <v>68.8</v>
       </c>
       <c r="Q2" t="n">
-        <v>8.800000000000001</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>8.800000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>9:08</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>73.1</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>49.2</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -653,141 +653,141 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="O3" t="n">
-        <v>55.2</v>
+        <v>35.5</v>
       </c>
       <c r="P3" t="n">
-        <v>37.9</v>
+        <v>58.1</v>
       </c>
       <c r="Q3" t="n">
-        <v>10.3</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>10.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="O4" t="n">
-        <v>46.2</v>
+        <v>36.4</v>
       </c>
       <c r="P4" t="n">
-        <v>44.2</v>
+        <v>59.1</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.7</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>7.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>3:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-1</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,22 +797,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -821,35 +821,35 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="O5" t="n">
-        <v>46.2</v>
+        <v>58.1</v>
       </c>
       <c r="P5" t="n">
-        <v>44.2</v>
+        <v>38.7</v>
       </c>
       <c r="Q5" t="n">
-        <v>7.7</v>
+        <v>6.5</v>
       </c>
       <c r="R5" t="n">
-        <v>7.7</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -884,12 +884,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -903,25 +903,25 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="O6" t="n">
-        <v>43.5</v>
+        <v>44.4</v>
       </c>
       <c r="P6" t="n">
-        <v>45.7</v>
+        <v>47.6</v>
       </c>
       <c r="Q6" t="n">
-        <v>4.3</v>
+        <v>3.2</v>
       </c>
       <c r="R6" t="n">
-        <v>4.3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -941,12 +941,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -985,13 +985,13 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="O7" t="n">
-        <v>44.4</v>
+        <v>41.7</v>
       </c>
       <c r="P7" t="n">
-        <v>48.1</v>
+        <v>54.2</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
@@ -1023,12 +1023,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1067,13 +1067,13 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="O8" t="n">
-        <v>38.1</v>
+        <v>41</v>
       </c>
       <c r="P8" t="n">
-        <v>52.4</v>
+        <v>53.8</v>
       </c>
       <c r="Q8" t="n">
         <v>0</v>
@@ -1085,17 +1085,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1105,17 +1105,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1125,17 +1125,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1149,19 +1149,19 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="O9" t="n">
-        <v>42.3</v>
+        <v>40.4</v>
       </c>
       <c r="P9" t="n">
-        <v>50</v>
+        <v>52.6</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="10">
@@ -1172,12 +1172,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1187,17 +1187,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,17 +1207,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>65.6</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>40.4</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1231,13 +1231,13 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="O10" t="n">
-        <v>40</v>
+        <v>43.4</v>
       </c>
       <c r="P10" t="n">
-        <v>53.3</v>
+        <v>49.1</v>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
@@ -1254,12 +1254,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1269,37 +1269,37 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1309,79 +1309,79 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="O11" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="P11" t="n">
         <v>40.5</v>
       </c>
-      <c r="P11" t="n">
-        <v>47.6</v>
-      </c>
       <c r="Q11" t="n">
-        <v>2.4</v>
+        <v>8.1</v>
       </c>
       <c r="R11" t="n">
-        <v>2.4</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>2:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>65.6</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>40.4</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1391,39 +1391,39 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="O12" t="n">
-        <v>39</v>
+        <v>48.3</v>
       </c>
       <c r="P12" t="n">
-        <v>51.2</v>
+        <v>43.1</v>
       </c>
       <c r="Q12" t="n">
-        <v>2.4</v>
+        <v>6.9</v>
       </c>
       <c r="R12" t="n">
-        <v>2.4</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>5:05</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1433,17 +1433,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1453,17 +1453,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,35 +1477,35 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="O13" t="n">
         <v>46.2</v>
       </c>
       <c r="P13" t="n">
-        <v>44.2</v>
+        <v>46.2</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.8</v>
+        <v>4.6</v>
       </c>
       <c r="R13" t="n">
-        <v>5.8</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>9:08</t>
+          <t>4:30</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1515,37 +1515,37 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>35.2</t>
+          <t>39.3</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>14.6</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1555,79 +1555,79 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="O14" t="n">
-        <v>42.6</v>
+        <v>46.2</v>
       </c>
       <c r="P14" t="n">
-        <v>46.8</v>
+        <v>46.2</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="R14" t="n">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>46.3</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>22.6</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1637,23 +1637,23 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N15" t="n">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="O15" t="n">
-        <v>42.6</v>
+        <v>47.4</v>
       </c>
       <c r="P15" t="n">
-        <v>46.8</v>
+        <v>43.9</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.3</v>
+        <v>7</v>
       </c>
       <c r="R15" t="n">
-        <v>4.3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
@@ -1679,17 +1679,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1699,17 +1699,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>35.2</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>14.6</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1723,19 +1723,19 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="O16" t="n">
-        <v>39</v>
+        <v>43.3</v>
       </c>
       <c r="P16" t="n">
-        <v>51.2</v>
+        <v>48.3</v>
       </c>
       <c r="Q16" t="n">
-        <v>2.4</v>
+        <v>1.7</v>
       </c>
       <c r="R16" t="n">
-        <v>2.4</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="17">
@@ -1746,12 +1746,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1761,17 +1761,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1805,132 +1805,132 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="O17" t="n">
-        <v>43.2</v>
+        <v>40.4</v>
       </c>
       <c r="P17" t="n">
-        <v>45.5</v>
+        <v>52.6</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.3</v>
+        <v>1.8</v>
       </c>
       <c r="R17" t="n">
-        <v>2.3</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
           <t>55.0</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>3-4</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N18" t="n">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="O18" t="n">
-        <v>37.5</v>
+        <v>44.4</v>
       </c>
       <c r="P18" t="n">
-        <v>50</v>
+        <v>47.6</v>
       </c>
       <c r="Q18" t="n">
-        <v>2.5</v>
+        <v>4.8</v>
       </c>
       <c r="R18" t="n">
-        <v>2.5</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>4:30</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1950,12 +1950,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>23.3</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>7.9</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1969,35 +1969,35 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="O19" t="n">
-        <v>44</v>
+        <v>44.4</v>
       </c>
       <c r="P19" t="n">
-        <v>46</v>
+        <v>47.6</v>
       </c>
       <c r="Q19" t="n">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="R19" t="n">
-        <v>6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>6:00</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2007,17 +2007,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2027,17 +2027,17 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2051,19 +2051,19 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="O20" t="n">
-        <v>44.4</v>
+        <v>45.5</v>
       </c>
       <c r="P20" t="n">
-        <v>46.3</v>
+        <v>47</v>
       </c>
       <c r="Q20" t="n">
-        <v>7.4</v>
+        <v>4.5</v>
       </c>
       <c r="R20" t="n">
-        <v>7.4</v>
+        <v>4.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-07 14:40
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,57 +511,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>23.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,17 +571,17 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="O2" t="n">
-        <v>68.8</v>
+        <v>28.6</v>
       </c>
       <c r="P2" t="n">
-        <v>31.2</v>
+        <v>66.7</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
@@ -593,37 +593,37 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,22 +633,22 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>23.3</t>
+          <t>39.3</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>7.9</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -657,50 +657,50 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="O3" t="n">
-        <v>36.6</v>
+        <v>30.4</v>
       </c>
       <c r="P3" t="n">
-        <v>56.3</v>
+        <v>65.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -720,12 +720,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>16.5</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -739,13 +739,13 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="O4" t="n">
-        <v>38.3</v>
+        <v>36.2</v>
       </c>
       <c r="P4" t="n">
-        <v>58.3</v>
+        <v>60.3</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
@@ -757,37 +757,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,22 +797,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>0.9</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -821,55 +821,55 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>74</v>
+        <v>29</v>
       </c>
       <c r="O5" t="n">
-        <v>39.2</v>
+        <v>37.9</v>
       </c>
       <c r="P5" t="n">
-        <v>54.1</v>
+        <v>58.6</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>8:45</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>1-4</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -879,22 +879,22 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>16.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -903,119 +903,119 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>78</v>
+        <v>33</v>
       </c>
       <c r="O6" t="n">
-        <v>41</v>
+        <v>33.3</v>
       </c>
       <c r="P6" t="n">
-        <v>52.6</v>
+        <v>63.6</v>
       </c>
       <c r="Q6" t="n">
-        <v>2.6</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>2.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="O7" t="n">
-        <v>46.5</v>
+        <v>35.8</v>
       </c>
       <c r="P7" t="n">
-        <v>46.5</v>
+        <v>60.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.6</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>5.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Atlanta Braves</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>New York Mets</t>
-        </is>
-      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>MLB</t>
@@ -1023,145 +1023,1703 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>3-6</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>80.2</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>58.7</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="O8" t="n">
-        <v>41.9</v>
+        <v>36</v>
       </c>
       <c r="P8" t="n">
-        <v>51.4</v>
+        <v>60</v>
       </c>
       <c r="Q8" t="n">
-        <v>4.1</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>4.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>53.1</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>28.2</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>69</v>
+      </c>
+      <c r="O9" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="P9" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>12.3</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>63</v>
+      </c>
+      <c r="O10" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="P10" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>39.0</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>61.0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>60.8</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>35.5</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>54</v>
+      </c>
+      <c r="O11" t="n">
+        <v>37</v>
+      </c>
+      <c r="P11" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>9:05</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>28.0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>32.4</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>12.9</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>28</v>
+      </c>
+      <c r="O12" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="P12" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="R12" t="n">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>10:40</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>San Diego Padres</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Arizona Diamondbacks</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>MLB</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>28.4</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>10.6</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>63</v>
+      </c>
+      <c r="O13" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="P13" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Yokohama BayStars</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Chunichi Dragons</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>68</v>
+      </c>
+      <c r="O14" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="P14" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R14" t="n">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Seibu Lions</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Rakuten Gold. Eagles</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>64.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>16.3</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>54</v>
+      </c>
+      <c r="O15" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="P15" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="R15" t="n">
+        <v>7.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>KT Wiz Suwon</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Kiwoom Heroes</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>44.9</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>21.5</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>71</v>
+      </c>
+      <c r="O16" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="P16" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="R16" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SSG Landers</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>82</v>
+      </c>
+      <c r="O17" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="P17" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="R17" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>3:15</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>83</v>
+      </c>
+      <c r="O18" t="n">
+        <v>41</v>
+      </c>
+      <c r="P18" t="n">
+        <v>53</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="R18" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>37.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>33.8</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>13.8</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>62</v>
+      </c>
+      <c r="O19" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P19" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="R19" t="n">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>31.1</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>82</v>
+      </c>
+      <c r="O20" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="P20" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="R20" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
         <is>
           <t>53.0</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>79</v>
+      </c>
+      <c r="O21" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="P21" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>68</v>
+      </c>
+      <c r="O22" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="P22" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R22" t="n">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>82</v>
+      </c>
+      <c r="O23" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="P23" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="R23" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>KIA Tigers</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>44.9</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>21.5</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>82</v>
+      </c>
+      <c r="O24" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="P24" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="R24" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Hanwha Eagles</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>NC Dinos</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-4</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>92.1</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>51.6</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>82</v>
+      </c>
+      <c r="O25" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="P25" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="R25" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>7:35</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>39.4</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>83</v>
+      </c>
+      <c r="O26" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="P26" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="R26" t="n">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
         <is>
           <t>6-4</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>87.0</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>39.3</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>17.4</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>40.7</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="N9" t="n">
-        <v>74</v>
-      </c>
-      <c r="O9" t="n">
-        <v>41.9</v>
-      </c>
-      <c r="P9" t="n">
-        <v>51.4</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="R9" t="n">
-        <v>4.1</v>
+      <c r="N27" t="n">
+        <v>72</v>
+      </c>
+      <c r="O27" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="P27" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="R27" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>40.7</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>83</v>
+      </c>
+      <c r="O28" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="P28" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="R28" t="n">
+        <v>3.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-08 14:18
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R28"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,57 +511,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>23.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,17 +571,17 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="O2" t="n">
-        <v>28.6</v>
+        <v>66.7</v>
       </c>
       <c r="P2" t="n">
-        <v>66.7</v>
+        <v>33.3</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
@@ -593,37 +593,37 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,22 +633,22 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -657,13 +657,13 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="O3" t="n">
-        <v>30.4</v>
+        <v>42.5</v>
       </c>
       <c r="P3" t="n">
-        <v>65.2</v>
+        <v>55</v>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
@@ -675,17 +675,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,37 +695,37 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>16.5</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,79 +735,79 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="O4" t="n">
-        <v>36.2</v>
+        <v>56.9</v>
       </c>
       <c r="P4" t="n">
-        <v>60.3</v>
+        <v>37.3</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>0.9</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -817,59 +817,59 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="O5" t="n">
-        <v>37.9</v>
+        <v>56.9</v>
       </c>
       <c r="P5" t="n">
-        <v>58.6</v>
+        <v>37.3</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>1-4</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -879,17 +879,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -903,55 +903,55 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>33</v>
+        <v>87</v>
       </c>
       <c r="O6" t="n">
-        <v>33.3</v>
+        <v>36.8</v>
       </c>
       <c r="P6" t="n">
-        <v>63.6</v>
+        <v>57.5</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="R6" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,17 +961,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,50 +985,50 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>53</v>
+        <v>87</v>
       </c>
       <c r="O7" t="n">
-        <v>35.8</v>
+        <v>36.8</v>
       </c>
       <c r="P7" t="n">
-        <v>60.4</v>
+        <v>57.5</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>73.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>49.1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>24.8</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1067,13 +1067,13 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="O8" t="n">
-        <v>36</v>
+        <v>38.9</v>
       </c>
       <c r="P8" t="n">
-        <v>60</v>
+        <v>61.1</v>
       </c>
       <c r="Q8" t="n">
         <v>0</v>
@@ -1085,57 +1085,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1145,59 +1145,59 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="O9" t="n">
-        <v>39.1</v>
+        <v>59.1</v>
       </c>
       <c r="P9" t="n">
-        <v>55.1</v>
+        <v>36.4</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>2-5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,22 +1207,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1231,13 +1231,13 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="O10" t="n">
-        <v>36.5</v>
+        <v>43.5</v>
       </c>
       <c r="P10" t="n">
-        <v>60.3</v>
+        <v>52.2</v>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
@@ -1249,37 +1249,37 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>1-4</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1289,22 +1289,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>60.8</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>35.5</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1313,13 +1313,13 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="O11" t="n">
-        <v>37</v>
+        <v>45.2</v>
       </c>
       <c r="P11" t="n">
-        <v>59.3</v>
+        <v>51.6</v>
       </c>
       <c r="Q11" t="n">
         <v>0</v>
@@ -1331,206 +1331,206 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>28</v>
+        <v>95</v>
       </c>
       <c r="O12" t="n">
-        <v>57.1</v>
+        <v>41.1</v>
       </c>
       <c r="P12" t="n">
-        <v>39.3</v>
+        <v>53.7</v>
       </c>
       <c r="Q12" t="n">
-        <v>3.6</v>
+        <v>2.1</v>
       </c>
       <c r="R12" t="n">
-        <v>3.6</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-1</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="O13" t="n">
-        <v>36.5</v>
+        <v>50</v>
       </c>
       <c r="P13" t="n">
-        <v>60.3</v>
+        <v>42.6</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>7:35</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1540,12 +1540,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1555,79 +1555,79 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="O14" t="n">
-        <v>47.1</v>
+        <v>41.7</v>
       </c>
       <c r="P14" t="n">
-        <v>45.6</v>
+        <v>53.1</v>
       </c>
       <c r="Q14" t="n">
-        <v>5.9</v>
+        <v>2.1</v>
       </c>
       <c r="R14" t="n">
-        <v>5.9</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1637,59 +1637,59 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N15" t="n">
-        <v>54</v>
+        <v>92</v>
       </c>
       <c r="O15" t="n">
-        <v>48.1</v>
+        <v>40.2</v>
       </c>
       <c r="P15" t="n">
-        <v>46.3</v>
+        <v>54.3</v>
       </c>
       <c r="Q15" t="n">
-        <v>7.4</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
-        <v>7.4</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1699,17 +1699,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1723,75 +1723,75 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="O16" t="n">
-        <v>47.9</v>
+        <v>47.5</v>
       </c>
       <c r="P16" t="n">
-        <v>45.1</v>
+        <v>46.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>5.6</v>
+        <v>5</v>
       </c>
       <c r="R16" t="n">
-        <v>5.6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1801,39 +1801,39 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="O17" t="n">
-        <v>40.2</v>
+        <v>47.5</v>
       </c>
       <c r="P17" t="n">
-        <v>53.7</v>
+        <v>46.2</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.4</v>
+        <v>5</v>
       </c>
       <c r="R17" t="n">
-        <v>2.4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3:15</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1863,17 +1863,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>60.8</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>35.5</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1887,35 +1887,35 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="O18" t="n">
-        <v>41</v>
+        <v>41.7</v>
       </c>
       <c r="P18" t="n">
-        <v>53</v>
+        <v>53.1</v>
       </c>
       <c r="Q18" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="R18" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>8:45</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1925,22 +1925,22 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1950,12 +1950,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>33.8</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1965,39 +1965,39 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N19" t="n">
-        <v>62</v>
+        <v>95</v>
       </c>
       <c r="O19" t="n">
-        <v>48.4</v>
+        <v>41.1</v>
       </c>
       <c r="P19" t="n">
-        <v>43.5</v>
+        <v>53.7</v>
       </c>
       <c r="Q19" t="n">
-        <v>6.5</v>
+        <v>2.1</v>
       </c>
       <c r="R19" t="n">
-        <v>6.5</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2007,22 +2007,22 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2032,12 +2032,12 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2047,59 +2047,59 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N20" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="O20" t="n">
-        <v>40.2</v>
+        <v>48.7</v>
       </c>
       <c r="P20" t="n">
-        <v>53.7</v>
+        <v>44.7</v>
       </c>
       <c r="Q20" t="n">
-        <v>2.4</v>
+        <v>5.3</v>
       </c>
       <c r="R20" t="n">
-        <v>2.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2109,17 +2109,17 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2133,55 +2133,55 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="O21" t="n">
-        <v>39.2</v>
+        <v>40.2</v>
       </c>
       <c r="P21" t="n">
-        <v>54.4</v>
+        <v>54.9</v>
       </c>
       <c r="Q21" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="R21" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>4-1</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2191,22 +2191,22 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2215,101 +2215,101 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>68</v>
+        <v>95</v>
       </c>
       <c r="O22" t="n">
-        <v>47.1</v>
+        <v>42.1</v>
       </c>
       <c r="P22" t="n">
-        <v>45.6</v>
+        <v>52.6</v>
       </c>
       <c r="Q22" t="n">
-        <v>5.9</v>
+        <v>3.2</v>
       </c>
       <c r="R22" t="n">
-        <v>5.9</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>48.0</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>52.0</t>
-        </is>
-      </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>82.4</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>62.1</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N23" t="n">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="O23" t="n">
-        <v>40.2</v>
+        <v>42.1</v>
       </c>
       <c r="P23" t="n">
-        <v>53.7</v>
+        <v>52.6</v>
       </c>
       <c r="Q23" t="n">
-        <v>2.4</v>
+        <v>3.2</v>
       </c>
       <c r="R23" t="n">
-        <v>2.4</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="24">
@@ -2335,12 +2335,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2379,55 +2379,55 @@
         </is>
       </c>
       <c r="N24" t="n">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="O24" t="n">
-        <v>41.5</v>
+        <v>41.3</v>
       </c>
       <c r="P24" t="n">
-        <v>52.4</v>
+        <v>53.3</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.7</v>
+        <v>3.3</v>
       </c>
       <c r="R24" t="n">
-        <v>3.7</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>4:45</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>7-4</t>
+          <t>4-1</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2437,17 +2437,17 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>51.6</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2461,35 +2461,35 @@
         </is>
       </c>
       <c r="N25" t="n">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="O25" t="n">
-        <v>41.5</v>
+        <v>44</v>
       </c>
       <c r="P25" t="n">
-        <v>52.4</v>
+        <v>50.5</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.7</v>
+        <v>4.4</v>
       </c>
       <c r="R25" t="n">
-        <v>3.7</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>7:35</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2499,17 +2499,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2519,17 +2519,17 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2543,35 +2543,35 @@
         </is>
       </c>
       <c r="N26" t="n">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="O26" t="n">
-        <v>42.2</v>
+        <v>41.5</v>
       </c>
       <c r="P26" t="n">
-        <v>51.8</v>
+        <v>53.2</v>
       </c>
       <c r="Q26" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
       <c r="R26" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2581,17 +2581,17 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2601,17 +2601,17 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2625,35 +2625,35 @@
         </is>
       </c>
       <c r="N27" t="n">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="O27" t="n">
-        <v>44.4</v>
+        <v>43.3</v>
       </c>
       <c r="P27" t="n">
-        <v>48.6</v>
+        <v>51.5</v>
       </c>
       <c r="Q27" t="n">
-        <v>5.6</v>
+        <v>3.1</v>
       </c>
       <c r="R27" t="n">
-        <v>5.6</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2663,17 +2663,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2683,17 +2683,17 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2707,19 +2707,101 @@
         </is>
       </c>
       <c r="N28" t="n">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="O28" t="n">
-        <v>42.2</v>
+        <v>43.3</v>
       </c>
       <c r="P28" t="n">
-        <v>51.8</v>
+        <v>51.5</v>
       </c>
       <c r="Q28" t="n">
-        <v>3.6</v>
+        <v>3.1</v>
       </c>
       <c r="R28" t="n">
-        <v>3.6</v>
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>94</v>
+      </c>
+      <c r="O29" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="P29" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="R29" t="n">
+        <v>4.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-10 12:35
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -511,37 +511,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -575,77 +575,77 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="O2" t="n">
-        <v>38.8</v>
+        <v>39.1</v>
       </c>
       <c r="P2" t="n">
-        <v>57.5</v>
+        <v>56.5</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="R2" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t>51.8</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>27.1</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>9.9</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>★★</t>
@@ -653,141 +653,141 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>52</v>
+        <v>115</v>
       </c>
       <c r="O3" t="n">
-        <v>59.6</v>
+        <v>39.1</v>
       </c>
       <c r="P3" t="n">
-        <v>34.6</v>
+        <v>56.5</v>
       </c>
       <c r="Q3" t="n">
-        <v>5.8</v>
+        <v>0.9</v>
       </c>
       <c r="R3" t="n">
-        <v>5.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>40.0</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>60.0</t>
-        </is>
-      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>46.3</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>22.6</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="O4" t="n">
-        <v>37.2</v>
+        <v>50</v>
       </c>
       <c r="P4" t="n">
-        <v>59</v>
+        <v>44.1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>3.9</v>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,22 +797,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -821,112 +821,112 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>46</v>
+        <v>97</v>
       </c>
       <c r="O5" t="n">
-        <v>60.9</v>
+        <v>49.5</v>
       </c>
       <c r="P5" t="n">
-        <v>34.8</v>
+        <v>44.3</v>
       </c>
       <c r="Q5" t="n">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="R5" t="n">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>110</v>
+        <v>76</v>
       </c>
       <c r="O6" t="n">
-        <v>40</v>
+        <v>51.3</v>
       </c>
       <c r="P6" t="n">
-        <v>55.5</v>
+        <v>43.4</v>
       </c>
       <c r="Q6" t="n">
-        <v>1.8</v>
+        <v>5.3</v>
       </c>
       <c r="R6" t="n">
-        <v>1.8</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -941,99 +941,99 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="O7" t="n">
-        <v>37.1</v>
+        <v>47.5</v>
       </c>
       <c r="P7" t="n">
-        <v>58.1</v>
+        <v>47.5</v>
       </c>
       <c r="Q7" t="n">
-        <v>1</v>
+        <v>3.4</v>
       </c>
       <c r="R7" t="n">
-        <v>1</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>8:45</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>3-6</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1067,19 +1067,19 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="O8" t="n">
-        <v>35.3</v>
+        <v>42.6</v>
       </c>
       <c r="P8" t="n">
-        <v>59.8</v>
+        <v>53.7</v>
       </c>
       <c r="Q8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1105,63 +1105,63 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>55</v>
+        <v>108</v>
       </c>
       <c r="O9" t="n">
-        <v>60</v>
+        <v>42.6</v>
       </c>
       <c r="P9" t="n">
-        <v>34.5</v>
+        <v>53.7</v>
       </c>
       <c r="Q9" t="n">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>5.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1172,12 +1172,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1187,22 +1187,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1222,64 +1222,64 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>26</v>
+        <v>123</v>
       </c>
       <c r="O10" t="n">
-        <v>38.5</v>
+        <v>43.9</v>
       </c>
       <c r="P10" t="n">
-        <v>53.8</v>
+        <v>52</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="R10" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1289,17 +1289,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1313,55 +1313,55 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>97</v>
+        <v>125</v>
       </c>
       <c r="O11" t="n">
-        <v>44.3</v>
+        <v>45.6</v>
       </c>
       <c r="P11" t="n">
-        <v>49.5</v>
+        <v>50.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.1</v>
+        <v>2.4</v>
       </c>
       <c r="R11" t="n">
-        <v>4.1</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1371,17 +1371,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>82.4</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>62.1</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1395,35 +1395,35 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="O12" t="n">
-        <v>40</v>
+        <v>44.4</v>
       </c>
       <c r="P12" t="n">
-        <v>55.5</v>
+        <v>51.6</v>
       </c>
       <c r="Q12" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
       <c r="R12" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2:10</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1433,17 +1433,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>7-6</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1453,17 +1453,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>97.4</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>79.4</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>57.5</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,55 +1477,55 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>97</v>
+        <v>123</v>
       </c>
       <c r="O13" t="n">
-        <v>44.3</v>
+        <v>43.9</v>
       </c>
       <c r="P13" t="n">
-        <v>49.5</v>
+        <v>52</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.1</v>
+        <v>2.4</v>
       </c>
       <c r="R13" t="n">
-        <v>4.1</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1535,17 +1535,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1559,19 +1559,19 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="O14" t="n">
-        <v>38.8</v>
+        <v>44.4</v>
       </c>
       <c r="P14" t="n">
-        <v>56.3</v>
+        <v>51.6</v>
       </c>
       <c r="Q14" t="n">
-        <v>2.9</v>
+        <v>2.4</v>
       </c>
       <c r="R14" t="n">
-        <v>2.9</v>
+        <v>2.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-11 13:27
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,37 +511,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -575,35 +575,35 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>115</v>
+        <v>90</v>
       </c>
       <c r="O2" t="n">
-        <v>39.1</v>
+        <v>41.1</v>
       </c>
       <c r="P2" t="n">
-        <v>56.5</v>
+        <v>55.6</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -613,37 +613,37 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>36.7</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -653,39 +653,39 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>115</v>
+        <v>59</v>
       </c>
       <c r="O3" t="n">
-        <v>39.1</v>
+        <v>55.9</v>
       </c>
       <c r="P3" t="n">
-        <v>56.5</v>
+        <v>39</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.9</v>
+        <v>3.4</v>
       </c>
       <c r="R3" t="n">
-        <v>0.9</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,37 +695,37 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,59 +735,59 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>102</v>
+        <v>136</v>
       </c>
       <c r="O4" t="n">
-        <v>50</v>
+        <v>44.1</v>
       </c>
       <c r="P4" t="n">
-        <v>44.1</v>
+        <v>52.2</v>
       </c>
       <c r="Q4" t="n">
-        <v>3.9</v>
+        <v>1.5</v>
       </c>
       <c r="R4" t="n">
-        <v>3.9</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,50 +821,50 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>97</v>
+        <v>129</v>
       </c>
       <c r="O5" t="n">
-        <v>49.5</v>
+        <v>48.1</v>
       </c>
       <c r="P5" t="n">
-        <v>44.3</v>
+        <v>47.3</v>
       </c>
       <c r="Q5" t="n">
-        <v>4.1</v>
+        <v>3.1</v>
       </c>
       <c r="R5" t="n">
-        <v>4.1</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -884,12 +884,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>13.3</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -903,75 +903,75 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="O6" t="n">
-        <v>51.3</v>
+        <v>49.5</v>
       </c>
       <c r="P6" t="n">
-        <v>43.4</v>
+        <v>44.2</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.3</v>
+        <v>4.2</v>
       </c>
       <c r="R6" t="n">
-        <v>5.3</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>57.0</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>43.0</t>
-        </is>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-6</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -981,39 +981,39 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="O7" t="n">
-        <v>47.5</v>
+        <v>43</v>
       </c>
       <c r="P7" t="n">
-        <v>47.5</v>
+        <v>53.5</v>
       </c>
       <c r="Q7" t="n">
-        <v>3.4</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>3.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-6</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,17 +1043,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1067,13 +1067,13 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="O8" t="n">
-        <v>42.6</v>
+        <v>43</v>
       </c>
       <c r="P8" t="n">
-        <v>53.7</v>
+        <v>53.5</v>
       </c>
       <c r="Q8" t="n">
         <v>0</v>
@@ -1085,42 +1085,42 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1130,38 +1130,38 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="O9" t="n">
-        <v>42.6</v>
+        <v>46.8</v>
       </c>
       <c r="P9" t="n">
-        <v>53.7</v>
+        <v>48.4</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="10">
@@ -1172,12 +1172,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1212,12 +1212,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1231,19 +1231,19 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="O10" t="n">
-        <v>43.9</v>
+        <v>47</v>
       </c>
       <c r="P10" t="n">
-        <v>52</v>
+        <v>48.5</v>
       </c>
       <c r="Q10" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="R10" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1254,12 +1254,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1289,17 +1289,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>0.9</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1313,35 +1313,35 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="O11" t="n">
-        <v>45.6</v>
+        <v>46.4</v>
       </c>
       <c r="P11" t="n">
-        <v>50.4</v>
+        <v>49.3</v>
       </c>
       <c r="Q11" t="n">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
       <c r="R11" t="n">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1351,12 +1351,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1376,12 +1376,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1395,35 +1395,35 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="O12" t="n">
-        <v>44.4</v>
+        <v>47</v>
       </c>
       <c r="P12" t="n">
-        <v>51.6</v>
+        <v>48.5</v>
       </c>
       <c r="Q12" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="R12" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1433,17 +1433,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7-6</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1453,17 +1453,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>97.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>79.4</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>57.5</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,101 +1477,183 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="O13" t="n">
-        <v>43.9</v>
+        <v>47</v>
       </c>
       <c r="P13" t="n">
-        <v>52</v>
+        <v>48.5</v>
       </c>
       <c r="Q13" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="R13" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>51.8</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>132</v>
+      </c>
+      <c r="O14" t="n">
+        <v>47</v>
+      </c>
+      <c r="P14" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>3</v>
+      </c>
+      <c r="R14" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>Uni Lions</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Wei Chuan Dragons</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>CPB</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>51.0</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>49.0</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
         <is>
           <t>3-2</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>23.8</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>0.7</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>9.7</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="N14" t="n">
-        <v>126</v>
-      </c>
-      <c r="O14" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="P14" t="n">
-        <v>51.6</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="R14" t="n">
-        <v>2.4</v>
+      <c r="N15" t="n">
+        <v>138</v>
+      </c>
+      <c r="O15" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="P15" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="R15" t="n">
+        <v>2.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-12 11:56
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:R21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,17 +511,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -575,35 +575,35 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>90</v>
+        <v>129</v>
       </c>
       <c r="O2" t="n">
         <v>41.1</v>
       </c>
       <c r="P2" t="n">
-        <v>55.6</v>
+        <v>55</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="R2" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>2:40</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -613,37 +613,37 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>26.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>2-5</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>36.7</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -653,39 +653,39 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="O3" t="n">
-        <v>55.9</v>
+        <v>37.5</v>
       </c>
       <c r="P3" t="n">
-        <v>39</v>
+        <v>58.3</v>
       </c>
       <c r="Q3" t="n">
-        <v>3.4</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>3.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,37 +695,37 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,59 +735,59 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="O4" t="n">
-        <v>44.1</v>
+        <v>48.9</v>
       </c>
       <c r="P4" t="n">
-        <v>52.2</v>
+        <v>46.7</v>
       </c>
       <c r="Q4" t="n">
-        <v>1.5</v>
+        <v>2.9</v>
       </c>
       <c r="R4" t="n">
-        <v>1.5</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,40 +821,40 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="O5" t="n">
-        <v>48.1</v>
+        <v>48</v>
       </c>
       <c r="P5" t="n">
-        <v>47.3</v>
+        <v>48</v>
       </c>
       <c r="Q5" t="n">
-        <v>3.1</v>
+        <v>2.7</v>
       </c>
       <c r="R5" t="n">
-        <v>3.1</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -884,12 +884,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>13.3</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -903,60 +903,60 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="O6" t="n">
-        <v>49.5</v>
+        <v>49</v>
       </c>
       <c r="P6" t="n">
-        <v>44.2</v>
+        <v>45.1</v>
       </c>
       <c r="Q6" t="n">
-        <v>4.2</v>
+        <v>3.9</v>
       </c>
       <c r="R6" t="n">
-        <v>4.2</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>1:15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3-6</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -966,12 +966,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -981,79 +981,79 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>114</v>
+        <v>148</v>
       </c>
       <c r="O7" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="P7" t="n">
-        <v>53.5</v>
+        <v>48</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1063,59 +1063,59 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>114</v>
+        <v>148</v>
       </c>
       <c r="O8" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="P8" t="n">
-        <v>53.5</v>
+        <v>48</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>2:40</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1125,22 +1125,22 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>36.7</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1149,137 +1149,137 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>124</v>
+        <v>61</v>
       </c>
       <c r="O9" t="n">
-        <v>46.8</v>
+        <v>54.1</v>
       </c>
       <c r="P9" t="n">
-        <v>48.4</v>
+        <v>41</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="R9" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>2:40</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>16.5</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="O10" t="n">
-        <v>47</v>
+        <v>44.4</v>
       </c>
       <c r="P10" t="n">
-        <v>48.5</v>
+        <v>52.1</v>
       </c>
       <c r="Q10" t="n">
-        <v>3</v>
+        <v>1.4</v>
       </c>
       <c r="R10" t="n">
-        <v>3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3-1</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1289,22 +1289,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>0.9</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1313,50 +1313,50 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="O11" t="n">
-        <v>46.4</v>
+        <v>50</v>
       </c>
       <c r="P11" t="n">
-        <v>49.3</v>
+        <v>45</v>
       </c>
       <c r="Q11" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
       <c r="R11" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1376,17 +1376,17 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1395,35 +1395,35 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>132</v>
+        <v>61</v>
       </c>
       <c r="O12" t="n">
-        <v>47</v>
+        <v>54.1</v>
       </c>
       <c r="P12" t="n">
-        <v>48.5</v>
+        <v>41</v>
       </c>
       <c r="Q12" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="R12" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>3:35</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1433,79 +1433,79 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="O13" t="n">
-        <v>47</v>
+        <v>44.2</v>
       </c>
       <c r="P13" t="n">
-        <v>48.5</v>
+        <v>52.5</v>
       </c>
       <c r="Q13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>5:05</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1515,17 +1515,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>72.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>28.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1535,22 +1535,22 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1559,101 +1559,593 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>132</v>
+        <v>49</v>
       </c>
       <c r="O14" t="n">
-        <v>47</v>
+        <v>53.1</v>
       </c>
       <c r="P14" t="n">
-        <v>48.5</v>
+        <v>42.9</v>
       </c>
       <c r="Q14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Chinatrust Brothers</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2-5</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>144</v>
+      </c>
+      <c r="O15" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="P15" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>36.6</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>144</v>
+      </c>
+      <c r="O16" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="P16" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="R16" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Fukuoka S. Hawks</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Rakuten Gold. Eagles</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>10.6</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>132</v>
+      </c>
+      <c r="O17" t="n">
+        <v>47</v>
+      </c>
+      <c r="P17" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>3</v>
+      </c>
+      <c r="R17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Yokohama BayStars</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Yomiuri Giants</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>16.3</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>145</v>
+      </c>
+      <c r="O18" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="P18" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="R18" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2:40</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>51.8</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>132</v>
+      </c>
+      <c r="O19" t="n">
+        <v>47</v>
+      </c>
+      <c r="P19" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>3</v>
+      </c>
+      <c r="R19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>3:15</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>145</v>
+      </c>
+      <c r="O20" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="P20" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="R20" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>17:05</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Uni Lions</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Wei Chuan Dragons</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>CPB</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>52.0</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>48.0</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>3-2</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>23.8</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>9.7</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="N15" t="n">
-        <v>138</v>
-      </c>
-      <c r="O15" t="n">
-        <v>44.2</v>
-      </c>
-      <c r="P15" t="n">
-        <v>52.2</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="R15" t="n">
-        <v>2.2</v>
+      <c r="N21" t="n">
+        <v>148</v>
+      </c>
+      <c r="O21" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="P21" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>2</v>
+      </c>
+      <c r="R21" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-15 12:43
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,17 +511,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,12 +531,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -556,17 +556,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -575,19 +575,19 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="O2" t="n">
-        <v>42.9</v>
+        <v>40.9</v>
       </c>
       <c r="P2" t="n">
-        <v>53.9</v>
+        <v>55.7</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.6</v>
+        <v>67.8</v>
       </c>
       <c r="R2" t="n">
-        <v>0.6</v>
+        <v>50.3</v>
       </c>
     </row>
     <row r="3">
@@ -598,12 +598,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -613,22 +613,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -638,74 +638,74 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>132</v>
+        <v>149</v>
       </c>
       <c r="O3" t="n">
-        <v>50</v>
+        <v>40.9</v>
       </c>
       <c r="P3" t="n">
-        <v>45.5</v>
+        <v>55.7</v>
       </c>
       <c r="Q3" t="n">
-        <v>3</v>
+        <v>67.8</v>
       </c>
       <c r="R3" t="n">
-        <v>3</v>
+        <v>50.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,22 +715,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -739,35 +739,35 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>154</v>
+        <v>106</v>
       </c>
       <c r="O4" t="n">
-        <v>42.9</v>
+        <v>40.6</v>
       </c>
       <c r="P4" t="n">
-        <v>53.9</v>
+        <v>56.6</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.6</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="R4" t="n">
-        <v>0.6</v>
+        <v>52.8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -777,17 +777,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,19 +821,19 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="O5" t="n">
-        <v>44.2</v>
+        <v>42</v>
       </c>
       <c r="P5" t="n">
-        <v>52.8</v>
+        <v>54.8</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.2</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="R5" t="n">
-        <v>1.2</v>
+        <v>49.7</v>
       </c>
     </row>
     <row r="6">
@@ -844,12 +844,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,37 +859,37 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>41.0</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>59.0</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,79 +899,79 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>110</v>
+        <v>147</v>
       </c>
       <c r="O6" t="n">
-        <v>42.7</v>
+        <v>49.7</v>
       </c>
       <c r="P6" t="n">
-        <v>54.5</v>
+        <v>46.3</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="R6" t="n">
-        <v>0</v>
+        <v>45.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -981,187 +981,269 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>154</v>
+        <v>123</v>
       </c>
       <c r="O7" t="n">
-        <v>42.9</v>
+        <v>50.4</v>
       </c>
       <c r="P7" t="n">
-        <v>53.9</v>
+        <v>44.7</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.6</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="R7" t="n">
-        <v>0.6</v>
+        <v>46.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
           <t>55.0</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>45.0</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>3-2</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>23.8</t>
-        </is>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N8" t="n">
         <v>170</v>
       </c>
       <c r="O8" t="n">
-        <v>47.6</v>
+        <v>43.5</v>
       </c>
       <c r="P8" t="n">
-        <v>48.8</v>
+        <v>53.5</v>
       </c>
       <c r="Q8" t="n">
-        <v>2.4</v>
+        <v>68.8</v>
       </c>
       <c r="R8" t="n">
-        <v>2.4</v>
+        <v>51.8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Yakult Swallows</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Yomiuri Giants</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>15.3</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>176</v>
+      </c>
+      <c r="O9" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="P9" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="R9" t="n">
+        <v>50.6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>19:35</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>TSG Hawks</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Fubon Guardians</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>CPB</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>54.0</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>46.0</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>47.7</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>23.7</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="N9" t="n">
-        <v>170</v>
-      </c>
-      <c r="O9" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="P9" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="R9" t="n">
-        <v>1.8</v>
+      <c r="N10" t="n">
+        <v>175</v>
+      </c>
+      <c r="O10" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="P10" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>68</v>
+      </c>
+      <c r="R10" t="n">
+        <v>49.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-16 13:17
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,57 +511,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>10-5</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>99.2</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>93.8</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>82.4</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,79 +571,79 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>149</v>
+        <v>62</v>
       </c>
       <c r="O2" t="n">
-        <v>40.9</v>
+        <v>58.1</v>
       </c>
       <c r="P2" t="n">
-        <v>55.7</v>
+        <v>38.7</v>
       </c>
       <c r="Q2" t="n">
-        <v>67.8</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="R2" t="n">
-        <v>50.3</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -653,121 +653,121 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>149</v>
+        <v>72</v>
       </c>
       <c r="O3" t="n">
-        <v>40.9</v>
+        <v>58.3</v>
       </c>
       <c r="P3" t="n">
-        <v>55.7</v>
+        <v>37.5</v>
       </c>
       <c r="Q3" t="n">
-        <v>67.8</v>
+        <v>65.3</v>
       </c>
       <c r="R3" t="n">
-        <v>50.3</v>
+        <v>43.1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>40.0</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>60.0</t>
-        </is>
-      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>106</v>
+        <v>146</v>
       </c>
       <c r="O4" t="n">
-        <v>40.6</v>
+        <v>50.7</v>
       </c>
       <c r="P4" t="n">
-        <v>56.6</v>
+        <v>45.2</v>
       </c>
       <c r="Q4" t="n">
-        <v>68.90000000000001</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="R4" t="n">
-        <v>52.8</v>
+        <v>46.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -777,37 +777,37 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -817,23 +817,23 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>157</v>
+        <v>185</v>
       </c>
       <c r="O5" t="n">
-        <v>42</v>
+        <v>48.6</v>
       </c>
       <c r="P5" t="n">
-        <v>54.8</v>
+        <v>48.1</v>
       </c>
       <c r="Q5" t="n">
-        <v>66.90000000000001</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="R5" t="n">
-        <v>49.7</v>
+        <v>48.1</v>
       </c>
     </row>
     <row r="6">
@@ -844,12 +844,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,37 +859,37 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,79 +899,79 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="O6" t="n">
-        <v>49.7</v>
+        <v>43.7</v>
       </c>
       <c r="P6" t="n">
-        <v>46.3</v>
+        <v>53.5</v>
       </c>
       <c r="Q6" t="n">
-        <v>68</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="R6" t="n">
-        <v>45.6</v>
+        <v>51.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>66.7</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>41.7</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -981,59 +981,59 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>123</v>
+        <v>177</v>
       </c>
       <c r="O7" t="n">
-        <v>50.4</v>
+        <v>44.1</v>
       </c>
       <c r="P7" t="n">
-        <v>44.7</v>
+        <v>53.1</v>
       </c>
       <c r="Q7" t="n">
-        <v>65.90000000000001</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="R7" t="n">
-        <v>46.3</v>
+        <v>52.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3-6</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,17 +1043,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1067,101 +1067,101 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>170</v>
+        <v>130</v>
       </c>
       <c r="O8" t="n">
-        <v>43.5</v>
+        <v>43.8</v>
       </c>
       <c r="P8" t="n">
-        <v>53.5</v>
+        <v>54.6</v>
       </c>
       <c r="Q8" t="n">
-        <v>68.8</v>
+        <v>71.5</v>
       </c>
       <c r="R8" t="n">
-        <v>51.8</v>
+        <v>53.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>67.8</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>42.9</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>176</v>
+        <v>142</v>
       </c>
       <c r="O9" t="n">
-        <v>45.5</v>
+        <v>43.7</v>
       </c>
       <c r="P9" t="n">
-        <v>51.7</v>
+        <v>53.5</v>
       </c>
       <c r="Q9" t="n">
-        <v>67.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="R9" t="n">
-        <v>50.6</v>
+        <v>51.4</v>
       </c>
     </row>
     <row r="10">
@@ -1187,63 +1187,309 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>53.0</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>168</v>
+      </c>
+      <c r="O10" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="P10" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="R10" t="n">
+        <v>51.2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Nippon Ham Fighters</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Fukuoka S. Hawks</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>47.0</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>40.7</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>183</v>
+      </c>
+      <c r="O11" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="P11" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="R11" t="n">
+        <v>50.3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Yakult Swallows</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Yomiuri Giants</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>3-2</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>23.8</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>0.7</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="N10" t="n">
-        <v>175</v>
-      </c>
-      <c r="O10" t="n">
-        <v>46.3</v>
-      </c>
-      <c r="P10" t="n">
-        <v>50.9</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>68</v>
-      </c>
-      <c r="R10" t="n">
-        <v>49.1</v>
+      <c r="N12" t="n">
+        <v>183</v>
+      </c>
+      <c r="O12" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="P12" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="R12" t="n">
+        <v>50.3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>7-5</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>81.7</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>60.9</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>160</v>
+      </c>
+      <c r="O13" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="P13" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="R13" t="n">
+        <v>46.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-17 14:36
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,57 +511,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>73.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>10-5</t>
+          <t>2-6</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>99.2</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>93.8</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>82.4</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,59 +571,59 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="O2" t="n">
-        <v>58.1</v>
+        <v>36</v>
       </c>
       <c r="P2" t="n">
-        <v>38.7</v>
+        <v>60</v>
       </c>
       <c r="Q2" t="n">
-        <v>69.40000000000001</v>
+        <v>72</v>
       </c>
       <c r="R2" t="n">
-        <v>43.5</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,55 +657,55 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="O3" t="n">
-        <v>58.3</v>
+        <v>55.7</v>
       </c>
       <c r="P3" t="n">
-        <v>37.5</v>
+        <v>41.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>65.3</v>
+        <v>67</v>
       </c>
       <c r="R3" t="n">
-        <v>43.1</v>
+        <v>45.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,22 +715,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -739,19 +739,19 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>146</v>
+        <v>69</v>
       </c>
       <c r="O4" t="n">
-        <v>50.7</v>
+        <v>56.5</v>
       </c>
       <c r="P4" t="n">
-        <v>45.2</v>
+        <v>40.6</v>
       </c>
       <c r="Q4" t="n">
-        <v>67.09999999999999</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="R4" t="n">
-        <v>46.6</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="5">
@@ -762,12 +762,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -777,12 +777,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -802,12 +802,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,19 +821,19 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>185</v>
+        <v>132</v>
       </c>
       <c r="O5" t="n">
-        <v>48.6</v>
+        <v>49.2</v>
       </c>
       <c r="P5" t="n">
-        <v>48.1</v>
+        <v>46.2</v>
       </c>
       <c r="Q5" t="n">
-        <v>67.59999999999999</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="R5" t="n">
-        <v>48.1</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="6">
@@ -844,32 +844,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -879,17 +879,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>67.8</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>42.9</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -903,25 +903,25 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>142</v>
+        <v>172</v>
       </c>
       <c r="O6" t="n">
-        <v>43.7</v>
+        <v>43</v>
       </c>
       <c r="P6" t="n">
-        <v>53.5</v>
+        <v>54.1</v>
       </c>
       <c r="Q6" t="n">
-        <v>70.40000000000001</v>
+        <v>66.3</v>
       </c>
       <c r="R6" t="n">
-        <v>51.4</v>
+        <v>48.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -966,12 +966,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>66.7</t>
+          <t>65.6</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>41.7</t>
+          <t>40.4</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,35 +985,35 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="O7" t="n">
         <v>44.1</v>
       </c>
       <c r="P7" t="n">
-        <v>53.1</v>
+        <v>53.2</v>
       </c>
       <c r="Q7" t="n">
-        <v>68.90000000000001</v>
+        <v>68.3</v>
       </c>
       <c r="R7" t="n">
-        <v>52.5</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1023,37 +1023,37 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-6</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>81.7</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>60.9</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1063,79 +1063,79 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="O8" t="n">
-        <v>43.8</v>
+        <v>51.7</v>
       </c>
       <c r="P8" t="n">
-        <v>54.6</v>
+        <v>44.8</v>
       </c>
       <c r="Q8" t="n">
-        <v>71.5</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="R8" t="n">
-        <v>53.1</v>
+        <v>46.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>67.8</t>
+          <t>63.2</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>42.9</t>
+          <t>37.9</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1145,59 +1145,59 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="O9" t="n">
-        <v>43.7</v>
+        <v>48.7</v>
       </c>
       <c r="P9" t="n">
-        <v>53.5</v>
+        <v>47.4</v>
       </c>
       <c r="Q9" t="n">
-        <v>70.40000000000001</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="R9" t="n">
-        <v>51.4</v>
+        <v>44.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,17 +1207,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1231,55 +1231,55 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>168</v>
+        <v>190</v>
       </c>
       <c r="O10" t="n">
-        <v>42.9</v>
+        <v>45.3</v>
       </c>
       <c r="P10" t="n">
-        <v>54.2</v>
+        <v>52.1</v>
       </c>
       <c r="Q10" t="n">
-        <v>67.90000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="R10" t="n">
-        <v>51.2</v>
+        <v>48.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>9:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1289,22 +1289,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1313,183 +1313,1003 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>183</v>
+        <v>116</v>
       </c>
       <c r="O11" t="n">
-        <v>47.5</v>
+        <v>51.7</v>
       </c>
       <c r="P11" t="n">
-        <v>49.7</v>
+        <v>44.8</v>
       </c>
       <c r="Q11" t="n">
-        <v>68.3</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="R11" t="n">
-        <v>50.3</v>
+        <v>46.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>9:10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-7</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>73.1</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>49.2</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>183</v>
+        <v>118</v>
       </c>
       <c r="O12" t="n">
-        <v>47.5</v>
+        <v>44.1</v>
       </c>
       <c r="P12" t="n">
-        <v>49.7</v>
+        <v>53.4</v>
       </c>
       <c r="Q12" t="n">
-        <v>68.3</v>
+        <v>67.8</v>
       </c>
       <c r="R12" t="n">
-        <v>50.3</v>
+        <v>50.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>9:40</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>5-6</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>92.1</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>51.6</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>186</v>
+      </c>
+      <c r="O13" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="P13" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="R13" t="n">
+        <v>50.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>10:38</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>43.5</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>125</v>
+      </c>
+      <c r="O14" t="n">
+        <v>44</v>
+      </c>
+      <c r="P14" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="R14" t="n">
+        <v>50.4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>145</v>
+      </c>
+      <c r="O15" t="n">
+        <v>49</v>
+      </c>
+      <c r="P15" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="R15" t="n">
+        <v>46.9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Yokohama BayStars</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Yakult Swallows</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>192</v>
+      </c>
+      <c r="O16" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="P16" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="R16" t="n">
+        <v>48.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>Samsung Lions</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Lotte Giants</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>KBO</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>7-5</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>81.7</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>60.9</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>192</v>
+      </c>
+      <c r="O17" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="P17" t="n">
+        <v>49</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="R17" t="n">
+        <v>46.9</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2:35</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>58.0</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>42.0</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>7-5</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>95.4</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>81.7</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>60.9</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="N13" t="n">
-        <v>160</v>
-      </c>
-      <c r="O13" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="P13" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>69.40000000000001</v>
-      </c>
-      <c r="R13" t="n">
+      <c r="N18" t="n">
+        <v>166</v>
+      </c>
+      <c r="O18" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="P18" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="R18" t="n">
+        <v>45.8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>33.8</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>13.8</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>192</v>
+      </c>
+      <c r="O19" t="n">
         <v>46.9</v>
+      </c>
+      <c r="P19" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="R19" t="n">
+        <v>48.4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>51.8</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>180</v>
+      </c>
+      <c r="O20" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="P20" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="R20" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>32.4</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>12.9</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>193</v>
+      </c>
+      <c r="O21" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="P21" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="R21" t="n">
+        <v>49.2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>192</v>
+      </c>
+      <c r="O22" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="P22" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="R22" t="n">
+        <v>48.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>6-5</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>92.1</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>65.6</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>40.4</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>166</v>
+      </c>
+      <c r="O23" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="P23" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="R23" t="n">
+        <v>45.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-18 11:36
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:R17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,17 +531,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>73.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2-6</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,22 +551,22 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>35.2</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>14.6</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -575,55 +575,55 @@
         </is>
       </c>
       <c r="N2" t="n">
+        <v>28</v>
+      </c>
+      <c r="O2" t="n">
         <v>25</v>
       </c>
-      <c r="O2" t="n">
-        <v>36</v>
-      </c>
       <c r="P2" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="Q2" t="n">
-        <v>72</v>
+        <v>10.7</v>
       </c>
       <c r="R2" t="n">
-        <v>52</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>5:05</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,22 +633,22 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -657,55 +657,55 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>97</v>
+        <v>14</v>
       </c>
       <c r="O3" t="n">
-        <v>55.7</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="P3" t="n">
-        <v>41.2</v>
+        <v>21.4</v>
       </c>
       <c r="Q3" t="n">
-        <v>67</v>
+        <v>21.4</v>
       </c>
       <c r="R3" t="n">
-        <v>45.4</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,17 +715,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -739,25 +739,25 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>69</v>
+        <v>34</v>
       </c>
       <c r="O4" t="n">
-        <v>56.5</v>
+        <v>61.8</v>
       </c>
       <c r="P4" t="n">
-        <v>40.6</v>
+        <v>35.3</v>
       </c>
       <c r="Q4" t="n">
-        <v>69.59999999999999</v>
+        <v>11.8</v>
       </c>
       <c r="R4" t="n">
-        <v>46.4</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -777,17 +777,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,22 +797,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>14.3</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -821,19 +821,19 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>132</v>
+        <v>34</v>
       </c>
       <c r="O5" t="n">
-        <v>49.2</v>
+        <v>61.8</v>
       </c>
       <c r="P5" t="n">
-        <v>46.2</v>
+        <v>35.3</v>
       </c>
       <c r="Q5" t="n">
-        <v>65.90000000000001</v>
+        <v>11.8</v>
       </c>
       <c r="R5" t="n">
-        <v>45.5</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="6">
@@ -844,12 +844,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,12 +859,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -884,17 +884,17 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>67.8</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>42.9</t>
+          <t>50.4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -903,19 +903,19 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>172</v>
+        <v>17</v>
       </c>
       <c r="O6" t="n">
-        <v>43</v>
+        <v>41.2</v>
       </c>
       <c r="P6" t="n">
-        <v>54.1</v>
+        <v>58.8</v>
       </c>
       <c r="Q6" t="n">
-        <v>66.3</v>
+        <v>5.9</v>
       </c>
       <c r="R6" t="n">
-        <v>48.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -926,32 +926,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,17 +961,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>65.6</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>40.4</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,19 +985,19 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>186</v>
+        <v>70</v>
       </c>
       <c r="O7" t="n">
-        <v>44.1</v>
+        <v>42.9</v>
       </c>
       <c r="P7" t="n">
-        <v>53.2</v>
+        <v>54.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>68.3</v>
+        <v>15.7</v>
       </c>
       <c r="R7" t="n">
-        <v>50.5</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="8">
@@ -1008,52 +1008,52 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>81.7</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>60.9</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1063,59 +1063,59 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>116</v>
+        <v>70</v>
       </c>
       <c r="O8" t="n">
-        <v>51.7</v>
+        <v>42.9</v>
       </c>
       <c r="P8" t="n">
-        <v>44.8</v>
+        <v>54.3</v>
       </c>
       <c r="Q8" t="n">
-        <v>66.40000000000001</v>
+        <v>15.7</v>
       </c>
       <c r="R8" t="n">
-        <v>46.6</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1125,17 +1125,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>63.2</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>37.9</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1149,55 +1149,55 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>156</v>
+        <v>63</v>
       </c>
       <c r="O9" t="n">
-        <v>48.7</v>
+        <v>52.4</v>
       </c>
       <c r="P9" t="n">
-        <v>47.4</v>
+        <v>42.9</v>
       </c>
       <c r="Q9" t="n">
-        <v>67.90000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="R9" t="n">
-        <v>44.9</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,17 +1207,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>66.7</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>41.7</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1231,35 +1231,35 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>190</v>
+        <v>19</v>
       </c>
       <c r="O10" t="n">
-        <v>45.3</v>
+        <v>47.4</v>
       </c>
       <c r="P10" t="n">
-        <v>52.1</v>
+        <v>52.6</v>
       </c>
       <c r="Q10" t="n">
-        <v>66.8</v>
+        <v>26.3</v>
       </c>
       <c r="R10" t="n">
-        <v>48.9</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1289,17 +1289,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1313,35 +1313,35 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O11" t="n">
-        <v>51.7</v>
+        <v>48.7</v>
       </c>
       <c r="P11" t="n">
-        <v>44.8</v>
+        <v>48.7</v>
       </c>
       <c r="Q11" t="n">
-        <v>66.40000000000001</v>
+        <v>16.5</v>
       </c>
       <c r="R11" t="n">
-        <v>46.6</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1351,17 +1351,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4-7</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1371,17 +1371,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>73.1</t>
+          <t>63.2</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>49.2</t>
+          <t>37.9</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1395,35 +1395,35 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>118</v>
+        <v>19</v>
       </c>
       <c r="O12" t="n">
-        <v>44.1</v>
+        <v>47.4</v>
       </c>
       <c r="P12" t="n">
-        <v>53.4</v>
+        <v>52.6</v>
       </c>
       <c r="Q12" t="n">
-        <v>67.8</v>
+        <v>26.3</v>
       </c>
       <c r="R12" t="n">
-        <v>50.8</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1433,37 +1433,37 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>51.6</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1473,59 +1473,59 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>186</v>
+        <v>115</v>
       </c>
       <c r="O13" t="n">
-        <v>44.1</v>
+        <v>48.7</v>
       </c>
       <c r="P13" t="n">
-        <v>53.2</v>
+        <v>48.7</v>
       </c>
       <c r="Q13" t="n">
-        <v>68.3</v>
+        <v>16.5</v>
       </c>
       <c r="R13" t="n">
-        <v>50.5</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>10:38</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1535,22 +1535,22 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1559,55 +1559,55 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>125</v>
+        <v>26</v>
       </c>
       <c r="O14" t="n">
-        <v>44</v>
+        <v>57.7</v>
       </c>
       <c r="P14" t="n">
-        <v>53.6</v>
+        <v>42.3</v>
       </c>
       <c r="Q14" t="n">
-        <v>69.59999999999999</v>
+        <v>19.2</v>
       </c>
       <c r="R14" t="n">
-        <v>50.4</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1617,22 +1617,22 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>81.7</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>60.9</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1641,19 +1641,19 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>145</v>
+        <v>16</v>
       </c>
       <c r="O15" t="n">
-        <v>49</v>
+        <v>43.8</v>
       </c>
       <c r="P15" t="n">
-        <v>46.9</v>
+        <v>56.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>66.90000000000001</v>
+        <v>37.5</v>
       </c>
       <c r="R15" t="n">
-        <v>46.9</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16">
@@ -1664,32 +1664,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1699,17 +1699,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>81.7</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>60.9</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1723,75 +1723,75 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>192</v>
+        <v>16</v>
       </c>
       <c r="O16" t="n">
-        <v>46.9</v>
+        <v>43.8</v>
       </c>
       <c r="P16" t="n">
-        <v>50.5</v>
+        <v>56.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>67.7</v>
+        <v>37.5</v>
       </c>
       <c r="R16" t="n">
-        <v>48.4</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>9:08</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>81.7</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>60.9</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1801,515 +1801,23 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>192</v>
+        <v>51</v>
       </c>
       <c r="O17" t="n">
-        <v>47.9</v>
+        <v>49</v>
       </c>
       <c r="P17" t="n">
         <v>49</v>
       </c>
       <c r="Q17" t="n">
-        <v>67.7</v>
+        <v>21.6</v>
       </c>
       <c r="R17" t="n">
-        <v>46.9</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2:35</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>58.0</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>42.0</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>27.1</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>9.9</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N18" t="n">
-        <v>166</v>
-      </c>
-      <c r="O18" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="P18" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>69.90000000000001</v>
-      </c>
-      <c r="R18" t="n">
-        <v>45.8</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>8:10</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Cleveland Guardians</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Pittsburgh Pirates</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>33.8</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>13.8</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N19" t="n">
-        <v>192</v>
-      </c>
-      <c r="O19" t="n">
-        <v>46.9</v>
-      </c>
-      <c r="P19" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>67.7</v>
-      </c>
-      <c r="R19" t="n">
-        <v>48.4</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>8:15</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Toronto Blue Jays</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Chicago White Sox</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>56.0</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>44.0</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>51.8</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>27.1</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N20" t="n">
-        <v>180</v>
-      </c>
-      <c r="O20" t="n">
-        <v>47.8</v>
-      </c>
-      <c r="P20" t="n">
-        <v>48.9</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>67.2</v>
-      </c>
-      <c r="R20" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>8:15</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Atlanta Braves</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Texas Rangers</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>52.0</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>48.0</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>32.4</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>12.9</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N21" t="n">
-        <v>193</v>
-      </c>
-      <c r="O21" t="n">
-        <v>46.1</v>
-      </c>
-      <c r="P21" t="n">
-        <v>51.3</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>67.40000000000001</v>
-      </c>
-      <c r="R21" t="n">
-        <v>49.2</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Arizona Diamondbacks</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>St.Louis Cardinals</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>29.7</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>11.3</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N22" t="n">
-        <v>192</v>
-      </c>
-      <c r="O22" t="n">
-        <v>46.9</v>
-      </c>
-      <c r="P22" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>67.7</v>
-      </c>
-      <c r="R22" t="n">
-        <v>48.4</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Athletics</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Washington Nationals</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>58.0</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>42.0</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>6-5</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>92.1</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>65.6</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>40.4</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N23" t="n">
-        <v>166</v>
-      </c>
-      <c r="O23" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="P23" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>69.90000000000001</v>
-      </c>
-      <c r="R23" t="n">
-        <v>45.8</v>
+        <v>17.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-19 14:11
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R17"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -575,25 +575,25 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="O2" t="n">
-        <v>25</v>
+        <v>27.6</v>
       </c>
       <c r="P2" t="n">
-        <v>75</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="Q2" t="n">
-        <v>10.7</v>
+        <v>10.3</v>
       </c>
       <c r="R2" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>5:05</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -613,12 +613,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -638,12 +638,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -675,37 +675,37 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>3:20</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,22 +715,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -739,19 +739,19 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="O4" t="n">
-        <v>61.8</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="P4" t="n">
-        <v>35.3</v>
+        <v>21.4</v>
       </c>
       <c r="Q4" t="n">
-        <v>11.8</v>
+        <v>21.4</v>
       </c>
       <c r="R4" t="n">
-        <v>5.9</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="5">
@@ -777,12 +777,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -821,19 +821,19 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O5" t="n">
-        <v>61.8</v>
+        <v>58.3</v>
       </c>
       <c r="P5" t="n">
-        <v>35.3</v>
+        <v>38.9</v>
       </c>
       <c r="Q5" t="n">
-        <v>11.8</v>
+        <v>11.1</v>
       </c>
       <c r="R5" t="n">
-        <v>5.9</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="6">
@@ -844,52 +844,52 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,23 +899,23 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="O6" t="n">
-        <v>41.2</v>
+        <v>58</v>
       </c>
       <c r="P6" t="n">
-        <v>58.8</v>
+        <v>39.1</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.9</v>
+        <v>24.6</v>
       </c>
       <c r="R6" t="n">
-        <v>0</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="7">
@@ -926,12 +926,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -941,63 +941,63 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="O7" t="n">
-        <v>42.9</v>
+        <v>58.3</v>
       </c>
       <c r="P7" t="n">
-        <v>54.3</v>
+        <v>38.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>15.7</v>
+        <v>11.1</v>
       </c>
       <c r="R7" t="n">
-        <v>11.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="8">
@@ -1008,32 +1008,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>66.7</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>41.7</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1067,19 +1067,19 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="O8" t="n">
-        <v>42.9</v>
+        <v>45</v>
       </c>
       <c r="P8" t="n">
-        <v>54.3</v>
+        <v>55</v>
       </c>
       <c r="Q8" t="n">
-        <v>15.7</v>
+        <v>30</v>
       </c>
       <c r="R8" t="n">
-        <v>11.4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1105,186 +1105,186 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>50.4</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="O9" t="n">
-        <v>52.4</v>
+        <v>36.8</v>
       </c>
       <c r="P9" t="n">
-        <v>42.9</v>
+        <v>63.2</v>
       </c>
       <c r="Q9" t="n">
-        <v>9.5</v>
+        <v>15.8</v>
       </c>
       <c r="R9" t="n">
-        <v>7.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>25.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>66.7</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>41.7</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="O10" t="n">
-        <v>47.4</v>
+        <v>58</v>
       </c>
       <c r="P10" t="n">
-        <v>52.6</v>
+        <v>39.1</v>
       </c>
       <c r="Q10" t="n">
-        <v>26.3</v>
+        <v>24.6</v>
       </c>
       <c r="R10" t="n">
-        <v>15.8</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>73.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1309,59 +1309,59 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>115</v>
+        <v>72</v>
       </c>
       <c r="O11" t="n">
-        <v>48.7</v>
+        <v>43.1</v>
       </c>
       <c r="P11" t="n">
-        <v>48.7</v>
+        <v>54.2</v>
       </c>
       <c r="Q11" t="n">
-        <v>16.5</v>
+        <v>16.7</v>
       </c>
       <c r="R11" t="n">
-        <v>9.6</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>6-7</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1371,17 +1371,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>97.4</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>63.2</t>
+          <t>85.8</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>37.9</t>
+          <t>67.3</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1395,35 +1395,35 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="O12" t="n">
-        <v>47.4</v>
+        <v>48</v>
       </c>
       <c r="P12" t="n">
-        <v>52.6</v>
+        <v>52</v>
       </c>
       <c r="Q12" t="n">
-        <v>26.3</v>
+        <v>32</v>
       </c>
       <c r="R12" t="n">
-        <v>15.8</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>1:15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1453,17 +1453,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>33.8</t>
+          <t>39.3</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,137 +1477,137 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>115</v>
+        <v>65</v>
       </c>
       <c r="O13" t="n">
-        <v>48.7</v>
+        <v>50.8</v>
       </c>
       <c r="P13" t="n">
-        <v>48.7</v>
+        <v>44.6</v>
       </c>
       <c r="Q13" t="n">
-        <v>16.5</v>
+        <v>12.3</v>
       </c>
       <c r="R13" t="n">
-        <v>9.6</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>26</v>
+        <v>119</v>
       </c>
       <c r="O14" t="n">
-        <v>57.7</v>
+        <v>48.7</v>
       </c>
       <c r="P14" t="n">
-        <v>42.3</v>
+        <v>48.7</v>
       </c>
       <c r="Q14" t="n">
-        <v>19.2</v>
+        <v>18.5</v>
       </c>
       <c r="R14" t="n">
-        <v>3.8</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>2:40</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1617,22 +1617,22 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>81.7</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>60.9</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1641,55 +1641,55 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="O15" t="n">
-        <v>43.8</v>
+        <v>53.3</v>
       </c>
       <c r="P15" t="n">
-        <v>56.2</v>
+        <v>33.3</v>
       </c>
       <c r="Q15" t="n">
-        <v>37.5</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1699,22 +1699,22 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>81.7</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>60.9</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1723,101 +1723,757 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="O16" t="n">
-        <v>43.8</v>
+        <v>50.8</v>
       </c>
       <c r="P16" t="n">
-        <v>56.2</v>
+        <v>44.6</v>
       </c>
       <c r="Q16" t="n">
-        <v>37.5</v>
+        <v>12.3</v>
       </c>
       <c r="R16" t="n">
-        <v>25</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>9:08</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>31.1</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>72</v>
+      </c>
+      <c r="O17" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="P17" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="R17" t="n">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>5:10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>119</v>
+      </c>
+      <c r="O18" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="P18" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="R18" t="n">
+        <v>10.1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Orix Buffaloes</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Nippon Ham Fighters</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>9.7</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>27</v>
+      </c>
+      <c r="O19" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="P19" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="R19" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>69.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>31.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>7-4</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>92.1</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>51.6</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>54</v>
+      </c>
+      <c r="O20" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="P20" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="R20" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Hanwha Eagles</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Kiwoom Heroes</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>7-4</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>92.1</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>51.6</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>54</v>
+      </c>
+      <c r="O21" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="P21" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="R21" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1:35</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>New York Yankees</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>MLB</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>40.0</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>60.0</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>4-5</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>79.3</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>42.1</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>19.4</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>원정승</t>
         </is>
       </c>
-      <c r="N17" t="n">
-        <v>51</v>
-      </c>
-      <c r="O17" t="n">
-        <v>49</v>
-      </c>
-      <c r="P17" t="n">
-        <v>49</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="R17" t="n">
-        <v>17.6</v>
+      <c r="N22" t="n">
+        <v>52</v>
+      </c>
+      <c r="O22" t="n">
+        <v>50</v>
+      </c>
+      <c r="P22" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="R22" t="n">
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2:35</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>52</v>
+      </c>
+      <c r="O23" t="n">
+        <v>50</v>
+      </c>
+      <c r="P23" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="R23" t="n">
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>31.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>69.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>4-8</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>80.9</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>59.8</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>9</v>
+      </c>
+      <c r="O24" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="P24" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="R24" t="n">
+        <v>22.2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>5:10</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>37.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-4</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>92.1</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>71.0</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>46.7</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>54</v>
+      </c>
+      <c r="O25" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="P25" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="R25" t="n">
+        <v>14.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-20 13:38
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R25"/>
+  <dimension ref="A1:R22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,57 +511,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,39 +571,39 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="O2" t="n">
-        <v>27.6</v>
+        <v>80</v>
       </c>
       <c r="P2" t="n">
-        <v>72.40000000000001</v>
+        <v>20</v>
       </c>
       <c r="Q2" t="n">
-        <v>10.3</v>
+        <v>20</v>
       </c>
       <c r="R2" t="n">
-        <v>3.4</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2:35</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -613,12 +613,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -638,12 +638,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,35 +657,35 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="O3" t="n">
-        <v>78.59999999999999</v>
+        <v>80</v>
       </c>
       <c r="P3" t="n">
-        <v>21.4</v>
+        <v>20</v>
       </c>
       <c r="Q3" t="n">
-        <v>21.4</v>
+        <v>20</v>
       </c>
       <c r="R3" t="n">
-        <v>14.3</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3:20</t>
+          <t>8:07</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,17 +695,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,22 +715,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -739,55 +739,55 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>14</v>
+        <v>70</v>
       </c>
       <c r="O4" t="n">
-        <v>78.59999999999999</v>
+        <v>58.6</v>
       </c>
       <c r="P4" t="n">
-        <v>21.4</v>
+        <v>38.6</v>
       </c>
       <c r="Q4" t="n">
-        <v>21.4</v>
+        <v>24.3</v>
       </c>
       <c r="R4" t="n">
-        <v>14.3</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,40 +821,40 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="O5" t="n">
-        <v>58.3</v>
+        <v>58.6</v>
       </c>
       <c r="P5" t="n">
-        <v>38.9</v>
+        <v>38.6</v>
       </c>
       <c r="Q5" t="n">
-        <v>11.1</v>
+        <v>24.3</v>
       </c>
       <c r="R5" t="n">
-        <v>5.6</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -884,12 +884,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -903,50 +903,50 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="O6" t="n">
-        <v>58</v>
+        <v>58.6</v>
       </c>
       <c r="P6" t="n">
-        <v>39.1</v>
+        <v>38.6</v>
       </c>
       <c r="Q6" t="n">
-        <v>24.6</v>
+        <v>24.3</v>
       </c>
       <c r="R6" t="n">
-        <v>17.4</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -966,12 +966,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,55 +985,55 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="O7" t="n">
-        <v>58.3</v>
+        <v>57.9</v>
       </c>
       <c r="P7" t="n">
-        <v>38.9</v>
+        <v>39.5</v>
       </c>
       <c r="Q7" t="n">
-        <v>11.1</v>
+        <v>13.2</v>
       </c>
       <c r="R7" t="n">
-        <v>5.6</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>9:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>6-7</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,17 +1043,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>97.4</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>66.7</t>
+          <t>80.9</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>41.7</t>
+          <t>59.8</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1067,183 +1067,183 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="O8" t="n">
-        <v>45</v>
+        <v>42.9</v>
       </c>
       <c r="P8" t="n">
-        <v>55</v>
+        <v>57.1</v>
       </c>
       <c r="Q8" t="n">
-        <v>30</v>
+        <v>39.3</v>
       </c>
       <c r="R8" t="n">
-        <v>20</v>
+        <v>32.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N9" t="n">
+        <v>121</v>
+      </c>
+      <c r="O9" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="P9" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="Q9" t="n">
         <v>19</v>
       </c>
-      <c r="O9" t="n">
-        <v>36.8</v>
-      </c>
-      <c r="P9" t="n">
-        <v>63.2</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>15.8</v>
-      </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>73.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="O10" t="n">
-        <v>58</v>
+        <v>42.5</v>
       </c>
       <c r="P10" t="n">
-        <v>39.1</v>
+        <v>54.8</v>
       </c>
       <c r="Q10" t="n">
-        <v>24.6</v>
+        <v>16.4</v>
       </c>
       <c r="R10" t="n">
-        <v>17.4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -1254,12 +1254,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1269,37 +1269,37 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>73.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1309,23 +1309,23 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>72</v>
+        <v>439</v>
       </c>
       <c r="O11" t="n">
-        <v>43.1</v>
+        <v>51.7</v>
       </c>
       <c r="P11" t="n">
-        <v>54.2</v>
+        <v>45.6</v>
       </c>
       <c r="Q11" t="n">
-        <v>16.7</v>
+        <v>18.5</v>
       </c>
       <c r="R11" t="n">
-        <v>11.1</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="12">
@@ -1336,52 +1336,52 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>6-7</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>97.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>85.8</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>67.3</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1391,59 +1391,59 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>25</v>
+        <v>121</v>
       </c>
       <c r="O12" t="n">
-        <v>48</v>
+        <v>48.8</v>
       </c>
       <c r="P12" t="n">
-        <v>52</v>
+        <v>48.8</v>
       </c>
       <c r="Q12" t="n">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="R12" t="n">
-        <v>24</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1:15</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1453,17 +1453,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,35 +1477,35 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>65</v>
+        <v>121</v>
       </c>
       <c r="O13" t="n">
-        <v>50.8</v>
+        <v>48.8</v>
       </c>
       <c r="P13" t="n">
-        <v>44.6</v>
+        <v>48.8</v>
       </c>
       <c r="Q13" t="n">
-        <v>12.3</v>
+        <v>19</v>
       </c>
       <c r="R13" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2:35</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1540,12 +1540,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1559,30 +1559,30 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="O14" t="n">
-        <v>48.7</v>
+        <v>48.8</v>
       </c>
       <c r="P14" t="n">
-        <v>48.7</v>
+        <v>48.8</v>
       </c>
       <c r="Q14" t="n">
-        <v>18.5</v>
+        <v>19</v>
       </c>
       <c r="R14" t="n">
-        <v>10.1</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2:40</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1597,17 +1597,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1622,12 +1622,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>33.8</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1641,35 +1641,35 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>15</v>
+        <v>121</v>
       </c>
       <c r="O15" t="n">
-        <v>53.3</v>
+        <v>48.8</v>
       </c>
       <c r="P15" t="n">
-        <v>33.3</v>
+        <v>48.8</v>
       </c>
       <c r="Q15" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="R15" t="n">
-        <v>0</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1679,17 +1679,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1699,17 +1699,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1723,35 +1723,35 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>65</v>
+        <v>121</v>
       </c>
       <c r="O16" t="n">
-        <v>50.8</v>
+        <v>48.8</v>
       </c>
       <c r="P16" t="n">
-        <v>44.6</v>
+        <v>48.8</v>
       </c>
       <c r="Q16" t="n">
-        <v>12.3</v>
+        <v>19</v>
       </c>
       <c r="R16" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1761,22 +1761,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1786,12 +1786,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1801,39 +1801,39 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>72</v>
+        <v>121</v>
       </c>
       <c r="O17" t="n">
-        <v>43.1</v>
+        <v>48.8</v>
       </c>
       <c r="P17" t="n">
-        <v>54.2</v>
+        <v>48.8</v>
       </c>
       <c r="Q17" t="n">
-        <v>16.7</v>
+        <v>19</v>
       </c>
       <c r="R17" t="n">
-        <v>11.1</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1843,12 +1843,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1868,12 +1868,12 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1887,19 +1887,19 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="O18" t="n">
-        <v>48.7</v>
+        <v>48.8</v>
       </c>
       <c r="P18" t="n">
-        <v>48.7</v>
+        <v>48.8</v>
       </c>
       <c r="Q18" t="n">
-        <v>18.5</v>
+        <v>19</v>
       </c>
       <c r="R18" t="n">
-        <v>10.1</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="19">
@@ -1925,12 +1925,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1950,12 +1950,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1969,75 +1969,75 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="O19" t="n">
-        <v>59.3</v>
+        <v>57.1</v>
       </c>
       <c r="P19" t="n">
-        <v>40.7</v>
+        <v>42.9</v>
       </c>
       <c r="Q19" t="n">
-        <v>18.5</v>
+        <v>17.9</v>
       </c>
       <c r="R19" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>7-4</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>39.3</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>51.6</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2047,79 +2047,79 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N20" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="O20" t="n">
-        <v>38.9</v>
+        <v>59.4</v>
       </c>
       <c r="P20" t="n">
-        <v>61.1</v>
+        <v>40.6</v>
       </c>
       <c r="Q20" t="n">
-        <v>22.2</v>
+        <v>15.6</v>
       </c>
       <c r="R20" t="n">
-        <v>14.8</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>9:10</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>7-4</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>51.6</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2129,39 +2129,39 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N21" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="O21" t="n">
-        <v>38.9</v>
+        <v>59.4</v>
       </c>
       <c r="P21" t="n">
-        <v>61.1</v>
+        <v>40.6</v>
       </c>
       <c r="Q21" t="n">
-        <v>22.2</v>
+        <v>15.6</v>
       </c>
       <c r="R21" t="n">
-        <v>14.8</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1:35</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2171,17 +2171,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>4-7</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2191,17 +2191,17 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>50.4</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2215,265 +2215,19 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="O22" t="n">
-        <v>50</v>
+        <v>52.4</v>
       </c>
       <c r="P22" t="n">
-        <v>48.1</v>
+        <v>47.6</v>
       </c>
       <c r="Q22" t="n">
-        <v>21.2</v>
+        <v>23.8</v>
       </c>
       <c r="R22" t="n">
-        <v>17.3</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2:35</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Atlanta Braves</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Texas Rangers</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>48.0</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>52.0</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>4-5</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>54.4</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>29.4</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N23" t="n">
-        <v>52</v>
-      </c>
-      <c r="O23" t="n">
-        <v>50</v>
-      </c>
-      <c r="P23" t="n">
-        <v>48.1</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>21.2</v>
-      </c>
-      <c r="R23" t="n">
-        <v>17.3</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>4:10</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Colorado Rockies</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Cincinnati Reds</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>31.0</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>69.0</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>4-8</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>95.4</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>80.9</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>59.8</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N24" t="n">
-        <v>9</v>
-      </c>
-      <c r="O24" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="P24" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>33.3</v>
-      </c>
-      <c r="R24" t="n">
-        <v>22.2</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>5:10</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Arizona Diamondbacks</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>St.Louis Cardinals</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>63.0</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>37.0</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>7-4</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>92.1</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>71.0</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>46.7</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N25" t="n">
-        <v>54</v>
-      </c>
-      <c r="O25" t="n">
-        <v>38.9</v>
-      </c>
-      <c r="P25" t="n">
-        <v>61.1</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>22.2</v>
-      </c>
-      <c r="R25" t="n">
-        <v>14.8</v>
+        <v>15.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-21 13:15
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R22"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,32 +511,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -556,12 +556,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -575,55 +575,55 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="O2" t="n">
-        <v>80</v>
+        <v>72.2</v>
       </c>
       <c r="P2" t="n">
-        <v>20</v>
+        <v>27.8</v>
       </c>
       <c r="Q2" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="R2" t="n">
-        <v>13.3</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,22 +633,22 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -657,75 +657,75 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="O3" t="n">
-        <v>80</v>
+        <v>61.1</v>
       </c>
       <c r="P3" t="n">
-        <v>20</v>
+        <v>38.9</v>
       </c>
       <c r="Q3" t="n">
-        <v>20</v>
+        <v>44.4</v>
       </c>
       <c r="R3" t="n">
-        <v>13.3</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>8:07</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,39 +735,39 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="O4" t="n">
-        <v>58.6</v>
+        <v>41.3</v>
       </c>
       <c r="P4" t="n">
-        <v>38.6</v>
+        <v>56</v>
       </c>
       <c r="Q4" t="n">
-        <v>24.3</v>
+        <v>44</v>
       </c>
       <c r="R4" t="n">
-        <v>17.1</v>
+        <v>26.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -802,12 +802,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,35 +821,35 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O5" t="n">
-        <v>58.6</v>
+        <v>57.7</v>
       </c>
       <c r="P5" t="n">
-        <v>38.6</v>
+        <v>39.4</v>
       </c>
       <c r="Q5" t="n">
-        <v>24.3</v>
+        <v>54.9</v>
       </c>
       <c r="R5" t="n">
-        <v>17.1</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,17 +859,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -879,17 +879,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -903,35 +903,35 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="O6" t="n">
-        <v>58.6</v>
+        <v>61.1</v>
       </c>
       <c r="P6" t="n">
-        <v>38.6</v>
+        <v>38.9</v>
       </c>
       <c r="Q6" t="n">
-        <v>24.3</v>
+        <v>44.4</v>
       </c>
       <c r="R6" t="n">
-        <v>17.1</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -941,17 +941,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,17 +961,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,55 +985,55 @@
         </is>
       </c>
       <c r="N7" t="n">
+        <v>71</v>
+      </c>
+      <c r="O7" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="P7" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="R7" t="n">
         <v>38</v>
-      </c>
-      <c r="O7" t="n">
-        <v>57.9</v>
-      </c>
-      <c r="P7" t="n">
-        <v>39.5</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="R7" t="n">
-        <v>5.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>6-7</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,17 +1043,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>97.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>80.9</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>59.8</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1067,55 +1067,55 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="O8" t="n">
-        <v>42.9</v>
+        <v>41.3</v>
       </c>
       <c r="P8" t="n">
-        <v>57.1</v>
+        <v>56</v>
       </c>
       <c r="Q8" t="n">
-        <v>39.3</v>
+        <v>44</v>
       </c>
       <c r="R8" t="n">
-        <v>32.1</v>
+        <v>26.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1125,22 +1125,22 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1149,35 +1149,35 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>121</v>
+        <v>82</v>
       </c>
       <c r="O9" t="n">
-        <v>48.8</v>
+        <v>59.8</v>
       </c>
       <c r="P9" t="n">
-        <v>48.8</v>
+        <v>40.2</v>
       </c>
       <c r="Q9" t="n">
-        <v>19</v>
+        <v>45.1</v>
       </c>
       <c r="R9" t="n">
-        <v>10.7</v>
+        <v>30.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1187,22 +1187,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>73.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1212,12 +1212,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1227,23 +1227,23 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>73</v>
+        <v>126</v>
       </c>
       <c r="O10" t="n">
-        <v>42.5</v>
+        <v>49.2</v>
       </c>
       <c r="P10" t="n">
-        <v>54.8</v>
+        <v>48.4</v>
       </c>
       <c r="Q10" t="n">
-        <v>16.4</v>
+        <v>45.2</v>
       </c>
       <c r="R10" t="n">
-        <v>11</v>
+        <v>29.4</v>
       </c>
     </row>
     <row r="11">
@@ -1254,12 +1254,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1289,17 +1289,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1313,50 +1313,50 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>439</v>
+        <v>16</v>
       </c>
       <c r="O11" t="n">
-        <v>51.7</v>
+        <v>50</v>
       </c>
       <c r="P11" t="n">
-        <v>45.6</v>
+        <v>37.5</v>
       </c>
       <c r="Q11" t="n">
-        <v>18.5</v>
+        <v>18.8</v>
       </c>
       <c r="R11" t="n">
-        <v>11.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1376,12 +1376,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1395,55 +1395,55 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="O12" t="n">
-        <v>48.8</v>
+        <v>49.2</v>
       </c>
       <c r="P12" t="n">
-        <v>48.8</v>
+        <v>48.4</v>
       </c>
       <c r="Q12" t="n">
-        <v>19</v>
+        <v>45.2</v>
       </c>
       <c r="R12" t="n">
-        <v>10.7</v>
+        <v>29.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1453,17 +1453,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>58.3</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,35 +1477,35 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>121</v>
+        <v>67</v>
       </c>
       <c r="O13" t="n">
-        <v>48.8</v>
+        <v>50.7</v>
       </c>
       <c r="P13" t="n">
-        <v>48.8</v>
+        <v>44.8</v>
       </c>
       <c r="Q13" t="n">
-        <v>19</v>
+        <v>53.7</v>
       </c>
       <c r="R13" t="n">
-        <v>10.7</v>
+        <v>35.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1515,17 +1515,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1535,17 +1535,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1559,35 +1559,35 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>121</v>
+        <v>67</v>
       </c>
       <c r="O14" t="n">
-        <v>48.8</v>
+        <v>50.7</v>
       </c>
       <c r="P14" t="n">
-        <v>48.8</v>
+        <v>44.8</v>
       </c>
       <c r="Q14" t="n">
-        <v>19</v>
+        <v>53.7</v>
       </c>
       <c r="R14" t="n">
-        <v>10.7</v>
+        <v>35.8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1597,17 +1597,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1617,17 +1617,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1641,35 +1641,35 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>121</v>
+        <v>67</v>
       </c>
       <c r="O15" t="n">
-        <v>48.8</v>
+        <v>50.7</v>
       </c>
       <c r="P15" t="n">
-        <v>48.8</v>
+        <v>44.8</v>
       </c>
       <c r="Q15" t="n">
-        <v>19</v>
+        <v>53.7</v>
       </c>
       <c r="R15" t="n">
-        <v>10.7</v>
+        <v>35.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>26.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1704,12 +1704,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1723,219 +1723,219 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="O16" t="n">
-        <v>48.8</v>
+        <v>49.2</v>
       </c>
       <c r="P16" t="n">
-        <v>48.8</v>
+        <v>48.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>19</v>
+        <v>45.2</v>
       </c>
       <c r="R16" t="n">
-        <v>10.7</v>
+        <v>29.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>121</v>
+        <v>29</v>
       </c>
       <c r="O17" t="n">
-        <v>48.8</v>
+        <v>58.6</v>
       </c>
       <c r="P17" t="n">
-        <v>48.8</v>
+        <v>41.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>19</v>
+        <v>24.1</v>
       </c>
       <c r="R17" t="n">
-        <v>10.7</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>53.0</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N18" t="n">
-        <v>121</v>
+        <v>54</v>
       </c>
       <c r="O18" t="n">
-        <v>48.8</v>
+        <v>50</v>
       </c>
       <c r="P18" t="n">
-        <v>48.8</v>
+        <v>48.1</v>
       </c>
       <c r="Q18" t="n">
-        <v>19</v>
+        <v>46.3</v>
       </c>
       <c r="R18" t="n">
-        <v>10.7</v>
+        <v>38.9</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>8:07</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1945,17 +1945,17 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1969,265 +1969,19 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="O19" t="n">
-        <v>57.1</v>
+        <v>50</v>
       </c>
       <c r="P19" t="n">
-        <v>42.9</v>
+        <v>48.1</v>
       </c>
       <c r="Q19" t="n">
-        <v>17.9</v>
+        <v>46.3</v>
       </c>
       <c r="R19" t="n">
-        <v>3.6</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>8:10</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Baltimore Orioles</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>49.0</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>51.0</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>4-6</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>87.0</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>39.3</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>17.4</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N20" t="n">
-        <v>32</v>
-      </c>
-      <c r="O20" t="n">
-        <v>59.4</v>
-      </c>
-      <c r="P20" t="n">
-        <v>40.6</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="R20" t="n">
-        <v>9.4</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>9:10</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Houston Astros</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Miami Marlins</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>4-6</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>87.0</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>40.7</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>18.4</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N21" t="n">
-        <v>32</v>
-      </c>
-      <c r="O21" t="n">
-        <v>59.4</v>
-      </c>
-      <c r="P21" t="n">
-        <v>40.6</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="R21" t="n">
-        <v>9.4</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>11:10</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Los Angeles Angels</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>St.Louis Cardinals</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>46.0</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>54.0</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>4-7</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>92.1</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>74.0</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>50.4</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N22" t="n">
-        <v>63</v>
-      </c>
-      <c r="O22" t="n">
-        <v>52.4</v>
-      </c>
-      <c r="P22" t="n">
-        <v>47.6</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="R22" t="n">
-        <v>15.9</v>
+        <v>38.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-22 15:21
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -556,12 +556,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>55.7</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>30.6</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -575,19 +575,19 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="O2" t="n">
-        <v>72.2</v>
+        <v>70</v>
       </c>
       <c r="P2" t="n">
-        <v>27.8</v>
+        <v>25</v>
       </c>
       <c r="Q2" t="n">
         <v>50</v>
       </c>
       <c r="R2" t="n">
-        <v>27.8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -598,12 +598,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -613,17 +613,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>39.3</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,75 +657,75 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="O3" t="n">
-        <v>61.1</v>
+        <v>58.1</v>
       </c>
       <c r="P3" t="n">
-        <v>38.9</v>
+        <v>39.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>44.4</v>
+        <v>52.7</v>
       </c>
       <c r="R3" t="n">
-        <v>30.6</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,39 +735,39 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>75</v>
+        <v>39</v>
       </c>
       <c r="O4" t="n">
-        <v>41.3</v>
+        <v>56.4</v>
       </c>
       <c r="P4" t="n">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="Q4" t="n">
-        <v>44</v>
+        <v>33.3</v>
       </c>
       <c r="R4" t="n">
-        <v>26.7</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -777,17 +777,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,55 +821,55 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O5" t="n">
-        <v>57.7</v>
+        <v>61.6</v>
       </c>
       <c r="P5" t="n">
-        <v>39.4</v>
+        <v>38.4</v>
       </c>
       <c r="Q5" t="n">
-        <v>54.9</v>
+        <v>43.8</v>
       </c>
       <c r="R5" t="n">
-        <v>38</v>
+        <v>30.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -879,17 +879,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>16.5</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -903,55 +903,55 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="O6" t="n">
-        <v>61.1</v>
+        <v>58.1</v>
       </c>
       <c r="P6" t="n">
-        <v>38.9</v>
+        <v>39.2</v>
       </c>
       <c r="Q6" t="n">
-        <v>44.4</v>
+        <v>52.7</v>
       </c>
       <c r="R6" t="n">
-        <v>30.6</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,17 +961,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,137 +985,137 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="O7" t="n">
-        <v>57.7</v>
+        <v>60.7</v>
       </c>
       <c r="P7" t="n">
-        <v>39.4</v>
+        <v>39.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>54.9</v>
+        <v>44</v>
       </c>
       <c r="R7" t="n">
-        <v>38</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>75</v>
+        <v>491</v>
       </c>
       <c r="O8" t="n">
-        <v>41.3</v>
+        <v>52.1</v>
       </c>
       <c r="P8" t="n">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="Q8" t="n">
-        <v>44</v>
+        <v>46.8</v>
       </c>
       <c r="R8" t="n">
-        <v>26.7</v>
+        <v>30.8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3-1</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1125,22 +1125,22 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1149,55 +1149,55 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>82</v>
+        <v>133</v>
       </c>
       <c r="O9" t="n">
-        <v>59.8</v>
+        <v>50.4</v>
       </c>
       <c r="P9" t="n">
-        <v>40.2</v>
+        <v>47.4</v>
       </c>
       <c r="Q9" t="n">
-        <v>45.1</v>
+        <v>46.6</v>
       </c>
       <c r="R9" t="n">
-        <v>30.5</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,17 +1207,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1231,55 +1231,55 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>126</v>
+        <v>68</v>
       </c>
       <c r="O10" t="n">
-        <v>49.2</v>
+        <v>51.5</v>
       </c>
       <c r="P10" t="n">
-        <v>48.4</v>
+        <v>44.1</v>
       </c>
       <c r="Q10" t="n">
-        <v>45.2</v>
+        <v>52.9</v>
       </c>
       <c r="R10" t="n">
-        <v>29.4</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>72.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>28.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1294,12 +1294,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1313,50 +1313,50 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>16</v>
+        <v>133</v>
       </c>
       <c r="O11" t="n">
-        <v>50</v>
+        <v>50.4</v>
       </c>
       <c r="P11" t="n">
-        <v>37.5</v>
+        <v>47.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>18.8</v>
+        <v>46.6</v>
       </c>
       <c r="R11" t="n">
-        <v>18.8</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1376,12 +1376,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1395,40 +1395,40 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="O12" t="n">
-        <v>49.2</v>
+        <v>50.4</v>
       </c>
       <c r="P12" t="n">
-        <v>48.4</v>
+        <v>47.4</v>
       </c>
       <c r="Q12" t="n">
-        <v>45.2</v>
+        <v>46.6</v>
       </c>
       <c r="R12" t="n">
-        <v>29.4</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>4:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1453,17 +1453,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>58.3</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,35 +1477,35 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>67</v>
+        <v>133</v>
       </c>
       <c r="O13" t="n">
-        <v>50.7</v>
+        <v>50.4</v>
       </c>
       <c r="P13" t="n">
-        <v>44.8</v>
+        <v>47.4</v>
       </c>
       <c r="Q13" t="n">
-        <v>53.7</v>
+        <v>46.6</v>
       </c>
       <c r="R13" t="n">
-        <v>35.8</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1515,17 +1515,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1535,17 +1535,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1559,35 +1559,35 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>67</v>
+        <v>133</v>
       </c>
       <c r="O14" t="n">
-        <v>50.7</v>
+        <v>50.4</v>
       </c>
       <c r="P14" t="n">
-        <v>44.8</v>
+        <v>47.4</v>
       </c>
       <c r="Q14" t="n">
-        <v>53.7</v>
+        <v>46.6</v>
       </c>
       <c r="R14" t="n">
-        <v>35.8</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1597,12 +1597,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1622,12 +1622,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1641,35 +1641,35 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="O15" t="n">
-        <v>50.7</v>
+        <v>51.5</v>
       </c>
       <c r="P15" t="n">
-        <v>44.8</v>
+        <v>44.1</v>
       </c>
       <c r="Q15" t="n">
-        <v>53.7</v>
+        <v>52.9</v>
       </c>
       <c r="R15" t="n">
-        <v>35.8</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>8:07</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1679,17 +1679,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1699,17 +1699,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1723,137 +1723,137 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>126</v>
+        <v>68</v>
       </c>
       <c r="O16" t="n">
-        <v>49.2</v>
+        <v>51.5</v>
       </c>
       <c r="P16" t="n">
-        <v>48.4</v>
+        <v>44.1</v>
       </c>
       <c r="Q16" t="n">
-        <v>45.2</v>
+        <v>52.9</v>
       </c>
       <c r="R16" t="n">
-        <v>29.4</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>29</v>
+        <v>133</v>
       </c>
       <c r="O17" t="n">
-        <v>58.6</v>
+        <v>50.4</v>
       </c>
       <c r="P17" t="n">
-        <v>41.4</v>
+        <v>47.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>24.1</v>
+        <v>46.6</v>
       </c>
       <c r="R17" t="n">
-        <v>10.3</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1863,17 +1863,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>31.8</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1887,101 +1887,839 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="O18" t="n">
-        <v>50</v>
+        <v>56.7</v>
       </c>
       <c r="P18" t="n">
-        <v>48.1</v>
+        <v>43.3</v>
       </c>
       <c r="Q18" t="n">
-        <v>46.3</v>
+        <v>26.7</v>
       </c>
       <c r="R18" t="n">
-        <v>38.9</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>8:07</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>9.7</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>30</v>
+      </c>
+      <c r="O19" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="P19" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="R19" t="n">
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>SSG Landers</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>46.3</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>22.6</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>39</v>
+      </c>
+      <c r="O20" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="P20" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>59</v>
+      </c>
+      <c r="R20" t="n">
+        <v>35.9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>NC Dinos</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>47.7</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>23.7</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>39</v>
+      </c>
+      <c r="O21" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="P21" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>59</v>
+      </c>
+      <c r="R21" t="n">
+        <v>35.9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>KIA Tigers</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Hanwha Eagles</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>47.7</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>23.7</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>39</v>
+      </c>
+      <c r="O22" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="P22" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>59</v>
+      </c>
+      <c r="R22" t="n">
+        <v>35.9</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Kiwoom Heroes</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>3-6</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>55.7</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>30.6</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>13</v>
+      </c>
+      <c r="O23" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="P23" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="R23" t="n">
+        <v>38.5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>5:07</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
           <t>MLB</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>34</v>
+      </c>
+      <c r="O24" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="P24" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>50</v>
+      </c>
+      <c r="R24" t="n">
+        <v>32.4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>43.5</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>29</v>
+      </c>
+      <c r="O25" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="P25" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="R25" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7-6</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>97.4</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>80.2</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>58.7</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>22</v>
+      </c>
+      <c r="O26" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="P26" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="R26" t="n">
+        <v>36.4</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>7-6</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>97.4</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>85.1</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>66.3</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>22</v>
+      </c>
+      <c r="O27" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="P27" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="R27" t="n">
+        <v>36.4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Chinatrust Brothers</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
         <is>
           <t>4-5</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>79.3</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>51.8</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>27.1</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>36.6</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>원정승</t>
         </is>
       </c>
-      <c r="N19" t="n">
-        <v>54</v>
-      </c>
-      <c r="O19" t="n">
-        <v>50</v>
-      </c>
-      <c r="P19" t="n">
-        <v>48.1</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>46.3</v>
-      </c>
-      <c r="R19" t="n">
-        <v>38.9</v>
+      <c r="N28" t="n">
+        <v>55</v>
+      </c>
+      <c r="O28" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="P28" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="R28" t="n">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-24 15:30
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -511,57 +511,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,23 +571,23 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="O2" t="n">
-        <v>71.40000000000001</v>
+        <v>26.7</v>
       </c>
       <c r="P2" t="n">
-        <v>23.8</v>
+        <v>73.3</v>
       </c>
       <c r="Q2" t="n">
-        <v>52.4</v>
+        <v>30</v>
       </c>
       <c r="R2" t="n">
-        <v>33.3</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="3">
@@ -598,12 +598,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -613,17 +613,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,75 +657,75 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="O3" t="n">
-        <v>57.7</v>
+        <v>60.8</v>
       </c>
       <c r="P3" t="n">
-        <v>39.7</v>
+        <v>39.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>51.3</v>
+        <v>44.6</v>
       </c>
       <c r="R3" t="n">
-        <v>35.9</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,23 +735,23 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="O4" t="n">
-        <v>41.6</v>
+        <v>60.9</v>
       </c>
       <c r="P4" t="n">
-        <v>55.8</v>
+        <v>39.1</v>
       </c>
       <c r="Q4" t="n">
-        <v>45.5</v>
+        <v>44.8</v>
       </c>
       <c r="R4" t="n">
-        <v>27.3</v>
+        <v>29.9</v>
       </c>
     </row>
     <row r="5">
@@ -762,12 +762,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>45.4</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,55 +821,55 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>77</v>
+        <v>22</v>
       </c>
       <c r="O5" t="n">
-        <v>41.6</v>
+        <v>40.9</v>
       </c>
       <c r="P5" t="n">
-        <v>55.8</v>
+        <v>59.1</v>
       </c>
       <c r="Q5" t="n">
-        <v>45.5</v>
+        <v>68.2</v>
       </c>
       <c r="R5" t="n">
-        <v>27.3</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -879,22 +879,22 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>47.7</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>23.7</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -903,40 +903,40 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="O6" t="n">
-        <v>47.1</v>
+        <v>57.7</v>
       </c>
       <c r="P6" t="n">
-        <v>41.2</v>
+        <v>39.7</v>
       </c>
       <c r="Q6" t="n">
-        <v>17.6</v>
+        <v>51.3</v>
       </c>
       <c r="R6" t="n">
-        <v>17.6</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2:10</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,22 +961,22 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>14.3</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -985,137 +985,137 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>135</v>
+        <v>40</v>
       </c>
       <c r="O7" t="n">
-        <v>49.6</v>
+        <v>57.5</v>
       </c>
       <c r="P7" t="n">
-        <v>48.1</v>
+        <v>40</v>
       </c>
       <c r="Q7" t="n">
-        <v>45.9</v>
+        <v>35</v>
       </c>
       <c r="R7" t="n">
-        <v>31.1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6:15</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>56.0</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>44.0</t>
-        </is>
-      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>2-6</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>16.5</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>135</v>
+        <v>29</v>
       </c>
       <c r="O8" t="n">
-        <v>49.6</v>
+        <v>37.9</v>
       </c>
       <c r="P8" t="n">
-        <v>48.1</v>
+        <v>58.6</v>
       </c>
       <c r="Q8" t="n">
-        <v>45.9</v>
+        <v>55.2</v>
       </c>
       <c r="R8" t="n">
-        <v>31.1</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1130,12 +1130,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1149,19 +1149,19 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>17</v>
+        <v>135</v>
       </c>
       <c r="O9" t="n">
-        <v>47.1</v>
+        <v>49.6</v>
       </c>
       <c r="P9" t="n">
-        <v>41.2</v>
+        <v>48.1</v>
       </c>
       <c r="Q9" t="n">
-        <v>17.6</v>
+        <v>45.9</v>
       </c>
       <c r="R9" t="n">
-        <v>17.6</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="10">
@@ -1172,12 +1172,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1212,12 +1212,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1289,17 +1289,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1313,19 +1313,19 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="O11" t="n">
-        <v>48.8</v>
+        <v>59.4</v>
       </c>
       <c r="P11" t="n">
-        <v>48.8</v>
+        <v>40.6</v>
       </c>
       <c r="Q11" t="n">
-        <v>61</v>
+        <v>28.1</v>
       </c>
       <c r="R11" t="n">
-        <v>34.1</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="12">
@@ -1336,12 +1336,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1351,12 +1351,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1376,12 +1376,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1413,57 +1413,57 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1:15</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>80.9</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>59.8</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1473,59 +1473,59 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="O13" t="n">
-        <v>48.8</v>
+        <v>44.4</v>
       </c>
       <c r="P13" t="n">
-        <v>48.8</v>
+        <v>55.6</v>
       </c>
       <c r="Q13" t="n">
-        <v>61</v>
+        <v>61.1</v>
       </c>
       <c r="R13" t="n">
-        <v>34.1</v>
+        <v>38.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4:07</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1535,17 +1535,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1559,19 +1559,19 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="O14" t="n">
-        <v>61.8</v>
+        <v>49.1</v>
       </c>
       <c r="P14" t="n">
-        <v>38.2</v>
+        <v>49.1</v>
       </c>
       <c r="Q14" t="n">
-        <v>50</v>
+        <v>49.1</v>
       </c>
       <c r="R14" t="n">
-        <v>32.4</v>
+        <v>42.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-24 22:57
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -921,57 +921,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -981,64 +981,64 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>40</v>
+        <v>77</v>
       </c>
       <c r="O7" t="n">
-        <v>57.5</v>
+        <v>41.6</v>
       </c>
       <c r="P7" t="n">
-        <v>40</v>
+        <v>55.8</v>
       </c>
       <c r="Q7" t="n">
-        <v>35</v>
+        <v>45.5</v>
       </c>
       <c r="R7" t="n">
-        <v>15</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2-6</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>16.5</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1063,59 +1063,59 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>29</v>
+        <v>78</v>
       </c>
       <c r="O8" t="n">
-        <v>37.9</v>
+        <v>57.7</v>
       </c>
       <c r="P8" t="n">
-        <v>58.6</v>
+        <v>39.7</v>
       </c>
       <c r="Q8" t="n">
-        <v>55.2</v>
+        <v>51.3</v>
       </c>
       <c r="R8" t="n">
-        <v>31</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1125,22 +1125,22 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1149,55 +1149,55 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>135</v>
+        <v>78</v>
       </c>
       <c r="O9" t="n">
-        <v>49.6</v>
+        <v>57.7</v>
       </c>
       <c r="P9" t="n">
-        <v>48.1</v>
+        <v>39.7</v>
       </c>
       <c r="Q9" t="n">
-        <v>45.9</v>
+        <v>51.3</v>
       </c>
       <c r="R9" t="n">
-        <v>31.1</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>9:15</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,22 +1207,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1231,137 +1231,137 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>135</v>
+        <v>78</v>
       </c>
       <c r="O10" t="n">
-        <v>49.6</v>
+        <v>57.7</v>
       </c>
       <c r="P10" t="n">
-        <v>48.1</v>
+        <v>39.7</v>
       </c>
       <c r="Q10" t="n">
-        <v>45.9</v>
+        <v>51.3</v>
       </c>
       <c r="R10" t="n">
-        <v>31.1</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>14.3</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="O11" t="n">
-        <v>59.4</v>
+        <v>57.5</v>
       </c>
       <c r="P11" t="n">
-        <v>40.6</v>
+        <v>40</v>
       </c>
       <c r="Q11" t="n">
-        <v>28.1</v>
+        <v>35</v>
       </c>
       <c r="R11" t="n">
-        <v>15.6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>2-6</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1371,22 +1371,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>16.5</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1395,55 +1395,55 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="O12" t="n">
-        <v>49.1</v>
+        <v>37.9</v>
       </c>
       <c r="P12" t="n">
-        <v>49.1</v>
+        <v>58.6</v>
       </c>
       <c r="Q12" t="n">
-        <v>49.1</v>
+        <v>55.2</v>
       </c>
       <c r="R12" t="n">
-        <v>42.1</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1453,22 +1453,22 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>80.9</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>59.8</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1477,101 +1477,1249 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>18</v>
+        <v>135</v>
       </c>
       <c r="O13" t="n">
-        <v>44.4</v>
+        <v>49.6</v>
       </c>
       <c r="P13" t="n">
-        <v>55.6</v>
+        <v>48.1</v>
       </c>
       <c r="Q13" t="n">
-        <v>61.1</v>
+        <v>45.9</v>
       </c>
       <c r="R13" t="n">
-        <v>38.9</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>69.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>31.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>135</v>
+      </c>
+      <c r="O14" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P14" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R14" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>135</v>
+      </c>
+      <c r="O15" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P15" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R15" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>68</v>
+      </c>
+      <c r="O16" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="P16" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R16" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>51.8</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>68</v>
+      </c>
+      <c r="O17" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="P17" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R17" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>24.5</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>135</v>
+      </c>
+      <c r="O18" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P18" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R18" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Seibu Lions</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Fukuoka S. Hawks</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>32</v>
+      </c>
+      <c r="O19" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="P19" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="R19" t="n">
+        <v>15.6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>KT Wiz Suwon</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>57</v>
+      </c>
+      <c r="O20" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="P20" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="R20" t="n">
+        <v>42.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>KIA Tigers</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Kiwoom Heroes</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>7-5</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>80.9</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>59.8</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>18</v>
+      </c>
+      <c r="O21" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="P21" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="R21" t="n">
+        <v>38.9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>Doosan Bears</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Samsung Lions</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>KBO</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>42.0</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>58.0</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>4-5</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>79.3</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>54.4</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>29.4</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>원정승</t>
         </is>
       </c>
-      <c r="N14" t="n">
+      <c r="N22" t="n">
         <v>57</v>
       </c>
-      <c r="O14" t="n">
+      <c r="O22" t="n">
         <v>49.1</v>
       </c>
-      <c r="P14" t="n">
+      <c r="P22" t="n">
         <v>49.1</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="Q22" t="n">
         <v>49.1</v>
       </c>
-      <c r="R14" t="n">
+      <c r="R22" t="n">
         <v>42.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>3-7</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>63.2</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>37.9</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>22</v>
+      </c>
+      <c r="O23" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="P23" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>50</v>
+      </c>
+      <c r="R23" t="n">
+        <v>31.8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>43.5</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>41</v>
+      </c>
+      <c r="O24" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="P24" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>61</v>
+      </c>
+      <c r="R24" t="n">
+        <v>34.1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>44.9</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>21.5</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>29</v>
+      </c>
+      <c r="O25" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="P25" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="R25" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>8:05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>3-6</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>53.1</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>28.2</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>14</v>
+      </c>
+      <c r="O26" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="P26" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>50</v>
+      </c>
+      <c r="R26" t="n">
+        <v>35.7</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>41</v>
+      </c>
+      <c r="O27" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="P27" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>61</v>
+      </c>
+      <c r="R27" t="n">
+        <v>34.1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>32</v>
+      </c>
+      <c r="O28" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="P28" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="R28" t="n">
+        <v>15.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-26 13:09
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,17 +511,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,22 +531,22 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -556,156 +556,156 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O2" t="n">
-        <v>57.5</v>
+        <v>26.7</v>
       </c>
       <c r="P2" t="n">
-        <v>40</v>
+        <v>73.3</v>
       </c>
       <c r="Q2" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="R2" t="n">
-        <v>15</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>74</v>
+        <v>30</v>
       </c>
       <c r="O3" t="n">
-        <v>60.8</v>
+        <v>26.7</v>
       </c>
       <c r="P3" t="n">
-        <v>39.2</v>
+        <v>73.3</v>
       </c>
       <c r="Q3" t="n">
-        <v>44.6</v>
+        <v>30</v>
       </c>
       <c r="R3" t="n">
-        <v>31.1</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,22 +715,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -739,35 +739,35 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="O4" t="n">
-        <v>41.6</v>
+        <v>26.7</v>
       </c>
       <c r="P4" t="n">
-        <v>55.8</v>
+        <v>73.3</v>
       </c>
       <c r="Q4" t="n">
-        <v>45.5</v>
+        <v>30</v>
       </c>
       <c r="R4" t="n">
-        <v>27.3</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -777,17 +777,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>73.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,75 +821,75 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="O5" t="n">
-        <v>57.7</v>
+        <v>60.9</v>
       </c>
       <c r="P5" t="n">
-        <v>39.7</v>
+        <v>39.1</v>
       </c>
       <c r="Q5" t="n">
-        <v>51.3</v>
+        <v>44.8</v>
       </c>
       <c r="R5" t="n">
-        <v>35.9</v>
+        <v>29.9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>47.7</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>23.7</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,23 +899,23 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O6" t="n">
-        <v>57.7</v>
+        <v>41.6</v>
       </c>
       <c r="P6" t="n">
-        <v>39.7</v>
+        <v>55.8</v>
       </c>
       <c r="Q6" t="n">
-        <v>51.3</v>
+        <v>45.5</v>
       </c>
       <c r="R6" t="n">
-        <v>35.9</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="7">
@@ -926,32 +926,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6-5</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,17 +961,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>77.7</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>55.2</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,55 +985,55 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>17</v>
+        <v>74</v>
       </c>
       <c r="O7" t="n">
-        <v>58.8</v>
+        <v>60.8</v>
       </c>
       <c r="P7" t="n">
-        <v>35.3</v>
+        <v>39.2</v>
       </c>
       <c r="Q7" t="n">
-        <v>35.3</v>
+        <v>44.6</v>
       </c>
       <c r="R7" t="n">
-        <v>35.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2-6</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,17 +1043,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>16.5</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1067,55 +1067,55 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="O8" t="n">
-        <v>37.9</v>
+        <v>41.6</v>
       </c>
       <c r="P8" t="n">
-        <v>58.6</v>
+        <v>55.8</v>
       </c>
       <c r="Q8" t="n">
-        <v>55.2</v>
+        <v>45.5</v>
       </c>
       <c r="R8" t="n">
-        <v>31</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>6-5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1125,17 +1125,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1149,55 +1149,55 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="O9" t="n">
-        <v>57.5</v>
+        <v>58.8</v>
       </c>
       <c r="P9" t="n">
-        <v>40</v>
+        <v>35.3</v>
       </c>
       <c r="Q9" t="n">
-        <v>35</v>
+        <v>35.3</v>
       </c>
       <c r="R9" t="n">
-        <v>15</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>7-3</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,22 +1207,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>68.9</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>44.2</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1231,35 +1231,35 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>135</v>
+        <v>36</v>
       </c>
       <c r="O10" t="n">
-        <v>49.6</v>
+        <v>58.3</v>
       </c>
       <c r="P10" t="n">
-        <v>48.1</v>
+        <v>36.1</v>
       </c>
       <c r="Q10" t="n">
-        <v>45.9</v>
+        <v>63.9</v>
       </c>
       <c r="R10" t="n">
-        <v>31.1</v>
+        <v>47.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>2:40</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1269,22 +1269,22 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1294,74 +1294,74 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>135</v>
+        <v>77</v>
       </c>
       <c r="O11" t="n">
-        <v>49.6</v>
+        <v>41.6</v>
       </c>
       <c r="P11" t="n">
-        <v>48.1</v>
+        <v>55.8</v>
       </c>
       <c r="Q11" t="n">
-        <v>45.9</v>
+        <v>45.5</v>
       </c>
       <c r="R11" t="n">
-        <v>31.1</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1371,22 +1371,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1395,55 +1395,55 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>135</v>
+        <v>78</v>
       </c>
       <c r="O12" t="n">
-        <v>49.6</v>
+        <v>57.7</v>
       </c>
       <c r="P12" t="n">
-        <v>48.1</v>
+        <v>39.7</v>
       </c>
       <c r="Q12" t="n">
-        <v>45.9</v>
+        <v>51.3</v>
       </c>
       <c r="R12" t="n">
-        <v>31.1</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1453,22 +1453,22 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1477,137 +1477,137 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>32</v>
+        <v>77</v>
       </c>
       <c r="O13" t="n">
-        <v>59.4</v>
+        <v>41.6</v>
       </c>
       <c r="P13" t="n">
-        <v>40.6</v>
+        <v>55.8</v>
       </c>
       <c r="Q13" t="n">
-        <v>28.1</v>
+        <v>45.5</v>
       </c>
       <c r="R13" t="n">
-        <v>15.6</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>3:35</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>55.7</t>
+          <t>13.3</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>30.6</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="O14" t="n">
-        <v>49.1</v>
+        <v>60.8</v>
       </c>
       <c r="P14" t="n">
-        <v>49.1</v>
+        <v>39.2</v>
       </c>
       <c r="Q14" t="n">
-        <v>49.1</v>
+        <v>44.6</v>
       </c>
       <c r="R14" t="n">
-        <v>42.1</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>5:05</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1617,22 +1617,22 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>80.9</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>59.8</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1641,101 +1641,1003 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>18</v>
+        <v>78</v>
       </c>
       <c r="O15" t="n">
-        <v>44.4</v>
+        <v>57.7</v>
       </c>
       <c r="P15" t="n">
-        <v>55.6</v>
+        <v>39.7</v>
       </c>
       <c r="Q15" t="n">
-        <v>61.1</v>
+        <v>51.3</v>
       </c>
       <c r="R15" t="n">
-        <v>38.9</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Nippon Ham Fighters</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Rakuten Gold. Eagles</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>61.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>39.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>135</v>
+      </c>
+      <c r="O16" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P16" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R16" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2:35</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>135</v>
+      </c>
+      <c r="O17" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P17" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R17" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2:35</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>32.4</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>12.9</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>135</v>
+      </c>
+      <c r="O18" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P18" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R18" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2:40</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>135</v>
+      </c>
+      <c r="O19" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P19" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R19" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2:40</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>67.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>33.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>28.4</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>10.6</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>135</v>
+      </c>
+      <c r="O20" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P20" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R20" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>3:10</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>28.4</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>10.6</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>135</v>
+      </c>
+      <c r="O21" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P21" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R21" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>3:15</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>68</v>
+      </c>
+      <c r="O22" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="P22" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R22" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>16.3</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>135</v>
+      </c>
+      <c r="O23" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P23" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R23" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>24.5</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>17</v>
+      </c>
+      <c r="O24" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="P24" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="R24" t="n">
+        <v>17.6</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Lotte Giants</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>KT Wiz Suwon</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Yakult Swallows</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Hiroshima Carp</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>33.8</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>13.8</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>29</v>
+      </c>
+      <c r="O25" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="P25" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="R25" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>KIA Tigers</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Kiwoom Heroes</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
         <is>
           <t>KBO</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>41.0</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>59.0</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>4-6</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7-6</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>97.4</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>86.4</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>68.3</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>22</v>
+      </c>
+      <c r="O26" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="P26" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="R26" t="n">
+        <v>36.4</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>64.0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>87.0</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>42.1</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>19.4</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>원정승</t>
         </is>
       </c>
-      <c r="N16" t="n">
-        <v>34</v>
-      </c>
-      <c r="O16" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="P16" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>50</v>
-      </c>
-      <c r="R16" t="n">
-        <v>32.4</v>
+      <c r="N27" t="n">
+        <v>57</v>
+      </c>
+      <c r="O27" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="P27" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="R27" t="n">
+        <v>42.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-28 15:58
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:R21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -757,57 +757,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -817,223 +817,223 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="O5" t="n">
-        <v>60.8</v>
+        <v>41.6</v>
       </c>
       <c r="P5" t="n">
-        <v>39.2</v>
+        <v>55.8</v>
       </c>
       <c r="Q5" t="n">
-        <v>44.6</v>
+        <v>45.5</v>
       </c>
       <c r="R5" t="n">
-        <v>31.1</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>10:38</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>55.7</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>30.6</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="O6" t="n">
-        <v>51.5</v>
+        <v>41.6</v>
       </c>
       <c r="P6" t="n">
-        <v>44.1</v>
+        <v>55.8</v>
       </c>
       <c r="Q6" t="n">
-        <v>52.9</v>
+        <v>45.5</v>
       </c>
       <c r="R6" t="n">
-        <v>35.3</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="O7" t="n">
-        <v>51.5</v>
+        <v>41.6</v>
       </c>
       <c r="P7" t="n">
-        <v>44.1</v>
+        <v>55.8</v>
       </c>
       <c r="Q7" t="n">
-        <v>52.9</v>
+        <v>45.5</v>
       </c>
       <c r="R7" t="n">
-        <v>35.3</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1067,19 +1067,19 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="O8" t="n">
-        <v>41.4</v>
+        <v>60.8</v>
       </c>
       <c r="P8" t="n">
-        <v>58.6</v>
+        <v>39.2</v>
       </c>
       <c r="Q8" t="n">
-        <v>51.7</v>
+        <v>44.6</v>
       </c>
       <c r="R8" t="n">
-        <v>34.5</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="9">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1105,89 +1105,89 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>65.6</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>40.4</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="O9" t="n">
-        <v>61.8</v>
+        <v>51.5</v>
       </c>
       <c r="P9" t="n">
-        <v>38.2</v>
+        <v>44.1</v>
       </c>
       <c r="Q9" t="n">
-        <v>50</v>
+        <v>52.9</v>
       </c>
       <c r="R9" t="n">
-        <v>32.4</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,22 +1207,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>67.8</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>42.9</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1231,101 +1231,921 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="O10" t="n">
-        <v>44.4</v>
+        <v>51.5</v>
       </c>
       <c r="P10" t="n">
-        <v>55.6</v>
+        <v>44.1</v>
       </c>
       <c r="Q10" t="n">
-        <v>61.1</v>
+        <v>52.9</v>
       </c>
       <c r="R10" t="n">
-        <v>38.9</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>39.3</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>68</v>
+      </c>
+      <c r="O11" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="P11" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R11" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>31.1</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>135</v>
+      </c>
+      <c r="O12" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P12" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R12" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>50.4</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>25.9</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>68</v>
+      </c>
+      <c r="O13" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="P13" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R13" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Hanwha Eagles</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>43.5</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>29</v>
+      </c>
+      <c r="O14" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="P14" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="R14" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NC Dinos</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>KT Wiz Suwon</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>37.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>65.6</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>40.4</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>34</v>
+      </c>
+      <c r="O15" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="P15" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>50</v>
+      </c>
+      <c r="R15" t="n">
+        <v>32.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>KIA Tigers</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>7-5</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>67.8</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>42.9</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>18</v>
+      </c>
+      <c r="O16" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="P16" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="R16" t="n">
+        <v>38.9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>12.3</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>32</v>
+      </c>
+      <c r="O17" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="P17" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="R17" t="n">
+        <v>15.6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>65.6</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>40.4</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>34</v>
+      </c>
+      <c r="O18" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="P18" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>50</v>
+      </c>
+      <c r="R18" t="n">
+        <v>32.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>8:40</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Minnesota Twins</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Kansas City Royals</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>MLB</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>44.0</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>56.0</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>3-5</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>68.7</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>20.8</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>6.7</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>원정승</t>
         </is>
       </c>
-      <c r="N11" t="n">
+      <c r="N19" t="n">
         <v>41</v>
       </c>
-      <c r="O11" t="n">
+      <c r="O19" t="n">
         <v>48.8</v>
       </c>
-      <c r="P11" t="n">
+      <c r="P19" t="n">
         <v>48.8</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="Q19" t="n">
         <v>61</v>
       </c>
-      <c r="R11" t="n">
+      <c r="R19" t="n">
         <v>34.1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>8:45</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>36.7</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>34</v>
+      </c>
+      <c r="O20" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="P20" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>50</v>
+      </c>
+      <c r="R20" t="n">
+        <v>32.4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>63.2</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>37.9</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>34</v>
+      </c>
+      <c r="O21" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="P21" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>50</v>
+      </c>
+      <c r="R21" t="n">
+        <v>32.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-29 14:38
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:R17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,17 +511,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,37 +531,37 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>82.0</t>
+          <t>24.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>76.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7-2</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,23 +571,23 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="O2" t="n">
-        <v>69.7</v>
+        <v>26.7</v>
       </c>
       <c r="P2" t="n">
-        <v>30.3</v>
+        <v>73.3</v>
       </c>
       <c r="Q2" t="n">
-        <v>57.6</v>
+        <v>30</v>
       </c>
       <c r="R2" t="n">
-        <v>51.5</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="3">
@@ -598,27 +598,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Central league</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Pacific league</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -638,12 +638,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -680,12 +680,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,37 +695,37 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>6-5</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>23.3</t>
+          <t>67.8</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>7.9</t>
+          <t>42.9</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,79 +735,79 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="O4" t="n">
-        <v>41.6</v>
+        <v>58.8</v>
       </c>
       <c r="P4" t="n">
-        <v>55.8</v>
+        <v>35.3</v>
       </c>
       <c r="Q4" t="n">
-        <v>45.5</v>
+        <v>35.3</v>
       </c>
       <c r="R4" t="n">
-        <v>27.3</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -817,39 +817,39 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>77</v>
+        <v>40</v>
       </c>
       <c r="O5" t="n">
-        <v>41.6</v>
+        <v>57.5</v>
       </c>
       <c r="P5" t="n">
-        <v>55.8</v>
+        <v>40</v>
       </c>
       <c r="Q5" t="n">
-        <v>45.5</v>
+        <v>35</v>
       </c>
       <c r="R5" t="n">
-        <v>27.3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>10:38</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,37 +859,37 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>46.0</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>54.0</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,79 +899,79 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O6" t="n">
-        <v>41.6</v>
+        <v>57.7</v>
       </c>
       <c r="P6" t="n">
-        <v>55.8</v>
+        <v>39.7</v>
       </c>
       <c r="Q6" t="n">
-        <v>45.5</v>
+        <v>51.3</v>
       </c>
       <c r="R6" t="n">
-        <v>27.3</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>39.3</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -981,23 +981,23 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O7" t="n">
-        <v>41.6</v>
+        <v>57.7</v>
       </c>
       <c r="P7" t="n">
-        <v>55.8</v>
+        <v>39.7</v>
       </c>
       <c r="Q7" t="n">
-        <v>45.5</v>
+        <v>51.3</v>
       </c>
       <c r="R7" t="n">
-        <v>27.3</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="8">
@@ -1008,12 +1008,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1023,37 +1023,37 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1063,59 +1063,59 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="O8" t="n">
-        <v>60.8</v>
+        <v>41.6</v>
       </c>
       <c r="P8" t="n">
-        <v>39.2</v>
+        <v>55.8</v>
       </c>
       <c r="Q8" t="n">
-        <v>44.6</v>
+        <v>45.5</v>
       </c>
       <c r="R8" t="n">
-        <v>31.1</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1125,22 +1125,22 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>55.7</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>30.6</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1149,55 +1149,55 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="O9" t="n">
-        <v>51.5</v>
+        <v>60.8</v>
       </c>
       <c r="P9" t="n">
-        <v>44.1</v>
+        <v>39.2</v>
       </c>
       <c r="Q9" t="n">
-        <v>52.9</v>
+        <v>44.6</v>
       </c>
       <c r="R9" t="n">
-        <v>35.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Pacific league</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Central league</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>79.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>21.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,17 +1207,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1231,50 +1231,50 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="O10" t="n">
-        <v>51.5</v>
+        <v>47.1</v>
       </c>
       <c r="P10" t="n">
-        <v>44.1</v>
+        <v>41.2</v>
       </c>
       <c r="Q10" t="n">
-        <v>52.9</v>
+        <v>17.6</v>
       </c>
       <c r="R10" t="n">
-        <v>35.3</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1294,12 +1294,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1331,17 +1331,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1351,12 +1351,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1376,12 +1376,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1413,139 +1413,139 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>64.4</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>39.2</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="O13" t="n">
-        <v>51.5</v>
+        <v>61.8</v>
       </c>
       <c r="P13" t="n">
-        <v>44.1</v>
+        <v>38.2</v>
       </c>
       <c r="Q13" t="n">
-        <v>52.9</v>
+        <v>50</v>
       </c>
       <c r="R13" t="n">
-        <v>35.3</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>1:35</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>54.4</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1555,54 +1555,54 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="O14" t="n">
-        <v>41.4</v>
+        <v>49.1</v>
       </c>
       <c r="P14" t="n">
-        <v>58.6</v>
+        <v>49.1</v>
       </c>
       <c r="Q14" t="n">
-        <v>51.7</v>
+        <v>49.1</v>
       </c>
       <c r="R14" t="n">
-        <v>34.5</v>
+        <v>42.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1659,57 +1659,57 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>8:45</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>67.8</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>42.9</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1719,39 +1719,39 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N16" t="n">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>44.4</v>
+        <v>48.8</v>
       </c>
       <c r="P16" t="n">
-        <v>55.6</v>
+        <v>48.8</v>
       </c>
       <c r="Q16" t="n">
-        <v>61.1</v>
+        <v>61</v>
       </c>
       <c r="R16" t="n">
-        <v>38.9</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1761,17 +1761,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>4-7</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1781,17 +1781,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>73.1</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>49.2</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1805,347 +1805,19 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>32</v>
+        <v>67</v>
       </c>
       <c r="O17" t="n">
-        <v>59.4</v>
+        <v>53.7</v>
       </c>
       <c r="P17" t="n">
-        <v>40.6</v>
+        <v>46.3</v>
       </c>
       <c r="Q17" t="n">
-        <v>28.1</v>
+        <v>58.2</v>
       </c>
       <c r="R17" t="n">
-        <v>15.6</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>8:10</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>New York Mets</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Atlanta Braves</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>48.0</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>52.0</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>4-6</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>87.0</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>65.6</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>40.4</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N18" t="n">
-        <v>34</v>
-      </c>
-      <c r="O18" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="P18" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>50</v>
-      </c>
-      <c r="R18" t="n">
-        <v>32.4</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>8:40</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Minnesota Twins</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Kansas City Royals</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>44.0</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>56.0</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>3-5</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>20.8</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>6.7</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N19" t="n">
-        <v>41</v>
-      </c>
-      <c r="O19" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="P19" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>61</v>
-      </c>
-      <c r="R19" t="n">
-        <v>34.1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>8:45</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>St.Louis Cardinals</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>44.0</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>56.0</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>4-6</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>87.0</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>62.0</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>36.7</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N20" t="n">
-        <v>34</v>
-      </c>
-      <c r="O20" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="P20" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>50</v>
-      </c>
-      <c r="R20" t="n">
-        <v>32.4</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Athletics</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>41.0</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>59.0</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>4-6</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>87.0</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>63.2</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>37.9</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N21" t="n">
-        <v>34</v>
-      </c>
-      <c r="O21" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="P21" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>50</v>
-      </c>
-      <c r="R21" t="n">
-        <v>32.4</v>
+        <v>40.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-30 15:06
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R17"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,37 +511,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>24.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>76.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>66.7</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>41.7</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -575,19 +575,19 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="O2" t="n">
-        <v>26.7</v>
+        <v>35</v>
       </c>
       <c r="P2" t="n">
-        <v>73.3</v>
+        <v>65</v>
       </c>
       <c r="Q2" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="R2" t="n">
-        <v>16.7</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
@@ -598,12 +598,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -613,37 +613,37 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>6-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>33.8</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -653,79 +653,79 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="O3" t="n">
-        <v>41.6</v>
+        <v>58.1</v>
       </c>
       <c r="P3" t="n">
-        <v>55.8</v>
+        <v>34.9</v>
       </c>
       <c r="Q3" t="n">
-        <v>45.5</v>
+        <v>44.2</v>
       </c>
       <c r="R3" t="n">
-        <v>27.3</v>
+        <v>32.6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>3:15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>39.0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>61.0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2-5</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>55.0</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>45.0</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>6-5</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>92.1</t>
-        </is>
-      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>67.8</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>42.9</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,59 +735,59 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>17</v>
+        <v>85</v>
       </c>
       <c r="O4" t="n">
-        <v>58.8</v>
+        <v>32.9</v>
       </c>
       <c r="P4" t="n">
-        <v>35.3</v>
+        <v>64.7</v>
       </c>
       <c r="Q4" t="n">
-        <v>35.3</v>
+        <v>49.4</v>
       </c>
       <c r="R4" t="n">
-        <v>35.3</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>6-5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>68.9</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>44.2</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,35 +821,35 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="O5" t="n">
-        <v>57.5</v>
+        <v>58.8</v>
       </c>
       <c r="P5" t="n">
-        <v>40</v>
+        <v>35.3</v>
       </c>
       <c r="Q5" t="n">
-        <v>35</v>
+        <v>35.3</v>
       </c>
       <c r="R5" t="n">
-        <v>15</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,37 +859,37 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,54 +899,54 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O6" t="n">
-        <v>57.7</v>
+        <v>41.6</v>
       </c>
       <c r="P6" t="n">
-        <v>39.7</v>
+        <v>55.8</v>
       </c>
       <c r="Q6" t="n">
-        <v>51.3</v>
+        <v>45.5</v>
       </c>
       <c r="R6" t="n">
-        <v>35.9</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1003,119 +1003,119 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>25.8</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="O8" t="n">
-        <v>41.6</v>
+        <v>51.5</v>
       </c>
       <c r="P8" t="n">
-        <v>55.8</v>
+        <v>44.1</v>
       </c>
       <c r="Q8" t="n">
-        <v>45.5</v>
+        <v>52.9</v>
       </c>
       <c r="R8" t="n">
-        <v>27.3</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>2:40</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1125,22 +1125,22 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1149,55 +1149,55 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="O9" t="n">
-        <v>60.8</v>
+        <v>51.5</v>
       </c>
       <c r="P9" t="n">
-        <v>39.2</v>
+        <v>44.1</v>
       </c>
       <c r="Q9" t="n">
-        <v>44.6</v>
+        <v>52.9</v>
       </c>
       <c r="R9" t="n">
-        <v>31.1</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pacific league</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Central league</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>79.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>21.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1212,12 +1212,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1231,55 +1231,55 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>17</v>
+        <v>135</v>
       </c>
       <c r="O10" t="n">
-        <v>47.1</v>
+        <v>49.6</v>
       </c>
       <c r="P10" t="n">
-        <v>41.2</v>
+        <v>48.1</v>
       </c>
       <c r="Q10" t="n">
-        <v>17.6</v>
+        <v>45.9</v>
       </c>
       <c r="R10" t="n">
-        <v>17.6</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1289,17 +1289,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>55.7</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>30.6</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1313,40 +1313,40 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>68</v>
+        <v>135</v>
       </c>
       <c r="O11" t="n">
-        <v>51.5</v>
+        <v>49.6</v>
       </c>
       <c r="P11" t="n">
-        <v>44.1</v>
+        <v>48.1</v>
       </c>
       <c r="Q11" t="n">
-        <v>52.9</v>
+        <v>45.9</v>
       </c>
       <c r="R11" t="n">
-        <v>35.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1371,22 +1371,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>66.7</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>41.7</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1395,19 +1395,19 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>135</v>
+        <v>29</v>
       </c>
       <c r="O12" t="n">
-        <v>49.6</v>
+        <v>41.4</v>
       </c>
       <c r="P12" t="n">
-        <v>48.1</v>
+        <v>58.6</v>
       </c>
       <c r="Q12" t="n">
-        <v>45.9</v>
+        <v>51.7</v>
       </c>
       <c r="R12" t="n">
-        <v>31.1</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="13">
@@ -1418,12 +1418,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1433,17 +1433,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1453,17 +1453,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>64.4</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>39.2</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,35 +1477,35 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="O13" t="n">
-        <v>61.8</v>
+        <v>48.8</v>
       </c>
       <c r="P13" t="n">
-        <v>38.2</v>
+        <v>48.8</v>
       </c>
       <c r="Q13" t="n">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="R13" t="n">
-        <v>32.4</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1:35</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1515,17 +1515,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1535,17 +1535,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1559,265 +1559,19 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="O14" t="n">
-        <v>49.1</v>
+        <v>48.8</v>
       </c>
       <c r="P14" t="n">
-        <v>49.1</v>
+        <v>48.8</v>
       </c>
       <c r="Q14" t="n">
-        <v>49.1</v>
+        <v>61</v>
       </c>
       <c r="R14" t="n">
-        <v>42.1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>8:10</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>New York Mets</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Atlanta Braves</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>48.0</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>52.0</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>4-6</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>87.0</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>65.6</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>40.4</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N15" t="n">
-        <v>34</v>
-      </c>
-      <c r="O15" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="P15" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>50</v>
-      </c>
-      <c r="R15" t="n">
-        <v>32.4</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>8:45</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>St.Louis Cardinals</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>39.0</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>61.0</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>3-5</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>42.1</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>19.4</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N16" t="n">
-        <v>41</v>
-      </c>
-      <c r="O16" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="P16" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>61</v>
-      </c>
-      <c r="R16" t="n">
         <v>34.1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Athletics</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>39.0</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>61.0</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>4-7</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>92.1</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>73.1</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>49.2</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N17" t="n">
-        <v>67</v>
-      </c>
-      <c r="O17" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="P17" t="n">
-        <v>46.3</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>58.2</v>
-      </c>
-      <c r="R17" t="n">
-        <v>40.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-07-31 13:54
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,12 +516,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,12 +531,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -556,12 +556,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>66.7</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>41.7</t>
+          <t>51.6</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -593,139 +593,139 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6-2</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>73.1</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>49.2</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="O3" t="n">
-        <v>58.1</v>
+        <v>35</v>
       </c>
       <c r="P3" t="n">
-        <v>34.9</v>
+        <v>65</v>
       </c>
       <c r="Q3" t="n">
-        <v>44.2</v>
+        <v>50</v>
       </c>
       <c r="R3" t="n">
-        <v>32.6</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3:15</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2-5</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,79 +735,79 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>85</v>
+        <v>40</v>
       </c>
       <c r="O4" t="n">
-        <v>32.9</v>
+        <v>57.5</v>
       </c>
       <c r="P4" t="n">
-        <v>64.7</v>
+        <v>40</v>
       </c>
       <c r="Q4" t="n">
-        <v>49.4</v>
+        <v>35</v>
       </c>
       <c r="R4" t="n">
-        <v>27.1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>6-5</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>68.9</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>44.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -817,59 +817,59 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="O5" t="n">
-        <v>58.8</v>
+        <v>41.6</v>
       </c>
       <c r="P5" t="n">
-        <v>35.3</v>
+        <v>55.8</v>
       </c>
       <c r="Q5" t="n">
-        <v>35.3</v>
+        <v>45.5</v>
       </c>
       <c r="R5" t="n">
-        <v>35.3</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>2-5</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -884,12 +884,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -903,55 +903,55 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="O6" t="n">
-        <v>41.6</v>
+        <v>32.9</v>
       </c>
       <c r="P6" t="n">
-        <v>55.8</v>
+        <v>64.7</v>
       </c>
       <c r="Q6" t="n">
-        <v>45.5</v>
+        <v>49.4</v>
       </c>
       <c r="R6" t="n">
-        <v>27.3</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,17 +961,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,55 +985,55 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O7" t="n">
-        <v>57.7</v>
+        <v>57.5</v>
       </c>
       <c r="P7" t="n">
-        <v>39.7</v>
+        <v>40</v>
       </c>
       <c r="Q7" t="n">
-        <v>51.3</v>
+        <v>35</v>
       </c>
       <c r="R7" t="n">
-        <v>35.9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>3:20</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1067,35 +1067,35 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="O8" t="n">
-        <v>51.5</v>
+        <v>57.7</v>
       </c>
       <c r="P8" t="n">
-        <v>44.1</v>
+        <v>39.7</v>
       </c>
       <c r="Q8" t="n">
-        <v>52.9</v>
+        <v>51.3</v>
       </c>
       <c r="R8" t="n">
-        <v>35.3</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2:40</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1105,79 +1105,79 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="O9" t="n">
-        <v>51.5</v>
+        <v>41.6</v>
       </c>
       <c r="P9" t="n">
-        <v>44.1</v>
+        <v>55.8</v>
       </c>
       <c r="Q9" t="n">
-        <v>52.9</v>
+        <v>45.5</v>
       </c>
       <c r="R9" t="n">
-        <v>35.3</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>10:38</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1187,22 +1187,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>2-5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1212,74 +1212,74 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>135</v>
+        <v>85</v>
       </c>
       <c r="O10" t="n">
-        <v>49.6</v>
+        <v>32.9</v>
       </c>
       <c r="P10" t="n">
-        <v>48.1</v>
+        <v>64.7</v>
       </c>
       <c r="Q10" t="n">
-        <v>45.9</v>
+        <v>49.4</v>
       </c>
       <c r="R10" t="n">
-        <v>31.1</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1294,12 +1294,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1313,19 +1313,19 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>135</v>
+        <v>17</v>
       </c>
       <c r="O11" t="n">
-        <v>49.6</v>
+        <v>47.1</v>
       </c>
       <c r="P11" t="n">
-        <v>48.1</v>
+        <v>41.2</v>
       </c>
       <c r="Q11" t="n">
-        <v>45.9</v>
+        <v>17.6</v>
       </c>
       <c r="R11" t="n">
-        <v>31.1</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="12">
@@ -1336,12 +1336,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1351,42 +1351,42 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>57.0</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>43.0</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>6-4</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>87.0</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>66.7</t>
-        </is>
-      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>41.7</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1395,19 +1395,19 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="O12" t="n">
-        <v>41.4</v>
+        <v>51.5</v>
       </c>
       <c r="P12" t="n">
-        <v>58.6</v>
+        <v>44.1</v>
       </c>
       <c r="Q12" t="n">
-        <v>51.7</v>
+        <v>52.9</v>
       </c>
       <c r="R12" t="n">
-        <v>34.5</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="13">
@@ -1418,12 +1418,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1433,79 +1433,79 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>44.9</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>41</v>
+        <v>135</v>
       </c>
       <c r="O13" t="n">
-        <v>48.8</v>
+        <v>49.6</v>
       </c>
       <c r="P13" t="n">
-        <v>48.8</v>
+        <v>48.1</v>
       </c>
       <c r="Q13" t="n">
-        <v>61</v>
+        <v>45.9</v>
       </c>
       <c r="R13" t="n">
-        <v>34.1</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>7:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1515,63 +1515,1129 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>135</v>
+      </c>
+      <c r="O14" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P14" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R14" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>8:05</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>32.4</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>12.9</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>135</v>
+      </c>
+      <c r="O15" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P15" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R15" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>20.8</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>6.7</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>135</v>
+      </c>
+      <c r="O16" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P16" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R16" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>32.4</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>12.9</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>135</v>
+      </c>
+      <c r="O17" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P17" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R17" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>9:15</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>68</v>
+      </c>
+      <c r="O18" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="P18" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R18" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>9:40</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>43.5</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>68</v>
+      </c>
+      <c r="O19" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="P19" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R19" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>135</v>
+      </c>
+      <c r="O20" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P20" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R20" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>24.5</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>135</v>
+      </c>
+      <c r="O21" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P21" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R21" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Chinatrust Brothers</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>25.8</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>135</v>
+      </c>
+      <c r="O22" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P22" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R22" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Seibu Lions</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Orix Buffaloes</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>40.7</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>18.4</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>9.7</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>원정승</t>
         </is>
       </c>
-      <c r="N14" t="n">
-        <v>41</v>
-      </c>
-      <c r="O14" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="P14" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>61</v>
-      </c>
-      <c r="R14" t="n">
-        <v>34.1</v>
+      <c r="N23" t="n">
+        <v>32</v>
+      </c>
+      <c r="O23" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="P23" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="R23" t="n">
+        <v>15.6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>64.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>57</v>
+      </c>
+      <c r="O24" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="P24" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="R24" t="n">
+        <v>42.1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-6</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>97.4</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>81.7</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>60.9</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>22</v>
+      </c>
+      <c r="O25" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="P25" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="R25" t="n">
+        <v>36.4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>8:07</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>34</v>
+      </c>
+      <c r="O26" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="P26" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>50</v>
+      </c>
+      <c r="R26" t="n">
+        <v>32.4</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>37.0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>7-5</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>77.7</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>55.2</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>18</v>
+      </c>
+      <c r="O27" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="P27" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="R27" t="n">
+        <v>38.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-08-01 10:41
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R27"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,165 +511,165 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>51.6</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="O2" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="P2" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q2" t="n">
         <v>35</v>
       </c>
-      <c r="P2" t="n">
-        <v>65</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>50</v>
-      </c>
       <c r="R2" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>73.1</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>49.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="O3" t="n">
-        <v>35</v>
+        <v>57.7</v>
       </c>
       <c r="P3" t="n">
-        <v>65</v>
+        <v>39.7</v>
       </c>
       <c r="Q3" t="n">
-        <v>50</v>
+        <v>51.3</v>
       </c>
       <c r="R3" t="n">
-        <v>25</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="4">
@@ -680,12 +680,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,17 +695,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>4-1</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,17 +715,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -739,19 +739,19 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="O4" t="n">
-        <v>57.5</v>
+        <v>60</v>
       </c>
       <c r="P4" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="Q4" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="R4" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -777,12 +777,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -802,12 +802,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -844,12 +844,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,37 +859,37 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>34.0</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>66.0</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2-5</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,59 +899,59 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O6" t="n">
-        <v>32.9</v>
+        <v>60.9</v>
       </c>
       <c r="P6" t="n">
-        <v>64.7</v>
+        <v>39.1</v>
       </c>
       <c r="Q6" t="n">
-        <v>49.4</v>
+        <v>44.8</v>
       </c>
       <c r="R6" t="n">
-        <v>27.1</v>
+        <v>29.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,17 +961,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>39.3</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,75 +985,75 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="O7" t="n">
-        <v>57.5</v>
+        <v>57.7</v>
       </c>
       <c r="P7" t="n">
-        <v>40</v>
+        <v>39.7</v>
       </c>
       <c r="Q7" t="n">
-        <v>35</v>
+        <v>51.3</v>
       </c>
       <c r="R7" t="n">
-        <v>15</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3:20</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1063,187 +1063,187 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O8" t="n">
-        <v>57.7</v>
+        <v>41.6</v>
       </c>
       <c r="P8" t="n">
-        <v>39.7</v>
+        <v>55.8</v>
       </c>
       <c r="Q8" t="n">
-        <v>51.3</v>
+        <v>45.5</v>
       </c>
       <c r="R8" t="n">
-        <v>35.9</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="O9" t="n">
-        <v>41.6</v>
+        <v>51.5</v>
       </c>
       <c r="P9" t="n">
-        <v>55.8</v>
+        <v>44.1</v>
       </c>
       <c r="Q9" t="n">
-        <v>45.5</v>
+        <v>52.9</v>
       </c>
       <c r="R9" t="n">
-        <v>27.3</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>10:38</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2-5</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>58.3</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="O10" t="n">
-        <v>32.9</v>
+        <v>51.5</v>
       </c>
       <c r="P10" t="n">
-        <v>64.7</v>
+        <v>44.1</v>
       </c>
       <c r="Q10" t="n">
-        <v>49.4</v>
+        <v>52.9</v>
       </c>
       <c r="R10" t="n">
-        <v>27.1</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="11">
@@ -1254,52 +1254,52 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>7-9</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>99.6</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>90.9</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>76.5</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1309,29 +1309,29 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>17</v>
+        <v>568</v>
       </c>
       <c r="O11" t="n">
-        <v>47.1</v>
+        <v>48.6</v>
       </c>
       <c r="P11" t="n">
-        <v>41.2</v>
+        <v>48.9</v>
       </c>
       <c r="Q11" t="n">
-        <v>17.6</v>
+        <v>47.5</v>
       </c>
       <c r="R11" t="n">
-        <v>17.6</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1351,12 +1351,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1413,32 +1413,32 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1458,12 +1458,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>35.2</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>14.6</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1495,32 +1495,32 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>7:10</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1540,12 +1540,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1577,1067 +1577,165 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N15" t="n">
-        <v>135</v>
+        <v>40</v>
       </c>
       <c r="O15" t="n">
-        <v>49.6</v>
+        <v>55</v>
       </c>
       <c r="P15" t="n">
-        <v>48.1</v>
+        <v>40</v>
       </c>
       <c r="Q15" t="n">
-        <v>45.9</v>
+        <v>30</v>
       </c>
       <c r="R15" t="n">
-        <v>31.1</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>46.3</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>22.6</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N16" t="n">
-        <v>135</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>49.6</v>
+        <v>48.8</v>
       </c>
       <c r="P16" t="n">
-        <v>48.1</v>
+        <v>48.8</v>
       </c>
       <c r="Q16" t="n">
-        <v>45.9</v>
+        <v>61</v>
       </c>
       <c r="R16" t="n">
-        <v>31.1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>8:15</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Atlanta Braves</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Washington Nationals</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>54.0</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>46.0</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>32.4</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>12.9</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N17" t="n">
-        <v>135</v>
-      </c>
-      <c r="O17" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="P17" t="n">
-        <v>48.1</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="R17" t="n">
-        <v>31.1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>9:15</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Houston Astros</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Texas Rangers</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>58.0</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>42.0</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>42.1</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>19.4</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N18" t="n">
-        <v>68</v>
-      </c>
-      <c r="O18" t="n">
-        <v>51.5</v>
-      </c>
-      <c r="P18" t="n">
-        <v>44.1</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="R18" t="n">
-        <v>35.3</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>9:40</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Colorado Rockies</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Kansas City Royals</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>43.5</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>20.4</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N19" t="n">
-        <v>68</v>
-      </c>
-      <c r="O19" t="n">
-        <v>51.5</v>
-      </c>
-      <c r="P19" t="n">
-        <v>44.1</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="R19" t="n">
-        <v>35.3</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>19:35</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Fubon Guardians</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>TSG Hawks</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>52.0</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>48.0</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>27.1</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>9.9</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N20" t="n">
-        <v>135</v>
-      </c>
-      <c r="O20" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="P20" t="n">
-        <v>48.1</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="R20" t="n">
-        <v>31.1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>19:35</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Uni Lions</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Rakuten Monkeys</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>54.0</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>46.0</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>24.5</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N21" t="n">
-        <v>135</v>
-      </c>
-      <c r="O21" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="P21" t="n">
-        <v>48.1</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="R21" t="n">
-        <v>31.1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>19:35</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Wei Chuan Dragons</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Chinatrust Brothers</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>59.0</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>41.0</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>25.8</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>9.2</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N22" t="n">
-        <v>135</v>
-      </c>
-      <c r="O22" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="P22" t="n">
-        <v>48.1</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="R22" t="n">
-        <v>31.1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Seibu Lions</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Orix Buffaloes</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>NPB</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>46.0</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>54.0</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>2-3</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>23.8</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>9.7</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>2.3</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N23" t="n">
-        <v>32</v>
-      </c>
-      <c r="O23" t="n">
-        <v>59.4</v>
-      </c>
-      <c r="P23" t="n">
-        <v>40.6</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>28.1</v>
-      </c>
-      <c r="R23" t="n">
-        <v>15.6</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Doosan Bears</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>LG Twins</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>KBO</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>36.0</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>64.0</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>4-5</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>54.4</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>29.4</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N24" t="n">
-        <v>57</v>
-      </c>
-      <c r="O24" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="P24" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="R24" t="n">
-        <v>42.1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Lotte Giants</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Samsung Lions</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>KBO</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>54.0</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>46.0</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>7-6</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>97.4</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>81.7</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>60.9</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N25" t="n">
-        <v>22</v>
-      </c>
-      <c r="O25" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="P25" t="n">
-        <v>54.5</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>59.1</v>
-      </c>
-      <c r="R25" t="n">
-        <v>36.4</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>8:07</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Toronto Blue Jays</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>St.Louis Cardinals</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>49.0</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>51.0</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>4-6</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>87.0</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>42.1</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>19.4</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N26" t="n">
-        <v>34</v>
-      </c>
-      <c r="O26" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="P26" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>50</v>
-      </c>
-      <c r="R26" t="n">
-        <v>32.4</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>8:10</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>New York Mets</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Miami Marlins</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>63.0</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>37.0</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>7-5</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>95.4</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>77.7</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>55.2</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N27" t="n">
-        <v>18</v>
-      </c>
-      <c r="O27" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="P27" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>61.1</v>
-      </c>
-      <c r="R27" t="n">
-        <v>38.9</v>
+        <v>34.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-08-02 11:32
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -531,12 +531,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -593,17 +593,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -613,17 +613,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-1</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,35 +657,35 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="O3" t="n">
-        <v>57.7</v>
+        <v>60</v>
       </c>
       <c r="P3" t="n">
-        <v>39.7</v>
+        <v>38</v>
       </c>
       <c r="Q3" t="n">
-        <v>51.3</v>
+        <v>38</v>
       </c>
       <c r="R3" t="n">
-        <v>35.9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,17 +695,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4-1</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -720,12 +720,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -739,19 +739,19 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="O4" t="n">
-        <v>60</v>
+        <v>60.8</v>
       </c>
       <c r="P4" t="n">
-        <v>38</v>
+        <v>39.2</v>
       </c>
       <c r="Q4" t="n">
-        <v>38</v>
+        <v>44.6</v>
       </c>
       <c r="R4" t="n">
-        <v>18</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="5">
@@ -762,12 +762,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -777,37 +777,37 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -817,23 +817,23 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O5" t="n">
-        <v>41.6</v>
+        <v>57.7</v>
       </c>
       <c r="P5" t="n">
-        <v>55.8</v>
+        <v>39.7</v>
       </c>
       <c r="Q5" t="n">
-        <v>45.5</v>
+        <v>51.3</v>
       </c>
       <c r="R5" t="n">
-        <v>27.3</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="6">
@@ -844,52 +844,52 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-1</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>66.7</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>41.7</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,44 +899,44 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>87</v>
+        <v>22</v>
       </c>
       <c r="O6" t="n">
-        <v>60.9</v>
+        <v>40.9</v>
       </c>
       <c r="P6" t="n">
-        <v>39.1</v>
+        <v>59.1</v>
       </c>
       <c r="Q6" t="n">
-        <v>44.8</v>
+        <v>68.2</v>
       </c>
       <c r="R6" t="n">
-        <v>29.9</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,22 +961,22 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -985,101 +985,101 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>78</v>
+        <v>135</v>
       </c>
       <c r="O7" t="n">
-        <v>57.7</v>
+        <v>49.6</v>
       </c>
       <c r="P7" t="n">
-        <v>39.7</v>
+        <v>48.1</v>
       </c>
       <c r="Q7" t="n">
-        <v>51.3</v>
+        <v>45.9</v>
       </c>
       <c r="R7" t="n">
-        <v>35.9</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="O8" t="n">
-        <v>41.6</v>
+        <v>51.5</v>
       </c>
       <c r="P8" t="n">
-        <v>55.8</v>
+        <v>44.1</v>
       </c>
       <c r="Q8" t="n">
-        <v>45.5</v>
+        <v>52.9</v>
       </c>
       <c r="R8" t="n">
-        <v>27.3</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="9">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1105,37 +1105,37 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>7-8</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>99.2</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>90.9</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>76.5</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1145,59 +1145,59 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>68</v>
+        <v>568</v>
       </c>
       <c r="O9" t="n">
-        <v>51.5</v>
+        <v>48.6</v>
       </c>
       <c r="P9" t="n">
-        <v>44.1</v>
+        <v>48.9</v>
       </c>
       <c r="Q9" t="n">
-        <v>52.9</v>
+        <v>47.5</v>
       </c>
       <c r="R9" t="n">
-        <v>35.3</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>2:37</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,17 +1207,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>58.3</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1231,75 +1231,75 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>68</v>
+        <v>135</v>
       </c>
       <c r="O10" t="n">
-        <v>51.5</v>
+        <v>49.6</v>
       </c>
       <c r="P10" t="n">
-        <v>44.1</v>
+        <v>48.1</v>
       </c>
       <c r="Q10" t="n">
-        <v>52.9</v>
+        <v>45.9</v>
       </c>
       <c r="R10" t="n">
-        <v>35.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>7-9</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>99.6</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>90.9</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>76.5</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1309,44 +1309,44 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>568</v>
+        <v>135</v>
       </c>
       <c r="O11" t="n">
-        <v>48.6</v>
+        <v>49.6</v>
       </c>
       <c r="P11" t="n">
-        <v>48.9</v>
+        <v>48.1</v>
       </c>
       <c r="Q11" t="n">
-        <v>47.5</v>
+        <v>45.9</v>
       </c>
       <c r="R11" t="n">
-        <v>31.2</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1371,17 +1371,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>31.8</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1395,35 +1395,35 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>68</v>
+        <v>135</v>
       </c>
       <c r="O12" t="n">
-        <v>51.5</v>
+        <v>49.6</v>
       </c>
       <c r="P12" t="n">
-        <v>44.1</v>
+        <v>48.1</v>
       </c>
       <c r="Q12" t="n">
-        <v>52.9</v>
+        <v>45.9</v>
       </c>
       <c r="R12" t="n">
-        <v>35.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1458,12 +1458,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>23.3</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>7.9</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1500,12 +1500,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1540,12 +1540,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1577,17 +1577,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1597,17 +1597,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1617,17 +1617,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1641,19 +1641,19 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>55</v>
+        <v>48.8</v>
       </c>
       <c r="P15" t="n">
-        <v>40</v>
+        <v>48.8</v>
       </c>
       <c r="Q15" t="n">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="R15" t="n">
-        <v>17.5</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="16">
@@ -1664,78 +1664,406 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>40</v>
+      </c>
+      <c r="O16" t="n">
+        <v>55</v>
+      </c>
+      <c r="P16" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>30</v>
+      </c>
+      <c r="R16" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>KBO</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>41.0</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>59.0</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>3-5</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>46.3</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>22.6</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>원정승</t>
         </is>
       </c>
-      <c r="N16" t="n">
-        <v>41</v>
-      </c>
-      <c r="O16" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="P16" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>61</v>
-      </c>
-      <c r="R16" t="n">
-        <v>34.1</v>
+      <c r="N17" t="n">
+        <v>57</v>
+      </c>
+      <c r="O17" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="P17" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="R17" t="n">
+        <v>42.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2:40</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>3-6</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>51.8</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>14</v>
+      </c>
+      <c r="O18" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="P18" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>50</v>
+      </c>
+      <c r="R18" t="n">
+        <v>35.7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2:40</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>49.1</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>24.8</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>57</v>
+      </c>
+      <c r="O19" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="P19" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="R19" t="n">
+        <v>42.1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>3:20</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>63.2</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>37.9</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>34</v>
+      </c>
+      <c r="O20" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="P20" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>50</v>
+      </c>
+      <c r="R20" t="n">
+        <v>32.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-08-04 14:03
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,119 +511,119 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>28.0</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>72.0</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>28.0</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>74</v>
+        <v>30</v>
       </c>
       <c r="O2" t="n">
-        <v>60.8</v>
+        <v>26.7</v>
       </c>
       <c r="P2" t="n">
-        <v>39.2</v>
+        <v>73.3</v>
       </c>
       <c r="Q2" t="n">
-        <v>44.6</v>
+        <v>30</v>
       </c>
       <c r="R2" t="n">
-        <v>31.1</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6-5</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>72.1</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>47.9</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -657,19 +657,19 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>17</v>
+        <v>74</v>
       </c>
       <c r="O3" t="n">
-        <v>58.8</v>
+        <v>60.8</v>
       </c>
       <c r="P3" t="n">
-        <v>35.3</v>
+        <v>39.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>35.3</v>
+        <v>44.6</v>
       </c>
       <c r="R3" t="n">
-        <v>35.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="4">
@@ -680,12 +680,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,17 +695,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,22 +715,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -739,35 +739,35 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="O4" t="n">
-        <v>51.5</v>
+        <v>60.8</v>
       </c>
       <c r="P4" t="n">
-        <v>44.1</v>
+        <v>39.2</v>
       </c>
       <c r="Q4" t="n">
-        <v>52.9</v>
+        <v>44.6</v>
       </c>
       <c r="R4" t="n">
-        <v>35.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>7:35</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -777,17 +777,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,22 +797,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -821,35 +821,35 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="O5" t="n">
-        <v>51.5</v>
+        <v>57.7</v>
       </c>
       <c r="P5" t="n">
-        <v>44.1</v>
+        <v>39.7</v>
       </c>
       <c r="Q5" t="n">
-        <v>52.9</v>
+        <v>51.3</v>
       </c>
       <c r="R5" t="n">
-        <v>35.3</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,145 +859,1703 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="O6" t="n">
-        <v>41.4</v>
+        <v>41.6</v>
       </c>
       <c r="P6" t="n">
-        <v>58.6</v>
+        <v>55.8</v>
       </c>
       <c r="Q6" t="n">
-        <v>51.7</v>
+        <v>45.5</v>
       </c>
       <c r="R6" t="n">
-        <v>34.5</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>12.3</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>74</v>
+      </c>
+      <c r="O7" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="P7" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="R7" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>9:05</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>77</v>
+      </c>
+      <c r="O8" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="P8" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="R8" t="n">
+        <v>27.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>9:40</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Colorado Rockies</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>MLB</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>80.9</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>59.8</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>22</v>
+      </c>
+      <c r="O9" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="P9" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="R9" t="n">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Hiroshima Carp</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Yomiuri Giants</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>64.0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>24.5</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>17</v>
+      </c>
+      <c r="O10" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="R10" t="n">
+        <v>17.6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Kiwoom Heroes</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>61.0</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>39.0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>68</v>
+      </c>
+      <c r="O11" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="P11" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R11" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Hanwha Eagles</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>33.8</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>13.8</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>135</v>
+      </c>
+      <c r="O12" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P12" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R12" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>37.0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>40.7</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>68</v>
+      </c>
+      <c r="O13" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="P13" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R13" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>135</v>
+      </c>
+      <c r="O14" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P14" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R14" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>9:05</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>29.4</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>68</v>
+      </c>
+      <c r="O15" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="P15" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R15" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>67.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>33.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>28.4</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>10.6</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>135</v>
+      </c>
+      <c r="O16" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P16" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R16" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Chinatrust Brothers</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>66.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>28.4</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>10.6</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>17</v>
+      </c>
+      <c r="O17" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="P17" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="R17" t="n">
+        <v>17.6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>46.3</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>22.6</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>68</v>
+      </c>
+      <c r="O18" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="P18" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R18" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Chunichi Dragons</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Yakult Swallows</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>38.0</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>16.5</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>57</v>
+      </c>
+      <c r="O19" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="P19" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="R19" t="n">
+        <v>42.1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>NC Dinos</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>53.1</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>28.2</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>57</v>
+      </c>
+      <c r="O20" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="P20" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="R20" t="n">
+        <v>42.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>KIA Tigers</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>KT Wiz Suwon</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>55.7</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>30.6</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>57</v>
+      </c>
+      <c r="O21" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="P21" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="R21" t="n">
+        <v>42.1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SSG Landers</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
         <is>
           <t>62.0</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>4-6</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>87.0</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>44.9</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>21.5</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>68.9</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>44.2</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>원정승</t>
         </is>
       </c>
-      <c r="N7" t="n">
+      <c r="N22" t="n">
         <v>34</v>
       </c>
-      <c r="O7" t="n">
+      <c r="O22" t="n">
         <v>61.8</v>
       </c>
-      <c r="P7" t="n">
+      <c r="P22" t="n">
         <v>38.2</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="Q22" t="n">
         <v>50</v>
       </c>
-      <c r="R7" t="n">
+      <c r="R22" t="n">
         <v>32.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>8:05</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>39.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>61.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>53.1</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>28.2</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>57</v>
+      </c>
+      <c r="O23" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="P23" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="R23" t="n">
+        <v>42.1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>41.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>29</v>
+      </c>
+      <c r="O24" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="P24" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="R24" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>37.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7-5</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>79.4</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>57.5</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>18</v>
+      </c>
+      <c r="O25" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="P25" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="R25" t="n">
+        <v>38.9</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>18.5</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>41</v>
+      </c>
+      <c r="O26" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="P26" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>61</v>
+      </c>
+      <c r="R26" t="n">
+        <v>34.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-08-05 14:47
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -556,12 +556,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -593,83 +593,83 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>55.0</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>45.0</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>74</v>
+        <v>30</v>
       </c>
       <c r="O3" t="n">
-        <v>60.8</v>
+        <v>26.7</v>
       </c>
       <c r="P3" t="n">
-        <v>39.2</v>
+        <v>73.3</v>
       </c>
       <c r="Q3" t="n">
-        <v>44.6</v>
+        <v>30</v>
       </c>
       <c r="R3" t="n">
-        <v>31.1</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="4">
@@ -680,12 +680,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,12 +695,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>65.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -720,12 +720,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -757,37 +757,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7:35</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -797,17 +797,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,35 +821,35 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="O5" t="n">
-        <v>57.7</v>
+        <v>57.5</v>
       </c>
       <c r="P5" t="n">
-        <v>39.7</v>
+        <v>40</v>
       </c>
       <c r="Q5" t="n">
-        <v>51.3</v>
+        <v>35</v>
       </c>
       <c r="R5" t="n">
-        <v>35.9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>3:20</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,37 +859,37 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>33.8</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,39 +899,39 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O6" t="n">
-        <v>41.6</v>
+        <v>57.7</v>
       </c>
       <c r="P6" t="n">
-        <v>55.8</v>
+        <v>39.7</v>
       </c>
       <c r="Q6" t="n">
-        <v>45.5</v>
+        <v>51.3</v>
       </c>
       <c r="R6" t="n">
-        <v>27.3</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -941,17 +941,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>6-5</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,17 +961,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>63.2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>37.9</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -985,35 +985,35 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>74</v>
+        <v>17</v>
       </c>
       <c r="O7" t="n">
-        <v>60.8</v>
+        <v>58.8</v>
       </c>
       <c r="P7" t="n">
-        <v>39.2</v>
+        <v>35.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>44.6</v>
+        <v>35.3</v>
       </c>
       <c r="R7" t="n">
-        <v>31.1</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1023,37 +1023,37 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1063,59 +1063,59 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="O8" t="n">
-        <v>41.6</v>
+        <v>60.8</v>
       </c>
       <c r="P8" t="n">
-        <v>55.8</v>
+        <v>39.2</v>
       </c>
       <c r="Q8" t="n">
-        <v>45.5</v>
+        <v>44.6</v>
       </c>
       <c r="R8" t="n">
-        <v>27.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1125,22 +1125,22 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>80.9</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>59.8</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1149,19 +1149,19 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>22</v>
+        <v>531</v>
       </c>
       <c r="O9" t="n">
-        <v>40.9</v>
+        <v>48.4</v>
       </c>
       <c r="P9" t="n">
-        <v>59.1</v>
+        <v>49.3</v>
       </c>
       <c r="Q9" t="n">
-        <v>68.2</v>
+        <v>47.5</v>
       </c>
       <c r="R9" t="n">
-        <v>54.5</v>
+        <v>31.8</v>
       </c>
     </row>
     <row r="10">
@@ -1172,12 +1172,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1187,17 +1187,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1207,17 +1207,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>16.5</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1231,50 +1231,50 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="O10" t="n">
-        <v>47.1</v>
+        <v>51.5</v>
       </c>
       <c r="P10" t="n">
-        <v>41.2</v>
+        <v>44.1</v>
       </c>
       <c r="Q10" t="n">
-        <v>17.6</v>
+        <v>52.9</v>
       </c>
       <c r="R10" t="n">
-        <v>17.6</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1294,12 +1294,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>47.7</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>23.7</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1351,17 +1351,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1371,17 +1371,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>33.8</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1395,35 +1395,35 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>135</v>
+        <v>68</v>
       </c>
       <c r="O12" t="n">
-        <v>49.6</v>
+        <v>51.5</v>
       </c>
       <c r="P12" t="n">
-        <v>48.1</v>
+        <v>44.1</v>
       </c>
       <c r="Q12" t="n">
-        <v>45.9</v>
+        <v>52.9</v>
       </c>
       <c r="R12" t="n">
-        <v>31.1</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1433,17 +1433,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1453,17 +1453,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,35 +1477,35 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="O13" t="n">
-        <v>51.5</v>
+        <v>47.1</v>
       </c>
       <c r="P13" t="n">
-        <v>44.1</v>
+        <v>41.2</v>
       </c>
       <c r="Q13" t="n">
-        <v>52.9</v>
+        <v>17.6</v>
       </c>
       <c r="R13" t="n">
-        <v>35.3</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>4:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1515,37 +1515,37 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>8-9</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>99.8</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>97.3</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>90.8</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1555,39 +1555,39 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>135</v>
+        <v>265</v>
       </c>
       <c r="O14" t="n">
-        <v>49.6</v>
+        <v>43</v>
       </c>
       <c r="P14" t="n">
-        <v>48.1</v>
+        <v>54.7</v>
       </c>
       <c r="Q14" t="n">
-        <v>45.9</v>
+        <v>50.9</v>
       </c>
       <c r="R14" t="n">
-        <v>31.1</v>
+        <v>31.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1597,17 +1597,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1617,17 +1617,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1641,35 +1641,35 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>68</v>
+        <v>135</v>
       </c>
       <c r="O15" t="n">
-        <v>51.5</v>
+        <v>49.6</v>
       </c>
       <c r="P15" t="n">
-        <v>44.1</v>
+        <v>48.1</v>
       </c>
       <c r="Q15" t="n">
-        <v>52.9</v>
+        <v>45.9</v>
       </c>
       <c r="R15" t="n">
-        <v>35.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1741,37 +1741,37 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1805,19 +1805,19 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>17</v>
+        <v>135</v>
       </c>
       <c r="O17" t="n">
-        <v>47.1</v>
+        <v>49.6</v>
       </c>
       <c r="P17" t="n">
-        <v>41.2</v>
+        <v>48.1</v>
       </c>
       <c r="Q17" t="n">
-        <v>17.6</v>
+        <v>45.9</v>
       </c>
       <c r="R17" t="n">
-        <v>17.6</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="18">
@@ -1828,12 +1828,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1843,17 +1843,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1863,17 +1863,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>46.3</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>22.6</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1887,60 +1887,60 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="O18" t="n">
-        <v>51.5</v>
+        <v>47.1</v>
       </c>
       <c r="P18" t="n">
-        <v>44.1</v>
+        <v>41.2</v>
       </c>
       <c r="Q18" t="n">
-        <v>52.9</v>
+        <v>17.6</v>
       </c>
       <c r="R18" t="n">
-        <v>35.3</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1950,38 +1950,38 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>16.5</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N19" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="O19" t="n">
-        <v>49.1</v>
+        <v>51.5</v>
       </c>
       <c r="P19" t="n">
-        <v>49.1</v>
+        <v>44.1</v>
       </c>
       <c r="Q19" t="n">
-        <v>49.1</v>
+        <v>52.9</v>
       </c>
       <c r="R19" t="n">
-        <v>42.1</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="20">
@@ -1992,12 +1992,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2007,17 +2007,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2027,17 +2027,17 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>68.9</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>44.2</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2051,19 +2051,19 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="O20" t="n">
-        <v>49.1</v>
+        <v>61.8</v>
       </c>
       <c r="P20" t="n">
-        <v>49.1</v>
+        <v>38.2</v>
       </c>
       <c r="Q20" t="n">
-        <v>49.1</v>
+        <v>50</v>
       </c>
       <c r="R20" t="n">
-        <v>42.1</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="21">
@@ -2074,12 +2074,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2089,37 +2089,37 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>55.7</t>
+          <t>64.4</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>30.6</t>
+          <t>39.2</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2129,23 +2129,23 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N21" t="n">
-        <v>57</v>
+        <v>29</v>
       </c>
       <c r="O21" t="n">
-        <v>49.1</v>
+        <v>41.4</v>
       </c>
       <c r="P21" t="n">
-        <v>49.1</v>
+        <v>58.6</v>
       </c>
       <c r="Q21" t="n">
-        <v>49.1</v>
+        <v>51.7</v>
       </c>
       <c r="R21" t="n">
-        <v>42.1</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="22">
@@ -2156,12 +2156,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2171,17 +2171,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2191,17 +2191,17 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>68.9</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>44.2</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2215,55 +2215,55 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="O22" t="n">
-        <v>61.8</v>
+        <v>49.1</v>
       </c>
       <c r="P22" t="n">
-        <v>38.2</v>
+        <v>49.1</v>
       </c>
       <c r="Q22" t="n">
-        <v>50</v>
+        <v>49.1</v>
       </c>
       <c r="R22" t="n">
-        <v>32.4</v>
+        <v>42.1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2273,17 +2273,17 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2297,35 +2297,35 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="O23" t="n">
-        <v>49.1</v>
+        <v>48.8</v>
       </c>
       <c r="P23" t="n">
-        <v>49.1</v>
+        <v>48.8</v>
       </c>
       <c r="Q23" t="n">
-        <v>49.1</v>
+        <v>61</v>
       </c>
       <c r="R23" t="n">
-        <v>42.1</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>3:35</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2335,12 +2335,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2360,12 +2360,12 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>40.7</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2397,17 +2397,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2417,12 +2417,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2442,12 +2442,12 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>79.4</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>57.5</t>
+          <t>36.7</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2474,88 +2474,6 @@
       </c>
       <c r="R25" t="n">
         <v>38.9</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Seattle Mariners</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Detroit Tigers</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>3-5</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>18.5</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>5.6</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N26" t="n">
-        <v>41</v>
-      </c>
-      <c r="O26" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="P26" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>61</v>
-      </c>
-      <c r="R26" t="n">
-        <v>34.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-08-06 16:00
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R25"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,17 +511,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,22 +531,22 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -556,156 +556,156 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O2" t="n">
-        <v>26.7</v>
+        <v>57.5</v>
       </c>
       <c r="P2" t="n">
-        <v>73.3</v>
+        <v>40</v>
       </c>
       <c r="Q2" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="R2" t="n">
-        <v>16.7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="O3" t="n">
-        <v>26.7</v>
+        <v>62.5</v>
       </c>
       <c r="P3" t="n">
-        <v>73.3</v>
+        <v>37.5</v>
       </c>
       <c r="Q3" t="n">
-        <v>30</v>
+        <v>37.5</v>
       </c>
       <c r="R3" t="n">
-        <v>16.7</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>2:10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>6-5</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,17 +715,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>92.1</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>36.7</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -739,40 +739,40 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>74</v>
+        <v>17</v>
       </c>
       <c r="O4" t="n">
-        <v>60.8</v>
+        <v>58.8</v>
       </c>
       <c r="P4" t="n">
-        <v>39.2</v>
+        <v>35.3</v>
       </c>
       <c r="Q4" t="n">
-        <v>44.6</v>
+        <v>35.3</v>
       </c>
       <c r="R4" t="n">
-        <v>31.1</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -802,12 +802,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -839,17 +839,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3:20</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,17 +859,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -879,17 +879,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -903,55 +903,55 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="O6" t="n">
-        <v>57.7</v>
+        <v>60.8</v>
       </c>
       <c r="P6" t="n">
-        <v>39.7</v>
+        <v>39.2</v>
       </c>
       <c r="Q6" t="n">
-        <v>51.3</v>
+        <v>44.6</v>
       </c>
       <c r="R6" t="n">
-        <v>35.9</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6-5</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,22 +961,22 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>63.2</t>
+          <t>47.7</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>37.9</t>
+          <t>23.7</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -985,16 +985,16 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="O7" t="n">
-        <v>58.8</v>
+        <v>51.5</v>
       </c>
       <c r="P7" t="n">
-        <v>35.3</v>
+        <v>44.1</v>
       </c>
       <c r="Q7" t="n">
-        <v>35.3</v>
+        <v>52.9</v>
       </c>
       <c r="R7" t="n">
         <v>35.3</v>
@@ -1003,37 +1003,37 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1067,16 +1067,16 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>74</v>
+        <v>135</v>
       </c>
       <c r="O8" t="n">
-        <v>60.8</v>
+        <v>49.6</v>
       </c>
       <c r="P8" t="n">
-        <v>39.2</v>
+        <v>48.1</v>
       </c>
       <c r="Q8" t="n">
-        <v>44.6</v>
+        <v>45.9</v>
       </c>
       <c r="R8" t="n">
         <v>31.1</v>
@@ -1085,57 +1085,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1145,79 +1145,79 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>531</v>
+        <v>135</v>
       </c>
       <c r="O9" t="n">
-        <v>48.4</v>
+        <v>49.6</v>
       </c>
       <c r="P9" t="n">
-        <v>49.3</v>
+        <v>48.1</v>
       </c>
       <c r="Q9" t="n">
-        <v>47.5</v>
+        <v>45.9</v>
       </c>
       <c r="R9" t="n">
-        <v>31.8</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
           <t>55.0</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>45.0</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>16.5</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1231,50 +1231,50 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>68</v>
+        <v>135</v>
       </c>
       <c r="O10" t="n">
-        <v>51.5</v>
+        <v>49.6</v>
       </c>
       <c r="P10" t="n">
-        <v>44.1</v>
+        <v>48.1</v>
       </c>
       <c r="Q10" t="n">
-        <v>52.9</v>
+        <v>45.9</v>
       </c>
       <c r="R10" t="n">
-        <v>35.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1294,12 +1294,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>47.7</t>
+          <t>35.2</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>23.7</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1331,94 +1331,94 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>57.0</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>43.0</t>
-        </is>
-      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>55.7</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>30.6</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="O12" t="n">
-        <v>51.5</v>
+        <v>59.4</v>
       </c>
       <c r="P12" t="n">
-        <v>44.1</v>
+        <v>40.6</v>
       </c>
       <c r="Q12" t="n">
-        <v>52.9</v>
+        <v>28.1</v>
       </c>
       <c r="R12" t="n">
-        <v>35.3</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>3:20</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1433,79 +1433,79 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>63.2</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>37.9</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="O13" t="n">
-        <v>47.1</v>
+        <v>61.8</v>
       </c>
       <c r="P13" t="n">
-        <v>41.2</v>
+        <v>38.2</v>
       </c>
       <c r="Q13" t="n">
-        <v>17.6</v>
+        <v>50</v>
       </c>
       <c r="R13" t="n">
-        <v>17.6</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4:10</t>
+          <t>7:05</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1515,79 +1515,79 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>8-9</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>99.8</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>97.3</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>90.8</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>265</v>
+        <v>29</v>
       </c>
       <c r="O14" t="n">
-        <v>43</v>
+        <v>41.4</v>
       </c>
       <c r="P14" t="n">
-        <v>54.7</v>
+        <v>58.6</v>
       </c>
       <c r="Q14" t="n">
-        <v>50.9</v>
+        <v>51.7</v>
       </c>
       <c r="R14" t="n">
-        <v>31.3</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1597,17 +1597,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1617,22 +1617,22 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>63.2</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>37.9</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1641,35 +1641,35 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>135</v>
+        <v>29</v>
       </c>
       <c r="O15" t="n">
-        <v>49.6</v>
+        <v>41.4</v>
       </c>
       <c r="P15" t="n">
-        <v>48.1</v>
+        <v>58.6</v>
       </c>
       <c r="Q15" t="n">
-        <v>45.9</v>
+        <v>51.7</v>
       </c>
       <c r="R15" t="n">
-        <v>31.1</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1679,17 +1679,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1699,22 +1699,22 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>65.6</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>40.4</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1723,756 +1723,18 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>135</v>
+        <v>18</v>
       </c>
       <c r="O16" t="n">
-        <v>49.6</v>
+        <v>44.4</v>
       </c>
       <c r="P16" t="n">
-        <v>48.1</v>
+        <v>55.6</v>
       </c>
       <c r="Q16" t="n">
-        <v>45.9</v>
+        <v>61.1</v>
       </c>
       <c r="R16" t="n">
-        <v>31.1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Seattle Mariners</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Detroit Tigers</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>59.0</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>41.0</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>28.4</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>10.6</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N17" t="n">
-        <v>135</v>
-      </c>
-      <c r="O17" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="P17" t="n">
-        <v>48.1</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="R17" t="n">
-        <v>31.1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>19:35</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Chinatrust Brothers</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Fubon Guardians</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>58.0</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>42.0</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>5-2</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>28.4</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>10.6</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N18" t="n">
-        <v>17</v>
-      </c>
-      <c r="O18" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="P18" t="n">
-        <v>41.2</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="R18" t="n">
-        <v>17.6</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>19:35</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>TSG Hawks</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Rakuten Monkeys</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>57.0</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>43.0</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>35.2</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>14.6</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N19" t="n">
-        <v>68</v>
-      </c>
-      <c r="O19" t="n">
-        <v>51.5</v>
-      </c>
-      <c r="P19" t="n">
-        <v>44.1</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="R19" t="n">
-        <v>35.3</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>SSG Landers</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>LG Twins</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>KBO</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>39.0</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>61.0</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>4-6</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>87.0</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>68.9</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>44.2</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N20" t="n">
-        <v>34</v>
-      </c>
-      <c r="O20" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="P20" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>50</v>
-      </c>
-      <c r="R20" t="n">
-        <v>32.4</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Lotte Giants</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Kiwoom Heroes</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>KBO</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>58.0</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>42.0</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>6-4</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>87.0</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>64.4</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>39.2</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N21" t="n">
-        <v>29</v>
-      </c>
-      <c r="O21" t="n">
-        <v>41.4</v>
-      </c>
-      <c r="P21" t="n">
-        <v>58.6</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="R21" t="n">
-        <v>34.5</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>KIA Tigers</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>KT Wiz Suwon</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>KBO</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>49.0</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>51.0</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>4-5</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>55.7</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>30.6</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N22" t="n">
-        <v>57</v>
-      </c>
-      <c r="O22" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="P22" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="R22" t="n">
-        <v>42.1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Doosan Bears</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>NC Dinos</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>KBO</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>45.0</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>3-5</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>20.8</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>6.7</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N23" t="n">
-        <v>41</v>
-      </c>
-      <c r="O23" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="P23" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>61</v>
-      </c>
-      <c r="R23" t="n">
-        <v>34.1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>3:35</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Texas Rangers</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>San Francisco Giants</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>58.0</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>42.0</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>6-4</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>87.0</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>40.7</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>18.4</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N24" t="n">
-        <v>29</v>
-      </c>
-      <c r="O24" t="n">
-        <v>41.4</v>
-      </c>
-      <c r="P24" t="n">
-        <v>58.6</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="R24" t="n">
-        <v>34.5</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>8:05</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>New York Yankees</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>St.Louis Cardinals</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>58.0</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>42.0</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>7-5</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>95.4</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>62.0</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>36.7</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N25" t="n">
-        <v>18</v>
-      </c>
-      <c r="O25" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="P25" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>61.1</v>
-      </c>
-      <c r="R25" t="n">
         <v>38.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-08-07 15:34
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,12 +516,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,22 +531,22 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -556,38 +556,38 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="O2" t="n">
-        <v>57.5</v>
+        <v>26.7</v>
       </c>
       <c r="P2" t="n">
-        <v>40</v>
+        <v>73.3</v>
       </c>
       <c r="Q2" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="R2" t="n">
-        <v>15</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="3">
@@ -598,12 +598,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -613,37 +613,37 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -653,59 +653,59 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>8</v>
+        <v>77</v>
       </c>
       <c r="O3" t="n">
-        <v>62.5</v>
+        <v>41.6</v>
       </c>
       <c r="P3" t="n">
-        <v>37.5</v>
+        <v>55.8</v>
       </c>
       <c r="Q3" t="n">
-        <v>37.5</v>
+        <v>45.5</v>
       </c>
       <c r="R3" t="n">
-        <v>25</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6-5</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,17 +715,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>92.1</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>36.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -739,35 +739,35 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>17</v>
+        <v>74</v>
       </c>
       <c r="O4" t="n">
-        <v>58.8</v>
+        <v>60.8</v>
       </c>
       <c r="P4" t="n">
-        <v>35.3</v>
+        <v>39.2</v>
       </c>
       <c r="Q4" t="n">
-        <v>35.3</v>
+        <v>44.6</v>
       </c>
       <c r="R4" t="n">
-        <v>35.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>9:10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -777,37 +777,37 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>39.4</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>29.7</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>11.3</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -817,39 +817,39 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>40</v>
+        <v>77</v>
       </c>
       <c r="O5" t="n">
-        <v>57.5</v>
+        <v>41.6</v>
       </c>
       <c r="P5" t="n">
-        <v>40</v>
+        <v>55.8</v>
       </c>
       <c r="Q5" t="n">
-        <v>35</v>
+        <v>45.5</v>
       </c>
       <c r="R5" t="n">
-        <v>15</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,12 +859,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -921,37 +921,37 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -961,22 +961,22 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>47.7</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>23.7</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -985,19 +985,19 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="O7" t="n">
-        <v>51.5</v>
+        <v>60.8</v>
       </c>
       <c r="P7" t="n">
-        <v>44.1</v>
+        <v>39.2</v>
       </c>
       <c r="Q7" t="n">
-        <v>52.9</v>
+        <v>44.6</v>
       </c>
       <c r="R7" t="n">
-        <v>35.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="8">
@@ -1008,14 +1008,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>Hanshin Tigers</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Chunichi Dragons</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Yakult Swallows</t>
-        </is>
-      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>NPB</t>
@@ -1023,12 +1023,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1085,37 +1085,37 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>26.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1130,12 +1130,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1149,50 +1149,50 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>135</v>
+        <v>17</v>
       </c>
       <c r="O9" t="n">
-        <v>49.6</v>
+        <v>47.1</v>
       </c>
       <c r="P9" t="n">
-        <v>48.1</v>
+        <v>41.2</v>
       </c>
       <c r="Q9" t="n">
-        <v>45.9</v>
+        <v>17.6</v>
       </c>
       <c r="R9" t="n">
-        <v>31.1</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1212,12 +1212,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1249,32 +1249,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Wei Chuan Dragons</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1294,12 +1294,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>35.2</t>
+          <t>59.6</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>14.6</t>
+          <t>34.2</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1331,181 +1331,181 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>32</v>
+        <v>135</v>
       </c>
       <c r="O12" t="n">
-        <v>59.4</v>
+        <v>49.6</v>
       </c>
       <c r="P12" t="n">
-        <v>40.6</v>
+        <v>48.1</v>
       </c>
       <c r="Q12" t="n">
-        <v>28.1</v>
+        <v>45.9</v>
       </c>
       <c r="R12" t="n">
-        <v>15.6</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3:20</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>9-6</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>99.2</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>63.2</t>
+          <t>93.8</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>37.9</t>
+          <t>82.4</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>34</v>
+        <v>509</v>
       </c>
       <c r="O13" t="n">
-        <v>61.8</v>
+        <v>52.8</v>
       </c>
       <c r="P13" t="n">
-        <v>38.2</v>
+        <v>44.4</v>
       </c>
       <c r="Q13" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="R13" t="n">
-        <v>32.4</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>7:05</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1515,17 +1515,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>7-2</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1535,22 +1535,22 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1559,35 +1559,35 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>29</v>
+        <v>509</v>
       </c>
       <c r="O14" t="n">
-        <v>41.4</v>
+        <v>52.8</v>
       </c>
       <c r="P14" t="n">
-        <v>58.6</v>
+        <v>44.4</v>
       </c>
       <c r="Q14" t="n">
-        <v>51.7</v>
+        <v>46</v>
       </c>
       <c r="R14" t="n">
-        <v>34.5</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1597,17 +1597,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1617,22 +1617,22 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>63.2</t>
+          <t>39.3</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>37.9</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1641,35 +1641,35 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="O15" t="n">
-        <v>41.4</v>
+        <v>51.5</v>
       </c>
       <c r="P15" t="n">
-        <v>58.6</v>
+        <v>44.1</v>
       </c>
       <c r="Q15" t="n">
-        <v>51.7</v>
+        <v>52.9</v>
       </c>
       <c r="R15" t="n">
-        <v>34.5</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1679,63 +1679,637 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>47.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>31.1</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>135</v>
+      </c>
+      <c r="O16" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P16" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R16" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>9:15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>31.1</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>135</v>
+      </c>
+      <c r="O17" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P17" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R17" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>28.4</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>10.6</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>135</v>
+      </c>
+      <c r="O18" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="P18" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="R18" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>24.5</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>17</v>
+      </c>
+      <c r="O19" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="P19" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="R19" t="n">
+        <v>17.6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
           <t>7-5</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>95.4</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>65.6</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>40.4</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>80.2</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>58.7</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="N16" t="n">
+      <c r="N20" t="n">
         <v>18</v>
       </c>
-      <c r="O16" t="n">
+      <c r="O20" t="n">
         <v>44.4</v>
       </c>
-      <c r="P16" t="n">
+      <c r="P20" t="n">
         <v>55.6</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="Q20" t="n">
         <v>61.1</v>
       </c>
-      <c r="R16" t="n">
+      <c r="R20" t="n">
         <v>38.9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>KT Wiz Suwon</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>57</v>
+      </c>
+      <c r="O21" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="P21" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="R21" t="n">
+        <v>42.1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>8:05</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>3-7</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>59.6</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>34.2</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>22</v>
+      </c>
+      <c r="O22" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="P22" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>50</v>
+      </c>
+      <c r="R22" t="n">
+        <v>31.8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>37.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>33.8</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>13.8</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>41</v>
+      </c>
+      <c r="O23" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="P23" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>61</v>
+      </c>
+      <c r="R23" t="n">
+        <v>34.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-08-08 15:46
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,32 +511,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -556,12 +556,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -593,17 +593,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -613,37 +613,37 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -653,23 +653,23 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="O3" t="n">
-        <v>41.6</v>
+        <v>60.8</v>
       </c>
       <c r="P3" t="n">
-        <v>55.8</v>
+        <v>39.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>45.5</v>
+        <v>44.6</v>
       </c>
       <c r="R3" t="n">
-        <v>27.3</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="4">
@@ -680,12 +680,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,37 +695,37 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,79 +735,79 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="O4" t="n">
-        <v>60.8</v>
+        <v>41.6</v>
       </c>
       <c r="P4" t="n">
-        <v>39.2</v>
+        <v>55.8</v>
       </c>
       <c r="Q4" t="n">
-        <v>44.6</v>
+        <v>45.5</v>
       </c>
       <c r="R4" t="n">
-        <v>31.1</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>55.0</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>3-4</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -839,32 +839,32 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -884,12 +884,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -921,57 +921,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>23.8</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -981,59 +981,59 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="O7" t="n">
-        <v>60.8</v>
+        <v>41.6</v>
       </c>
       <c r="P7" t="n">
-        <v>39.2</v>
+        <v>55.8</v>
       </c>
       <c r="Q7" t="n">
-        <v>44.6</v>
+        <v>45.5</v>
       </c>
       <c r="R7" t="n">
-        <v>31.1</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1067,16 +1067,16 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>135</v>
+        <v>74</v>
       </c>
       <c r="O8" t="n">
-        <v>49.6</v>
+        <v>60.8</v>
       </c>
       <c r="P8" t="n">
-        <v>48.1</v>
+        <v>39.2</v>
       </c>
       <c r="Q8" t="n">
-        <v>45.9</v>
+        <v>44.6</v>
       </c>
       <c r="R8" t="n">
         <v>31.1</v>
@@ -1085,7 +1085,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1105,17 +1105,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1130,12 +1130,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1149,19 +1149,19 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>17</v>
+        <v>135</v>
       </c>
       <c r="O9" t="n">
-        <v>47.1</v>
+        <v>49.6</v>
       </c>
       <c r="P9" t="n">
-        <v>41.2</v>
+        <v>48.1</v>
       </c>
       <c r="Q9" t="n">
-        <v>17.6</v>
+        <v>45.9</v>
       </c>
       <c r="R9" t="n">
-        <v>17.6</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="10">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1212,12 +1212,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1249,17 +1249,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1269,17 +1269,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>9-6</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1289,17 +1289,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>99.2</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>59.6</t>
+          <t>93.8</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>34.2</t>
+          <t>82.4</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1313,25 +1313,25 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>68</v>
+        <v>509</v>
       </c>
       <c r="O11" t="n">
-        <v>51.5</v>
+        <v>52.8</v>
       </c>
       <c r="P11" t="n">
-        <v>44.1</v>
+        <v>44.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>52.9</v>
+        <v>46</v>
       </c>
       <c r="R11" t="n">
-        <v>35.3</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1413,17 +1413,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1433,17 +1433,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>9-6</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1453,17 +1453,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>99.2</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>93.8</t>
+          <t>59.6</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>82.4</t>
+          <t>34.2</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,35 +1477,35 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>509</v>
+        <v>68</v>
       </c>
       <c r="O13" t="n">
-        <v>52.8</v>
+        <v>51.5</v>
       </c>
       <c r="P13" t="n">
-        <v>44.4</v>
+        <v>44.1</v>
       </c>
       <c r="Q13" t="n">
-        <v>46</v>
+        <v>52.9</v>
       </c>
       <c r="R13" t="n">
-        <v>30.6</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1535,17 +1535,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>51.8</t>
+          <t>28.4</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1559,35 +1559,35 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>509</v>
+        <v>135</v>
       </c>
       <c r="O14" t="n">
-        <v>52.8</v>
+        <v>49.6</v>
       </c>
       <c r="P14" t="n">
-        <v>44.4</v>
+        <v>48.1</v>
       </c>
       <c r="Q14" t="n">
-        <v>46</v>
+        <v>45.9</v>
       </c>
       <c r="R14" t="n">
-        <v>30.6</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1622,12 +1622,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>39.3</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1659,17 +1659,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1679,37 +1679,37 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
           <t>55.0</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>45.0</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>55.0</t>
-        </is>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1741,17 +1741,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>9:15</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1761,12 +1761,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1786,12 +1786,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1823,119 +1823,119 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>28.4</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N18" t="n">
-        <v>135</v>
+        <v>57</v>
       </c>
       <c r="O18" t="n">
-        <v>49.6</v>
+        <v>49.1</v>
       </c>
       <c r="P18" t="n">
-        <v>48.1</v>
+        <v>49.1</v>
       </c>
       <c r="Q18" t="n">
-        <v>45.9</v>
+        <v>49.1</v>
       </c>
       <c r="R18" t="n">
-        <v>31.1</v>
+        <v>42.1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Uni Lions</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1945,22 +1945,22 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>95.4</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>80.2</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>58.7</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⚡</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1969,75 +1969,75 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="O19" t="n">
-        <v>47.1</v>
+        <v>44.4</v>
       </c>
       <c r="P19" t="n">
-        <v>41.2</v>
+        <v>55.6</v>
       </c>
       <c r="Q19" t="n">
-        <v>17.6</v>
+        <v>61.1</v>
       </c>
       <c r="R19" t="n">
-        <v>17.6</v>
+        <v>38.9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>80.2</t>
+          <t>50.4</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>58.7</t>
+          <t>25.9</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2047,54 +2047,54 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N20" t="n">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="O20" t="n">
-        <v>44.4</v>
+        <v>49.1</v>
       </c>
       <c r="P20" t="n">
-        <v>55.6</v>
+        <v>49.1</v>
       </c>
       <c r="Q20" t="n">
-        <v>61.1</v>
+        <v>49.1</v>
       </c>
       <c r="R20" t="n">
-        <v>38.9</v>
+        <v>42.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2114,12 +2114,12 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2151,17 +2151,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2171,17 +2171,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>3-7</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2191,17 +2191,17 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>59.6</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>34.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2215,100 +2215,346 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="O22" t="n">
-        <v>59.1</v>
+        <v>59.4</v>
       </c>
       <c r="P22" t="n">
-        <v>40.9</v>
+        <v>40.6</v>
       </c>
       <c r="Q22" t="n">
-        <v>50</v>
+        <v>28.1</v>
       </c>
       <c r="R22" t="n">
-        <v>31.8</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>29</v>
+      </c>
+      <c r="O23" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="P23" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="R23" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>41</v>
+      </c>
+      <c r="O24" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="P24" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>61</v>
+      </c>
+      <c r="R24" t="n">
+        <v>34.1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Fubon Guardians</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>35.2</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>14.6</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>29</v>
+      </c>
+      <c r="O25" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="P25" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="R25" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>Rakuten Monkeys</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Wei Chuan Dragons</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>CPB</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>37.0</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>63.0</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
         <is>
           <t>3-5</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>68.7</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>33.8</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>13.8</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>⚡</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>원정승</t>
         </is>
       </c>
-      <c r="N23" t="n">
+      <c r="N26" t="n">
         <v>41</v>
       </c>
-      <c r="O23" t="n">
+      <c r="O26" t="n">
         <v>48.8</v>
       </c>
-      <c r="P23" t="n">
+      <c r="P26" t="n">
         <v>48.8</v>
       </c>
-      <c r="Q23" t="n">
+      <c r="Q26" t="n">
         <v>61</v>
       </c>
-      <c r="R23" t="n">
+      <c r="R26" t="n">
         <v>34.1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-08-11 17:03
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,57 +511,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>1-4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>55.7</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>30.6</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -571,39 +571,39 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="O2" t="n">
-        <v>71.40000000000001</v>
+        <v>26.3</v>
       </c>
       <c r="P2" t="n">
-        <v>23.8</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="Q2" t="n">
-        <v>52.4</v>
+        <v>31.6</v>
       </c>
       <c r="R2" t="n">
-        <v>33.3</v>
+        <v>18.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -613,17 +613,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,22 +633,22 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>39.4</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -657,35 +657,35 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="O3" t="n">
-        <v>41.6</v>
+        <v>26.7</v>
       </c>
       <c r="P3" t="n">
-        <v>55.8</v>
+        <v>73.3</v>
       </c>
       <c r="Q3" t="n">
-        <v>45.5</v>
+        <v>30</v>
       </c>
       <c r="R3" t="n">
-        <v>27.3</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>10:38</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -695,17 +695,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>26.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>8-6</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -715,22 +715,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>98.6</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>79.4</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>57.5</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -739,60 +739,60 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>587</v>
+        <v>21</v>
       </c>
       <c r="O4" t="n">
-        <v>53.3</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="P4" t="n">
-        <v>44.1</v>
+        <v>23.8</v>
       </c>
       <c r="Q4" t="n">
-        <v>46.7</v>
+        <v>52.4</v>
       </c>
       <c r="R4" t="n">
-        <v>31.7</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -802,74 +802,74 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="O5" t="n">
-        <v>48.8</v>
+        <v>57.7</v>
       </c>
       <c r="P5" t="n">
-        <v>48.8</v>
+        <v>39.7</v>
       </c>
       <c r="Q5" t="n">
-        <v>61</v>
+        <v>51.3</v>
       </c>
       <c r="R5" t="n">
-        <v>34.1</v>
+        <v>35.9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -879,22 +879,22 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>40.7</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -903,101 +903,1905 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>41</v>
+        <v>77</v>
       </c>
       <c r="O6" t="n">
-        <v>48.8</v>
+        <v>41.6</v>
       </c>
       <c r="P6" t="n">
-        <v>48.8</v>
+        <v>55.8</v>
       </c>
       <c r="Q6" t="n">
-        <v>61</v>
+        <v>45.5</v>
       </c>
       <c r="R6" t="n">
-        <v>34.1</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rakuten Gold. Eagles</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Orix Buffaloes</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>8.9</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>74</v>
+      </c>
+      <c r="O7" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="P7" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="R7" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Hanwha Eagles</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>28.4</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>10.6</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>77</v>
+      </c>
+      <c r="O8" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="P8" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="R8" t="n">
+        <v>27.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SSG Landers</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>77</v>
+      </c>
+      <c r="O9" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="P9" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="R9" t="n">
+        <v>27.3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>8:07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>77</v>
+      </c>
+      <c r="O10" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="P10" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="R10" t="n">
+        <v>27.3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>44.9</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>21.5</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>78</v>
+      </c>
+      <c r="O11" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="P11" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="R11" t="n">
+        <v>35.9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>8:45</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>40.7</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>78</v>
+      </c>
+      <c r="O12" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="P12" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="R12" t="n">
+        <v>35.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>10:38</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>40.7</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>78</v>
+      </c>
+      <c r="O13" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="P13" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="R13" t="n">
+        <v>35.9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>71.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>29.0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>40.7</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>78</v>
+      </c>
+      <c r="O14" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="P14" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="R14" t="n">
+        <v>35.9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Uni Lions</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>52.0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>77</v>
+      </c>
+      <c r="O15" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="P15" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="R15" t="n">
+        <v>27.3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Fukuoka S. Hawks</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Chiba Lotte Marines</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>61.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>39.0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>136</v>
+      </c>
+      <c r="O16" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="P16" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="R16" t="n">
+        <v>30.9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Yakult Swallows</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Hiroshima Carp</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>61.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>39.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>46.3</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>22.6</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>68</v>
+      </c>
+      <c r="O17" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="P17" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R17" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>32.0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>50.4</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>25.9</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>68</v>
+      </c>
+      <c r="O18" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="P18" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R18" t="n">
+        <v>35.3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>62.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>31.1</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>17</v>
+      </c>
+      <c r="O19" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="P19" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="R19" t="n">
+        <v>17.6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Wei Chuan Dragons</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>55.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>25.8</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>136</v>
+      </c>
+      <c r="O20" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="P20" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="R20" t="n">
+        <v>30.9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>KIA Tigers</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>44.9</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>21.5</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>29</v>
+      </c>
+      <c r="O21" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="P21" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="R21" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Kiwoom Heroes</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>LG Twins</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>66.7</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>41.7</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>34</v>
+      </c>
+      <c r="O22" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="P22" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>50</v>
+      </c>
+      <c r="R22" t="n">
+        <v>32.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>NC Dinos</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>KT Wiz Suwon</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>3-6</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>55.7</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>30.6</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>14</v>
+      </c>
+      <c r="O23" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="P23" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>50</v>
+      </c>
+      <c r="R23" t="n">
+        <v>35.7</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>53.1</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>28.2</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>⚡</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>57</v>
+      </c>
+      <c r="O24" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="P2